<commit_message>
fix: allow negative opening balance in CO cashbook UI
</commit_message>
<xml_diff>
--- a/icare-group-member-onboarding-template.xlsx
+++ b/icare-group-member-onboarding-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\Master_ AY Projects\trustmicro-credit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9095ED9A-6729-4A8C-A2D3-9475BCD53776}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0229BF08-1474-4D13-8242-FD8CCC815105}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2478" uniqueCount="1281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2503" uniqueCount="1289">
   <si>
     <t>ICARE Group and Member Onboarding Template</t>
   </si>
@@ -3850,25 +3850,49 @@
     <t>Ojei Elizabeth</t>
   </si>
   <si>
+    <t>09047690900</t>
+  </si>
+  <si>
+    <t>08050412130</t>
+  </si>
+  <si>
+    <t>Koleosho Sherifat</t>
+  </si>
+  <si>
+    <t>11750</t>
+  </si>
+  <si>
+    <t>7000</t>
+  </si>
+  <si>
+    <t>17000</t>
+  </si>
+  <si>
     <t>Weekly 12W</t>
   </si>
   <si>
-    <t>09047690900</t>
-  </si>
-  <si>
-    <t>08050412130</t>
-  </si>
-  <si>
     <t>Weekly 24W</t>
   </si>
   <si>
-    <t>Koleosho Sherifat</t>
-  </si>
-  <si>
-    <t>35925</t>
-  </si>
-  <si>
-    <t>25125</t>
+    <t>Weekly 12W Asset</t>
+  </si>
+  <si>
+    <t>Osho Bunmi</t>
+  </si>
+  <si>
+    <t>09049017436</t>
+  </si>
+  <si>
+    <t>Oguntamo Modina</t>
+  </si>
+  <si>
+    <t>09035527146</t>
+  </si>
+  <si>
+    <t>MEM-349</t>
+  </si>
+  <si>
+    <t>MEM-350</t>
   </si>
 </sst>
 </file>
@@ -4068,7 +4092,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -4158,6 +4182,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="3" fontId="4" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -4188,26 +4218,327 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="4" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="19">
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9E2F3"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FFD9E2F3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9E2F3"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FFD9E2F3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9E2F3"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FFD9E2F3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9E2F3"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9E2F3"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9E2F3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFFCE4D6"/>
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
         </patternFill>
       </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9E2F3"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9E2F3"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9E2F3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9E2F3"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9E2F3"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9E2F3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9E2F3"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9E2F3"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9E2F3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9E2F3"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9E2F3"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9E2F3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9E2F3"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9E2F3"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9E2F3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9E2F3"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9E2F3"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9E2F3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -4263,161 +4594,27 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos"/>
-      </font>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
       <alignment horizontal="left" vertical="top"/>
-      <border outline="0">
-        <left style="thin">
-          <color rgb="FFD9E2F3"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color rgb="FFD9E2F3"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9E2F3"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos"/>
+        <color rgb="FF9C0006"/>
       </font>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
       <fill>
         <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFCE4D6"/>
         </patternFill>
       </fill>
-      <alignment horizontal="left" vertical="top"/>
-      <border>
-        <left style="thin">
-          <color rgb="FFD9E2F3"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color rgb="FFD9E2F3"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9E2F3"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos"/>
+        <color rgb="FF9C0006"/>
       </font>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
       <fill>
         <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFCE4D6"/>
         </patternFill>
       </fill>
-      <alignment horizontal="left" vertical="top"/>
-      <border outline="0">
-        <left style="thin">
-          <color rgb="FFD9E2F3"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color rgb="FFD9E2F3"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9E2F3"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos"/>
-      </font>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="top"/>
-      <border outline="0">
-        <left style="thin">
-          <color rgb="FFD9E2F3"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9E2F3"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9E2F3"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9E2F3"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="top"/>
     </dxf>
     <dxf>
       <font>
@@ -4476,6 +4673,16 @@
         <horizontal/>
       </border>
     </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -4495,31 +4702,31 @@
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Group Reference*"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Branch Name*"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Group Name*"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Group Leader Name*" dataDxfId="16"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Group Leader Name*" dataDxfId="17"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Meeting Day*"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Formation Date*"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Credit Officer Name*"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Credit Officer Phone"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Group Savings" dataDxfId="15"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Group Savings" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="MemberOnboardingTable" displayName="MemberOnboardingTable" ref="A3:K2000" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="MemberOnboardingTable" displayName="MemberOnboardingTable" ref="A3:K2002" dataDxfId="13">
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Member Reference*" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Group Reference*" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Member Number" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Full Name*" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Phone Number*" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Home Address*" dataDxfId="8"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Savings Balance*" dataDxfId="7"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0100-000015000000}" name="Loan Type (Product)*" dataDxfId="6"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0100-000016000000}" name="Principal Loan*" dataDxfId="5"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0100-000014000000}" name="Active Credit (Disbursed)*" dataDxfId="4"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0100-000013000000}" name="Current Credit Balance*" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Member Reference*" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Group Reference*" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Member Number" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Full Name*" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Phone Number*" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Home Address*" dataDxfId="4"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Savings Balance*" dataDxfId="3"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0100-000015000000}" name="Loan Type (Product)*" dataDxfId="2"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0100-000016000000}" name="Principal Loan*" dataDxfId="1"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0100-000014000000}" name="Active Credit (Disbursed)*" dataDxfId="0"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0100-000013000000}" name="Current Credit Balance*" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4684,28 +4891,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="33.9" customHeight="1">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="37"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="2"/>
@@ -4725,13 +4932,13 @@
         <v>3</v>
       </c>
       <c r="C4" s="2"/>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="37"/>
-      <c r="F4" s="37"/>
-      <c r="G4" s="37"/>
-      <c r="H4" s="37"/>
+      <c r="E4" s="39"/>
+      <c r="F4" s="39"/>
+      <c r="G4" s="39"/>
+      <c r="H4" s="39"/>
     </row>
     <row r="5" spans="1:8" ht="27.9" customHeight="1">
       <c r="A5" s="3" t="s">
@@ -4739,13 +4946,13 @@
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="39" t="s">
+      <c r="D5" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="34"/>
-      <c r="H5" s="35"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="37"/>
     </row>
     <row r="6" spans="1:8" ht="27.9" customHeight="1">
       <c r="A6" s="3" t="s">
@@ -4753,13 +4960,13 @@
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="39" t="s">
+      <c r="D6" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="35"/>
+      <c r="E6" s="36"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="36"/>
+      <c r="H6" s="37"/>
     </row>
     <row r="7" spans="1:8" ht="27.9" customHeight="1">
       <c r="A7" s="3" t="s">
@@ -4767,13 +4974,13 @@
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="39" t="s">
+      <c r="D7" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="34"/>
-      <c r="F7" s="34"/>
-      <c r="G7" s="34"/>
-      <c r="H7" s="35"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="37"/>
     </row>
     <row r="8" spans="1:8" ht="27.9" customHeight="1">
       <c r="A8" s="3" t="s">
@@ -4781,13 +4988,13 @@
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="2"/>
-      <c r="D8" s="39" t="s">
+      <c r="D8" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="35"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="36"/>
+      <c r="H8" s="37"/>
     </row>
     <row r="9" spans="1:8" ht="27.9" customHeight="1">
       <c r="A9" s="3" t="s">
@@ -4795,25 +5002,25 @@
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="2"/>
-      <c r="D9" s="39" t="s">
+      <c r="D9" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="34"/>
-      <c r="F9" s="34"/>
-      <c r="G9" s="34"/>
-      <c r="H9" s="35"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="36"/>
+      <c r="H9" s="37"/>
     </row>
     <row r="10" spans="1:8" ht="27.9" customHeight="1">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
-      <c r="D10" s="39" t="s">
+      <c r="D10" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="34"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="35"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="36"/>
+      <c r="H10" s="37"/>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="2"/>
@@ -4826,142 +5033,142 @@
       <c r="H11" s="2"/>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="45" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="37"/>
-      <c r="C12" s="37"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="37"/>
-      <c r="F12" s="37"/>
-      <c r="G12" s="37"/>
-      <c r="H12" s="37"/>
+      <c r="B12" s="39"/>
+      <c r="C12" s="39"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="39"/>
+      <c r="F12" s="39"/>
+      <c r="G12" s="39"/>
+      <c r="H12" s="39"/>
     </row>
     <row r="13" spans="1:8" ht="38.1" customHeight="1">
       <c r="A13" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="41" t="s">
+      <c r="B13" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="34"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="35"/>
+      <c r="C13" s="36"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="36"/>
+      <c r="H13" s="37"/>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="40" t="s">
+      <c r="B14" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="34"/>
-      <c r="D14" s="34"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="34"/>
-      <c r="G14" s="34"/>
-      <c r="H14" s="35"/>
+      <c r="C14" s="36"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="36"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="36"/>
+      <c r="H14" s="37"/>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="40" t="s">
+      <c r="B15" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="34"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="34"/>
-      <c r="G15" s="34"/>
-      <c r="H15" s="35"/>
+      <c r="C15" s="36"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="36"/>
+      <c r="H15" s="37"/>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="40" t="s">
+      <c r="B16" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="34"/>
-      <c r="G16" s="34"/>
-      <c r="H16" s="35"/>
+      <c r="C16" s="36"/>
+      <c r="D16" s="36"/>
+      <c r="E16" s="36"/>
+      <c r="F16" s="36"/>
+      <c r="G16" s="36"/>
+      <c r="H16" s="37"/>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="40" t="s">
+      <c r="B17" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="34"/>
-      <c r="D17" s="34"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="35"/>
+      <c r="C17" s="36"/>
+      <c r="D17" s="36"/>
+      <c r="E17" s="36"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="36"/>
+      <c r="H17" s="37"/>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="40" t="s">
+      <c r="B18" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="34"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="34"/>
-      <c r="G18" s="34"/>
-      <c r="H18" s="35"/>
+      <c r="C18" s="36"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="36"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="36"/>
+      <c r="H18" s="37"/>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="40" t="s">
+      <c r="B19" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="35"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="36"/>
+      <c r="H19" s="37"/>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="40" t="s">
+      <c r="B20" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="34"/>
-      <c r="D20" s="34"/>
-      <c r="E20" s="34"/>
-      <c r="F20" s="34"/>
-      <c r="G20" s="34"/>
-      <c r="H20" s="35"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="36"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="37"/>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="33" t="s">
+      <c r="B21" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="C21" s="34"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="35"/>
+      <c r="C21" s="36"/>
+      <c r="D21" s="36"/>
+      <c r="E21" s="36"/>
+      <c r="F21" s="36"/>
+      <c r="G21" s="36"/>
+      <c r="H21" s="37"/>
     </row>
   </sheetData>
   <autoFilter ref="A12:H21" xr:uid="{00000000-0009-0000-0000-000000000000}">
@@ -5015,30 +5222,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="33.9" customHeight="1">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="37"/>
-      <c r="I2" s="37"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
     </row>
     <row r="3" spans="1:9" ht="38.1" customHeight="1">
       <c r="A3" s="28" t="s">
@@ -5679,7 +5886,9 @@
       <c r="C28" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="D28" s="6"/>
+      <c r="D28" s="6" t="s">
+        <v>774</v>
+      </c>
       <c r="E28" s="6" t="s">
         <v>107</v>
       </c>
@@ -5692,7 +5901,9 @@
       <c r="H28" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="I28" s="14"/>
+      <c r="I28" s="14" t="s">
+        <v>1277</v>
+      </c>
     </row>
     <row r="29" spans="1:9">
       <c r="A29" s="6" t="s">
@@ -5704,7 +5915,9 @@
       <c r="C29" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="D29" s="6"/>
+      <c r="D29" s="6" t="s">
+        <v>804</v>
+      </c>
       <c r="E29" s="6" t="s">
         <v>107</v>
       </c>
@@ -5717,7 +5930,9 @@
       <c r="H29" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="I29" s="14"/>
+      <c r="I29" s="14" t="s">
+        <v>1278</v>
+      </c>
     </row>
     <row r="30" spans="1:9">
       <c r="A30" s="6" t="s">
@@ -5729,7 +5944,9 @@
       <c r="C30" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="D30" s="6"/>
+      <c r="D30" s="6" t="s">
+        <v>823</v>
+      </c>
       <c r="E30" s="6" t="s">
         <v>107</v>
       </c>
@@ -5742,7 +5959,9 @@
       <c r="H30" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="I30" s="14"/>
+      <c r="I30" s="14" t="s">
+        <v>1279</v>
+      </c>
     </row>
     <row r="31" spans="1:9">
       <c r="A31" s="6" t="s">
@@ -5755,7 +5974,7 @@
         <v>113</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>1278</v>
+        <v>1276</v>
       </c>
       <c r="E31" s="6" t="s">
         <v>114</v>
@@ -5769,9 +5988,7 @@
       <c r="H31" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="I31" s="48" t="s">
-        <v>1279</v>
-      </c>
+      <c r="I31" s="34"/>
     </row>
     <row r="32" spans="1:9">
       <c r="A32" s="6" t="s">
@@ -5798,9 +6015,7 @@
       <c r="H32" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="I32" s="48" t="s">
-        <v>1280</v>
-      </c>
+      <c r="I32" s="34"/>
     </row>
     <row r="33" spans="1:9">
       <c r="A33" s="6" t="s">
@@ -8519,7 +8734,7 @@
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <conditionalFormatting sqref="A4:A253">
-    <cfRule type="duplicateValues" dxfId="2" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="21"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -8531,7 +8746,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K2000"/>
+  <dimension ref="A1:K2002"/>
   <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="2" width="22.09765625" style="27" customWidth="1"/>
@@ -8543,34 +8758,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="33.9" customHeight="1">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>161</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
     </row>
     <row r="2" spans="1:11" ht="30" customHeight="1">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="46" t="s">
         <v>162</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
     </row>
     <row r="3" spans="1:11" ht="38.1" customHeight="1">
       <c r="A3" s="28" t="s">
@@ -13325,10 +13540,18 @@
       <c r="F193" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="G193" s="20"/>
-      <c r="H193" s="23"/>
-      <c r="I193" s="23"/>
-      <c r="J193" s="23"/>
+      <c r="G193" s="20">
+        <v>24550</v>
+      </c>
+      <c r="H193" s="23" t="s">
+        <v>1280</v>
+      </c>
+      <c r="I193" s="23">
+        <v>198000</v>
+      </c>
+      <c r="J193" s="23">
+        <v>82500</v>
+      </c>
       <c r="K193" s="23"/>
     </row>
     <row r="194" spans="1:11">
@@ -13350,10 +13573,18 @@
       <c r="F194" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="G194" s="20"/>
-      <c r="H194" s="23"/>
-      <c r="I194" s="23"/>
-      <c r="J194" s="23"/>
+      <c r="G194" s="20">
+        <v>22200</v>
+      </c>
+      <c r="H194" s="23" t="s">
+        <v>1280</v>
+      </c>
+      <c r="I194" s="23">
+        <v>48000</v>
+      </c>
+      <c r="J194" s="23">
+        <v>4000</v>
+      </c>
       <c r="K194" s="23"/>
     </row>
     <row r="195" spans="1:11">
@@ -13375,10 +13606,18 @@
       <c r="F195" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="G195" s="20"/>
-      <c r="H195" s="23"/>
-      <c r="I195" s="23"/>
-      <c r="J195" s="23"/>
+      <c r="G195" s="20">
+        <v>15000</v>
+      </c>
+      <c r="H195" s="23" t="s">
+        <v>1280</v>
+      </c>
+      <c r="I195" s="23">
+        <v>288000</v>
+      </c>
+      <c r="J195" s="23">
+        <v>288000</v>
+      </c>
       <c r="K195" s="23"/>
     </row>
     <row r="196" spans="1:11">
@@ -13400,10 +13639,18 @@
       <c r="F196" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="G196" s="20"/>
-      <c r="H196" s="23"/>
-      <c r="I196" s="23"/>
-      <c r="J196" s="23"/>
+      <c r="G196" s="20">
+        <v>13000</v>
+      </c>
+      <c r="H196" s="23" t="s">
+        <v>1280</v>
+      </c>
+      <c r="I196" s="23">
+        <v>60000</v>
+      </c>
+      <c r="J196" s="23">
+        <v>10000</v>
+      </c>
       <c r="K196" s="23"/>
     </row>
     <row r="197" spans="1:11">
@@ -13423,10 +13670,18 @@
       <c r="F197" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="G197" s="20"/>
-      <c r="H197" s="23"/>
-      <c r="I197" s="23"/>
-      <c r="J197" s="23"/>
+      <c r="G197" s="20">
+        <v>9500</v>
+      </c>
+      <c r="H197" s="23" t="s">
+        <v>1280</v>
+      </c>
+      <c r="I197" s="23">
+        <v>150000</v>
+      </c>
+      <c r="J197" s="23">
+        <v>100000</v>
+      </c>
       <c r="K197" s="23"/>
     </row>
     <row r="198" spans="1:11">
@@ -13449,7 +13704,9 @@
         <v>776</v>
       </c>
       <c r="G198" s="20"/>
-      <c r="H198" s="23"/>
+      <c r="H198" s="23" t="s">
+        <v>1281</v>
+      </c>
       <c r="I198" s="23"/>
       <c r="J198" s="23"/>
       <c r="K198" s="23"/>
@@ -13473,10 +13730,18 @@
       <c r="F199" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="G199" s="20"/>
-      <c r="H199" s="23"/>
-      <c r="I199" s="23"/>
-      <c r="J199" s="23"/>
+      <c r="G199" s="20">
+        <v>23600</v>
+      </c>
+      <c r="H199" s="23" t="s">
+        <v>1281</v>
+      </c>
+      <c r="I199" s="23">
+        <v>198000</v>
+      </c>
+      <c r="J199" s="23">
+        <v>41250</v>
+      </c>
       <c r="K199" s="23"/>
     </row>
     <row r="200" spans="1:11">
@@ -13498,8 +13763,12 @@
       <c r="F200" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="G200" s="20"/>
-      <c r="H200" s="23"/>
+      <c r="G200" s="20">
+        <v>63400</v>
+      </c>
+      <c r="H200" s="23" t="s">
+        <v>1281</v>
+      </c>
       <c r="I200" s="23"/>
       <c r="J200" s="23"/>
       <c r="K200" s="23"/>
@@ -13523,10 +13792,18 @@
       <c r="F201" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="G201" s="20"/>
-      <c r="H201" s="23"/>
-      <c r="I201" s="23"/>
-      <c r="J201" s="23"/>
+      <c r="G201" s="20">
+        <v>18725</v>
+      </c>
+      <c r="H201" s="23" t="s">
+        <v>1281</v>
+      </c>
+      <c r="I201" s="23">
+        <v>99000</v>
+      </c>
+      <c r="J201" s="23">
+        <v>28875</v>
+      </c>
       <c r="K201" s="23"/>
     </row>
     <row r="202" spans="1:11">
@@ -13548,8 +13825,12 @@
       <c r="F202" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="G202" s="20"/>
-      <c r="H202" s="23"/>
+      <c r="G202" s="20">
+        <v>89000</v>
+      </c>
+      <c r="H202" s="23" t="s">
+        <v>1281</v>
+      </c>
       <c r="I202" s="23"/>
       <c r="J202" s="23"/>
       <c r="K202" s="23"/>
@@ -13573,10 +13854,18 @@
       <c r="F203" s="22" t="s">
         <v>806</v>
       </c>
-      <c r="G203" s="20"/>
-      <c r="H203" s="23"/>
-      <c r="I203" s="23"/>
-      <c r="J203" s="23"/>
+      <c r="G203" s="20">
+        <v>5950</v>
+      </c>
+      <c r="H203" s="23" t="s">
+        <v>1280</v>
+      </c>
+      <c r="I203" s="23">
+        <v>99000</v>
+      </c>
+      <c r="J203" s="23">
+        <v>24750</v>
+      </c>
       <c r="K203" s="23"/>
     </row>
     <row r="204" spans="1:11">
@@ -13598,10 +13887,18 @@
       <c r="F204" s="22" t="s">
         <v>806</v>
       </c>
-      <c r="G204" s="20"/>
-      <c r="H204" s="23"/>
-      <c r="I204" s="23"/>
-      <c r="J204" s="23"/>
+      <c r="G204" s="20">
+        <v>4750</v>
+      </c>
+      <c r="H204" s="23" t="s">
+        <v>1280</v>
+      </c>
+      <c r="I204" s="23">
+        <v>99000</v>
+      </c>
+      <c r="J204" s="23">
+        <v>33000</v>
+      </c>
       <c r="K204" s="23"/>
     </row>
     <row r="205" spans="1:11">
@@ -13624,9 +13921,15 @@
         <v>806</v>
       </c>
       <c r="G205" s="20"/>
-      <c r="H205" s="23"/>
-      <c r="I205" s="23"/>
-      <c r="J205" s="23"/>
+      <c r="H205" s="23" t="s">
+        <v>1282</v>
+      </c>
+      <c r="I205" s="23">
+        <v>279000</v>
+      </c>
+      <c r="J205" s="23">
+        <v>46500</v>
+      </c>
       <c r="K205" s="23"/>
     </row>
     <row r="206" spans="1:11">
@@ -13648,10 +13951,18 @@
       <c r="F206" s="22" t="s">
         <v>806</v>
       </c>
-      <c r="G206" s="20"/>
-      <c r="H206" s="23"/>
-      <c r="I206" s="23"/>
-      <c r="J206" s="23"/>
+      <c r="G206" s="20">
+        <v>5000</v>
+      </c>
+      <c r="H206" s="23" t="s">
+        <v>1280</v>
+      </c>
+      <c r="I206" s="23">
+        <v>99000</v>
+      </c>
+      <c r="J206" s="23">
+        <v>24750</v>
+      </c>
       <c r="K206" s="23"/>
     </row>
     <row r="207" spans="1:11">
@@ -13673,10 +13984,18 @@
       <c r="F207" s="22" t="s">
         <v>806</v>
       </c>
-      <c r="G207" s="20"/>
-      <c r="H207" s="23"/>
-      <c r="I207" s="23"/>
-      <c r="J207" s="23"/>
+      <c r="G207" s="20">
+        <v>4750</v>
+      </c>
+      <c r="H207" s="23" t="s">
+        <v>1280</v>
+      </c>
+      <c r="I207" s="23">
+        <v>99000</v>
+      </c>
+      <c r="J207" s="23">
+        <v>33000</v>
+      </c>
       <c r="K207" s="23"/>
     </row>
     <row r="208" spans="1:11">
@@ -13698,10 +14017,18 @@
       <c r="F208" s="22" t="s">
         <v>806</v>
       </c>
-      <c r="G208" s="20"/>
-      <c r="H208" s="23"/>
-      <c r="I208" s="23"/>
-      <c r="J208" s="23"/>
+      <c r="G208" s="20">
+        <v>3000</v>
+      </c>
+      <c r="H208" s="23" t="s">
+        <v>1280</v>
+      </c>
+      <c r="I208" s="23">
+        <v>99000</v>
+      </c>
+      <c r="J208" s="23">
+        <v>57750</v>
+      </c>
       <c r="K208" s="23"/>
     </row>
     <row r="209" spans="1:11">
@@ -13709,24 +14036,32 @@
         <v>822</v>
       </c>
       <c r="B209" s="21" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C209" s="21" t="s">
-        <v>174</v>
+        <v>206</v>
       </c>
       <c r="D209" s="22" t="s">
-        <v>823</v>
+        <v>1283</v>
       </c>
       <c r="E209" s="21" t="s">
-        <v>824</v>
+        <v>1284</v>
       </c>
       <c r="F209" s="22" t="s">
-        <v>711</v>
-      </c>
-      <c r="G209" s="20"/>
-      <c r="H209" s="23"/>
-      <c r="I209" s="23"/>
-      <c r="J209" s="23"/>
+        <v>806</v>
+      </c>
+      <c r="G209" s="49">
+        <v>2750</v>
+      </c>
+      <c r="H209" s="23" t="s">
+        <v>1280</v>
+      </c>
+      <c r="I209" s="23">
+        <v>99000</v>
+      </c>
+      <c r="J209" s="33">
+        <v>66000</v>
+      </c>
       <c r="K209" s="23"/>
     </row>
     <row r="210" spans="1:11">
@@ -13734,24 +14069,32 @@
         <v>825</v>
       </c>
       <c r="B210" s="21" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C210" s="21" t="s">
-        <v>179</v>
+        <v>210</v>
       </c>
       <c r="D210" s="22" t="s">
-        <v>826</v>
+        <v>1285</v>
       </c>
       <c r="E210" s="21" t="s">
-        <v>827</v>
+        <v>1286</v>
       </c>
       <c r="F210" s="22" t="s">
-        <v>698</v>
-      </c>
-      <c r="G210" s="20"/>
-      <c r="H210" s="23"/>
-      <c r="I210" s="23"/>
-      <c r="J210" s="23"/>
+        <v>806</v>
+      </c>
+      <c r="G210" s="49">
+        <v>2750</v>
+      </c>
+      <c r="H210" s="23" t="s">
+        <v>1280</v>
+      </c>
+      <c r="I210" s="23">
+        <v>99000</v>
+      </c>
+      <c r="J210" s="33">
+        <v>66000</v>
+      </c>
       <c r="K210" s="23"/>
     </row>
     <row r="211" spans="1:11">
@@ -13762,21 +14105,29 @@
         <v>110</v>
       </c>
       <c r="C211" s="21" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D211" s="22" t="s">
-        <v>829</v>
+        <v>823</v>
       </c>
       <c r="E211" s="21" t="s">
-        <v>830</v>
+        <v>824</v>
       </c>
       <c r="F211" s="22" t="s">
-        <v>698</v>
-      </c>
-      <c r="G211" s="20"/>
-      <c r="H211" s="23"/>
-      <c r="I211" s="23"/>
-      <c r="J211" s="23"/>
+        <v>711</v>
+      </c>
+      <c r="G211" s="20">
+        <v>19200</v>
+      </c>
+      <c r="H211" s="23" t="s">
+        <v>1280</v>
+      </c>
+      <c r="I211" s="23">
+        <v>288000</v>
+      </c>
+      <c r="J211" s="23">
+        <v>288000</v>
+      </c>
       <c r="K211" s="23"/>
     </row>
     <row r="212" spans="1:11">
@@ -13787,21 +14138,29 @@
         <v>110</v>
       </c>
       <c r="C212" s="21" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="D212" s="22" t="s">
-        <v>832</v>
+        <v>826</v>
       </c>
       <c r="E212" s="21" t="s">
-        <v>833</v>
+        <v>827</v>
       </c>
       <c r="F212" s="22" t="s">
-        <v>711</v>
-      </c>
-      <c r="G212" s="20"/>
-      <c r="H212" s="23"/>
-      <c r="I212" s="23"/>
-      <c r="J212" s="23"/>
+        <v>698</v>
+      </c>
+      <c r="G212" s="20">
+        <v>11700</v>
+      </c>
+      <c r="H212" s="23" t="s">
+        <v>1280</v>
+      </c>
+      <c r="I212" s="23">
+        <v>288000</v>
+      </c>
+      <c r="J212" s="23">
+        <v>288000</v>
+      </c>
       <c r="K212" s="23"/>
     </row>
     <row r="213" spans="1:11">
@@ -13812,21 +14171,29 @@
         <v>110</v>
       </c>
       <c r="C213" s="21" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="D213" s="22" t="s">
-        <v>835</v>
+        <v>829</v>
       </c>
       <c r="E213" s="21" t="s">
-        <v>836</v>
+        <v>830</v>
       </c>
       <c r="F213" s="22" t="s">
-        <v>711</v>
-      </c>
-      <c r="G213" s="20"/>
-      <c r="H213" s="23"/>
-      <c r="I213" s="23"/>
-      <c r="J213" s="23"/>
+        <v>698</v>
+      </c>
+      <c r="G213" s="20">
+        <v>11700</v>
+      </c>
+      <c r="H213" s="23" t="s">
+        <v>1280</v>
+      </c>
+      <c r="I213" s="23">
+        <v>246000</v>
+      </c>
+      <c r="J213" s="23">
+        <v>246000</v>
+      </c>
       <c r="K213" s="23"/>
     </row>
     <row r="214" spans="1:11">
@@ -13834,28 +14201,32 @@
         <v>837</v>
       </c>
       <c r="B214" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C214" s="21" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
       <c r="D214" s="22" t="s">
-        <v>1271</v>
+        <v>832</v>
       </c>
       <c r="E214" s="21" t="s">
-        <v>838</v>
+        <v>833</v>
       </c>
       <c r="F214" s="22" t="s">
-        <v>839</v>
+        <v>711</v>
       </c>
       <c r="G214" s="20">
-        <v>38100</v>
+        <v>11000</v>
       </c>
       <c r="H214" s="23" t="s">
-        <v>1274</v>
-      </c>
-      <c r="I214" s="23"/>
-      <c r="J214" s="23"/>
+        <v>1280</v>
+      </c>
+      <c r="I214" s="23">
+        <v>288000</v>
+      </c>
+      <c r="J214" s="23">
+        <v>288000</v>
+      </c>
       <c r="K214" s="23"/>
     </row>
     <row r="215" spans="1:11">
@@ -13863,35 +14234,33 @@
         <v>840</v>
       </c>
       <c r="B215" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C215" s="21" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="D215" s="22" t="s">
-        <v>841</v>
+        <v>835</v>
       </c>
       <c r="E215" s="21" t="s">
-        <v>842</v>
+        <v>836</v>
       </c>
       <c r="F215" s="22" t="s">
-        <v>839</v>
+        <v>711</v>
       </c>
       <c r="G215" s="20">
-        <v>14100</v>
+        <v>9250</v>
       </c>
       <c r="H215" s="23" t="s">
-        <v>1274</v>
-      </c>
-      <c r="I215" s="47">
-        <v>200000</v>
+        <v>1280</v>
+      </c>
+      <c r="I215" s="23">
+        <v>99000</v>
       </c>
       <c r="J215" s="23">
-        <v>198000</v>
-      </c>
-      <c r="K215" s="23">
-        <v>148500</v>
-      </c>
+        <v>24750</v>
+      </c>
+      <c r="K215" s="23"/>
     </row>
     <row r="216" spans="1:11">
       <c r="A216" s="21" t="s">
@@ -13901,32 +14270,22 @@
         <v>112</v>
       </c>
       <c r="C216" s="21" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D216" s="22" t="s">
-        <v>844</v>
+        <v>1271</v>
       </c>
       <c r="E216" s="21" t="s">
-        <v>845</v>
+        <v>838</v>
       </c>
       <c r="F216" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G216" s="20">
-        <v>16000</v>
-      </c>
-      <c r="H216" s="23" t="s">
-        <v>1274</v>
-      </c>
-      <c r="I216" s="47">
-        <v>200000</v>
-      </c>
-      <c r="J216" s="23">
-        <v>198000</v>
-      </c>
-      <c r="K216" s="23">
-        <v>148500</v>
-      </c>
+      <c r="G216" s="20"/>
+      <c r="H216" s="23"/>
+      <c r="I216" s="23"/>
+      <c r="J216" s="23"/>
+      <c r="K216" s="23"/>
     </row>
     <row r="217" spans="1:11">
       <c r="A217" s="21" t="s">
@@ -13936,24 +14295,20 @@
         <v>112</v>
       </c>
       <c r="C217" s="21" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="D217" s="22" t="s">
-        <v>847</v>
+        <v>841</v>
       </c>
       <c r="E217" s="21" t="s">
-        <v>848</v>
+        <v>842</v>
       </c>
       <c r="F217" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G217" s="20">
-        <v>35000</v>
-      </c>
-      <c r="H217" s="23" t="s">
-        <v>1274</v>
-      </c>
-      <c r="I217" s="47"/>
+      <c r="G217" s="20"/>
+      <c r="H217" s="23"/>
+      <c r="I217" s="23"/>
       <c r="J217" s="23"/>
       <c r="K217" s="23"/>
     </row>
@@ -13965,22 +14320,20 @@
         <v>112</v>
       </c>
       <c r="C218" s="21" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="D218" s="22" t="s">
-        <v>1272</v>
+        <v>844</v>
       </c>
       <c r="E218" s="21" t="s">
-        <v>1275</v>
+        <v>845</v>
       </c>
       <c r="F218" s="22" t="s">
         <v>839</v>
       </c>
       <c r="G218" s="20"/>
-      <c r="H218" s="23" t="s">
-        <v>1274</v>
-      </c>
-      <c r="I218" s="47"/>
+      <c r="H218" s="23"/>
+      <c r="I218" s="23"/>
       <c r="J218" s="23"/>
       <c r="K218" s="23"/>
     </row>
@@ -13992,24 +14345,20 @@
         <v>112</v>
       </c>
       <c r="C219" s="21" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="D219" s="22" t="s">
-        <v>1273</v>
+        <v>847</v>
       </c>
       <c r="E219" s="21" t="s">
-        <v>1276</v>
+        <v>848</v>
       </c>
       <c r="F219" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G219" s="20">
-        <v>15500</v>
-      </c>
-      <c r="H219" s="23" t="s">
-        <v>1274</v>
-      </c>
-      <c r="I219" s="47"/>
+      <c r="G219" s="20"/>
+      <c r="H219" s="23"/>
+      <c r="I219" s="23"/>
       <c r="J219" s="23"/>
       <c r="K219" s="23"/>
     </row>
@@ -14021,32 +14370,22 @@
         <v>112</v>
       </c>
       <c r="C220" s="21" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="D220" s="22" t="s">
-        <v>852</v>
+        <v>1272</v>
       </c>
       <c r="E220" s="21" t="s">
-        <v>853</v>
+        <v>1274</v>
       </c>
       <c r="F220" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G220" s="20">
-        <v>52000</v>
-      </c>
-      <c r="H220" s="23" t="s">
-        <v>1277</v>
-      </c>
-      <c r="I220" s="47">
-        <v>250000</v>
-      </c>
-      <c r="J220" s="23">
-        <v>246000</v>
-      </c>
-      <c r="K220" s="23">
-        <v>102500</v>
-      </c>
+      <c r="G220" s="20"/>
+      <c r="H220" s="23"/>
+      <c r="I220" s="23"/>
+      <c r="J220" s="23"/>
+      <c r="K220" s="23"/>
     </row>
     <row r="221" spans="1:11">
       <c r="A221" s="21" t="s">
@@ -14056,32 +14395,22 @@
         <v>112</v>
       </c>
       <c r="C221" s="21" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="D221" s="22" t="s">
-        <v>855</v>
+        <v>1273</v>
       </c>
       <c r="E221" s="21" t="s">
-        <v>856</v>
+        <v>1275</v>
       </c>
       <c r="F221" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G221" s="20">
-        <v>30900</v>
-      </c>
-      <c r="H221" s="23" t="s">
-        <v>1277</v>
-      </c>
-      <c r="I221" s="47">
-        <v>250000</v>
-      </c>
-      <c r="J221" s="23">
-        <v>246000</v>
-      </c>
-      <c r="K221" s="23">
-        <v>112750</v>
-      </c>
+      <c r="G221" s="20"/>
+      <c r="H221" s="23"/>
+      <c r="I221" s="23"/>
+      <c r="J221" s="23"/>
+      <c r="K221" s="23"/>
     </row>
     <row r="222" spans="1:11">
       <c r="A222" s="21" t="s">
@@ -14091,102 +14420,72 @@
         <v>112</v>
       </c>
       <c r="C222" s="21" t="s">
-        <v>258</v>
+        <v>206</v>
       </c>
       <c r="D222" s="22" t="s">
-        <v>858</v>
+        <v>852</v>
       </c>
       <c r="E222" s="21" t="s">
-        <v>859</v>
+        <v>853</v>
       </c>
       <c r="F222" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G222" s="20">
-        <v>19750</v>
-      </c>
-      <c r="H222" s="23" t="s">
-        <v>1274</v>
-      </c>
-      <c r="I222" s="47">
-        <v>200000</v>
-      </c>
-      <c r="J222" s="23">
-        <v>198000</v>
-      </c>
-      <c r="K222" s="23">
-        <v>115500</v>
-      </c>
+      <c r="G222" s="20"/>
+      <c r="H222" s="23"/>
+      <c r="I222" s="23"/>
+      <c r="J222" s="23"/>
+      <c r="K222" s="23"/>
     </row>
     <row r="223" spans="1:11">
       <c r="A223" s="21" t="s">
         <v>860</v>
       </c>
       <c r="B223" s="21" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C223" s="21" t="s">
-        <v>174</v>
+        <v>210</v>
       </c>
       <c r="D223" s="22" t="s">
-        <v>861</v>
+        <v>855</v>
       </c>
       <c r="E223" s="21" t="s">
-        <v>862</v>
+        <v>856</v>
       </c>
       <c r="F223" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G223" s="20">
-        <v>10750</v>
-      </c>
-      <c r="H223" s="23" t="s">
-        <v>1274</v>
-      </c>
-      <c r="I223" s="47">
-        <v>100000</v>
-      </c>
-      <c r="J223" s="23">
-        <v>99000</v>
-      </c>
-      <c r="K223" s="23">
-        <v>57750</v>
-      </c>
+      <c r="G223" s="20"/>
+      <c r="H223" s="23"/>
+      <c r="I223" s="23"/>
+      <c r="J223" s="23"/>
+      <c r="K223" s="23"/>
     </row>
     <row r="224" spans="1:11">
       <c r="A224" s="21" t="s">
         <v>863</v>
       </c>
       <c r="B224" s="21" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C224" s="21" t="s">
-        <v>179</v>
+        <v>258</v>
       </c>
       <c r="D224" s="22" t="s">
-        <v>864</v>
+        <v>858</v>
       </c>
       <c r="E224" s="21" t="s">
-        <v>865</v>
+        <v>859</v>
       </c>
       <c r="F224" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G224" s="20">
-        <v>7200</v>
-      </c>
-      <c r="H224" s="23" t="s">
-        <v>1274</v>
-      </c>
-      <c r="I224" s="47">
-        <v>50000</v>
-      </c>
-      <c r="J224" s="23">
-        <v>48000</v>
-      </c>
-      <c r="K224" s="23">
-        <v>36000</v>
-      </c>
+      <c r="G224" s="20"/>
+      <c r="H224" s="23"/>
+      <c r="I224" s="23"/>
+      <c r="J224" s="23"/>
+      <c r="K224" s="23"/>
     </row>
     <row r="225" spans="1:11">
       <c r="A225" s="21" t="s">
@@ -14196,32 +14495,22 @@
         <v>115</v>
       </c>
       <c r="C225" s="21" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D225" s="22" t="s">
-        <v>867</v>
+        <v>861</v>
       </c>
       <c r="E225" s="21" t="s">
-        <v>868</v>
+        <v>862</v>
       </c>
       <c r="F225" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G225" s="20">
-        <v>10900</v>
-      </c>
-      <c r="H225" s="23" t="s">
-        <v>1277</v>
-      </c>
-      <c r="I225" s="47">
-        <v>80000</v>
-      </c>
-      <c r="J225" s="23">
-        <v>78000</v>
-      </c>
-      <c r="K225" s="23">
-        <v>45500</v>
-      </c>
+      <c r="G225" s="20"/>
+      <c r="H225" s="23"/>
+      <c r="I225" s="23"/>
+      <c r="J225" s="23"/>
+      <c r="K225" s="23"/>
     </row>
     <row r="226" spans="1:11">
       <c r="A226" s="21" t="s">
@@ -14231,32 +14520,22 @@
         <v>115</v>
       </c>
       <c r="C226" s="21" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="D226" s="22" t="s">
-        <v>870</v>
+        <v>864</v>
       </c>
       <c r="E226" s="21" t="s">
-        <v>871</v>
+        <v>865</v>
       </c>
       <c r="F226" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G226" s="20">
-        <v>8925</v>
-      </c>
-      <c r="H226" s="23" t="s">
-        <v>1277</v>
-      </c>
-      <c r="I226" s="47">
-        <v>100000</v>
-      </c>
-      <c r="J226" s="23">
-        <v>99000</v>
-      </c>
-      <c r="K226" s="23">
-        <v>49500</v>
-      </c>
+      <c r="G226" s="20"/>
+      <c r="H226" s="23"/>
+      <c r="I226" s="23"/>
+      <c r="J226" s="23"/>
+      <c r="K226" s="23"/>
     </row>
     <row r="227" spans="1:11">
       <c r="A227" s="21" t="s">
@@ -14266,21 +14545,19 @@
         <v>115</v>
       </c>
       <c r="C227" s="21" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="D227" s="22" t="s">
-        <v>873</v>
-      </c>
-      <c r="E227" s="21"/>
+        <v>867</v>
+      </c>
+      <c r="E227" s="21" t="s">
+        <v>868</v>
+      </c>
       <c r="F227" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G227" s="20">
-        <v>42925</v>
-      </c>
-      <c r="H227" s="23" t="s">
-        <v>1277</v>
-      </c>
+      <c r="G227" s="20"/>
+      <c r="H227" s="23"/>
       <c r="I227" s="23"/>
       <c r="J227" s="23"/>
       <c r="K227" s="23"/>
@@ -14290,19 +14567,19 @@
         <v>874</v>
       </c>
       <c r="B228" s="21" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C228" s="21" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
       <c r="D228" s="22" t="s">
-        <v>875</v>
+        <v>870</v>
       </c>
       <c r="E228" s="21" t="s">
-        <v>876</v>
+        <v>871</v>
       </c>
       <c r="F228" s="22" t="s">
-        <v>877</v>
+        <v>839</v>
       </c>
       <c r="G228" s="20"/>
       <c r="H228" s="23"/>
@@ -14315,19 +14592,17 @@
         <v>878</v>
       </c>
       <c r="B229" s="21" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C229" s="21" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="D229" s="22" t="s">
-        <v>879</v>
-      </c>
-      <c r="E229" s="21" t="s">
-        <v>880</v>
-      </c>
+        <v>873</v>
+      </c>
+      <c r="E229" s="21"/>
       <c r="F229" s="22" t="s">
-        <v>877</v>
+        <v>839</v>
       </c>
       <c r="G229" s="20"/>
       <c r="H229" s="23"/>
@@ -14343,13 +14618,13 @@
         <v>117</v>
       </c>
       <c r="C230" s="21" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D230" s="22" t="s">
-        <v>882</v>
+        <v>875</v>
       </c>
       <c r="E230" s="21" t="s">
-        <v>883</v>
+        <v>876</v>
       </c>
       <c r="F230" s="22" t="s">
         <v>877</v>
@@ -14368,13 +14643,13 @@
         <v>117</v>
       </c>
       <c r="C231" s="21" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="D231" s="22" t="s">
-        <v>885</v>
+        <v>879</v>
       </c>
       <c r="E231" s="21" t="s">
-        <v>886</v>
+        <v>880</v>
       </c>
       <c r="F231" s="22" t="s">
         <v>877</v>
@@ -14393,13 +14668,13 @@
         <v>117</v>
       </c>
       <c r="C232" s="21" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="D232" s="22" t="s">
-        <v>888</v>
+        <v>882</v>
       </c>
       <c r="E232" s="21" t="s">
-        <v>889</v>
+        <v>883</v>
       </c>
       <c r="F232" s="22" t="s">
         <v>877</v>
@@ -14418,13 +14693,13 @@
         <v>117</v>
       </c>
       <c r="C233" s="21" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="D233" s="22" t="s">
-        <v>891</v>
+        <v>885</v>
       </c>
       <c r="E233" s="21" t="s">
-        <v>892</v>
+        <v>886</v>
       </c>
       <c r="F233" s="22" t="s">
         <v>877</v>
@@ -14443,13 +14718,13 @@
         <v>117</v>
       </c>
       <c r="C234" s="21" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="D234" s="22" t="s">
-        <v>894</v>
+        <v>888</v>
       </c>
       <c r="E234" s="21" t="s">
-        <v>895</v>
+        <v>889</v>
       </c>
       <c r="F234" s="22" t="s">
         <v>877</v>
@@ -14468,13 +14743,13 @@
         <v>117</v>
       </c>
       <c r="C235" s="21" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="D235" s="22" t="s">
-        <v>897</v>
+        <v>891</v>
       </c>
       <c r="E235" s="21" t="s">
-        <v>898</v>
+        <v>892</v>
       </c>
       <c r="F235" s="22" t="s">
         <v>877</v>
@@ -14493,13 +14768,13 @@
         <v>117</v>
       </c>
       <c r="C236" s="21" t="s">
-        <v>258</v>
+        <v>206</v>
       </c>
       <c r="D236" s="22" t="s">
-        <v>900</v>
+        <v>894</v>
       </c>
       <c r="E236" s="21" t="s">
-        <v>901</v>
+        <v>895</v>
       </c>
       <c r="F236" s="22" t="s">
         <v>877</v>
@@ -14518,13 +14793,13 @@
         <v>117</v>
       </c>
       <c r="C237" s="21" t="s">
-        <v>262</v>
+        <v>210</v>
       </c>
       <c r="D237" s="22" t="s">
-        <v>903</v>
+        <v>897</v>
       </c>
       <c r="E237" s="21" t="s">
-        <v>904</v>
+        <v>898</v>
       </c>
       <c r="F237" s="22" t="s">
         <v>877</v>
@@ -14543,13 +14818,13 @@
         <v>117</v>
       </c>
       <c r="C238" s="21" t="s">
-        <v>296</v>
+        <v>258</v>
       </c>
       <c r="D238" s="22" t="s">
-        <v>906</v>
+        <v>900</v>
       </c>
       <c r="E238" s="21" t="s">
-        <v>907</v>
+        <v>901</v>
       </c>
       <c r="F238" s="22" t="s">
         <v>877</v>
@@ -14568,13 +14843,13 @@
         <v>117</v>
       </c>
       <c r="C239" s="21" t="s">
-        <v>300</v>
+        <v>262</v>
       </c>
       <c r="D239" s="22" t="s">
-        <v>909</v>
+        <v>903</v>
       </c>
       <c r="E239" s="21" t="s">
-        <v>910</v>
+        <v>904</v>
       </c>
       <c r="F239" s="22" t="s">
         <v>877</v>
@@ -14593,13 +14868,13 @@
         <v>117</v>
       </c>
       <c r="C240" s="21" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="D240" s="22" t="s">
-        <v>912</v>
+        <v>906</v>
       </c>
       <c r="E240" s="21" t="s">
-        <v>913</v>
+        <v>907</v>
       </c>
       <c r="F240" s="22" t="s">
         <v>877</v>
@@ -14618,13 +14893,13 @@
         <v>117</v>
       </c>
       <c r="C241" s="21" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
       <c r="D241" s="22" t="s">
-        <v>915</v>
+        <v>909</v>
       </c>
       <c r="E241" s="21" t="s">
-        <v>916</v>
+        <v>910</v>
       </c>
       <c r="F241" s="22" t="s">
         <v>877</v>
@@ -14640,19 +14915,19 @@
         <v>917</v>
       </c>
       <c r="B242" s="21" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="C242" s="21" t="s">
-        <v>174</v>
+        <v>304</v>
       </c>
       <c r="D242" s="22" t="s">
-        <v>918</v>
+        <v>912</v>
       </c>
       <c r="E242" s="21" t="s">
-        <v>919</v>
+        <v>913</v>
       </c>
       <c r="F242" s="22" t="s">
-        <v>920</v>
+        <v>877</v>
       </c>
       <c r="G242" s="20"/>
       <c r="H242" s="23"/>
@@ -14665,19 +14940,19 @@
         <v>921</v>
       </c>
       <c r="B243" s="21" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="C243" s="21" t="s">
-        <v>179</v>
+        <v>308</v>
       </c>
       <c r="D243" s="22" t="s">
-        <v>922</v>
+        <v>915</v>
       </c>
       <c r="E243" s="21" t="s">
-        <v>923</v>
+        <v>916</v>
       </c>
       <c r="F243" s="22" t="s">
-        <v>920</v>
+        <v>877</v>
       </c>
       <c r="G243" s="20"/>
       <c r="H243" s="23"/>
@@ -14693,13 +14968,13 @@
         <v>122</v>
       </c>
       <c r="C244" s="21" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D244" s="22" t="s">
-        <v>925</v>
+        <v>918</v>
       </c>
       <c r="E244" s="21" t="s">
-        <v>926</v>
+        <v>919</v>
       </c>
       <c r="F244" s="22" t="s">
         <v>920</v>
@@ -14718,13 +14993,13 @@
         <v>122</v>
       </c>
       <c r="C245" s="21" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="D245" s="22" t="s">
-        <v>928</v>
+        <v>922</v>
       </c>
       <c r="E245" s="21" t="s">
-        <v>929</v>
+        <v>923</v>
       </c>
       <c r="F245" s="22" t="s">
         <v>920</v>
@@ -14743,13 +15018,13 @@
         <v>122</v>
       </c>
       <c r="C246" s="21" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="D246" s="22" t="s">
-        <v>931</v>
+        <v>925</v>
       </c>
       <c r="E246" s="21" t="s">
-        <v>932</v>
+        <v>926</v>
       </c>
       <c r="F246" s="22" t="s">
         <v>920</v>
@@ -14768,13 +15043,13 @@
         <v>122</v>
       </c>
       <c r="C247" s="21" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="D247" s="22" t="s">
-        <v>934</v>
+        <v>928</v>
       </c>
       <c r="E247" s="21" t="s">
-        <v>935</v>
+        <v>929</v>
       </c>
       <c r="F247" s="22" t="s">
         <v>920</v>
@@ -14793,13 +15068,13 @@
         <v>122</v>
       </c>
       <c r="C248" s="21" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="D248" s="22" t="s">
-        <v>937</v>
+        <v>931</v>
       </c>
       <c r="E248" s="21" t="s">
-        <v>938</v>
+        <v>932</v>
       </c>
       <c r="F248" s="22" t="s">
         <v>920</v>
@@ -14815,19 +15090,19 @@
         <v>939</v>
       </c>
       <c r="B249" s="21" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C249" s="21" t="s">
-        <v>174</v>
+        <v>202</v>
       </c>
       <c r="D249" s="22" t="s">
-        <v>940</v>
+        <v>934</v>
       </c>
       <c r="E249" s="21" t="s">
-        <v>941</v>
+        <v>935</v>
       </c>
       <c r="F249" s="22" t="s">
-        <v>942</v>
+        <v>920</v>
       </c>
       <c r="G249" s="20"/>
       <c r="H249" s="23"/>
@@ -14840,19 +15115,19 @@
         <v>943</v>
       </c>
       <c r="B250" s="21" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C250" s="21" t="s">
-        <v>179</v>
+        <v>206</v>
       </c>
       <c r="D250" s="22" t="s">
-        <v>944</v>
+        <v>937</v>
       </c>
       <c r="E250" s="21" t="s">
-        <v>945</v>
+        <v>938</v>
       </c>
       <c r="F250" s="22" t="s">
-        <v>942</v>
+        <v>920</v>
       </c>
       <c r="G250" s="20"/>
       <c r="H250" s="23"/>
@@ -14868,13 +15143,13 @@
         <v>125</v>
       </c>
       <c r="C251" s="21" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D251" s="22" t="s">
-        <v>947</v>
+        <v>940</v>
       </c>
       <c r="E251" s="21" t="s">
-        <v>948</v>
+        <v>941</v>
       </c>
       <c r="F251" s="22" t="s">
         <v>942</v>
@@ -14893,13 +15168,13 @@
         <v>125</v>
       </c>
       <c r="C252" s="21" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="D252" s="22" t="s">
-        <v>950</v>
+        <v>944</v>
       </c>
       <c r="E252" s="21" t="s">
-        <v>951</v>
+        <v>945</v>
       </c>
       <c r="F252" s="22" t="s">
         <v>942</v>
@@ -14918,13 +15193,13 @@
         <v>125</v>
       </c>
       <c r="C253" s="21" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="D253" s="22" t="s">
-        <v>931</v>
+        <v>947</v>
       </c>
       <c r="E253" s="21" t="s">
-        <v>953</v>
+        <v>948</v>
       </c>
       <c r="F253" s="22" t="s">
         <v>942</v>
@@ -14943,13 +15218,13 @@
         <v>125</v>
       </c>
       <c r="C254" s="21" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="D254" s="22" t="s">
-        <v>955</v>
+        <v>950</v>
       </c>
       <c r="E254" s="21" t="s">
-        <v>956</v>
+        <v>951</v>
       </c>
       <c r="F254" s="22" t="s">
         <v>942</v>
@@ -14968,13 +15243,13 @@
         <v>125</v>
       </c>
       <c r="C255" s="21" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="D255" s="22" t="s">
-        <v>958</v>
+        <v>931</v>
       </c>
       <c r="E255" s="21" t="s">
-        <v>959</v>
+        <v>953</v>
       </c>
       <c r="F255" s="22" t="s">
         <v>942</v>
@@ -14993,13 +15268,13 @@
         <v>125</v>
       </c>
       <c r="C256" s="21" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="D256" s="22" t="s">
-        <v>961</v>
+        <v>955</v>
       </c>
       <c r="E256" s="21" t="s">
-        <v>962</v>
+        <v>956</v>
       </c>
       <c r="F256" s="22" t="s">
         <v>942</v>
@@ -15018,13 +15293,13 @@
         <v>125</v>
       </c>
       <c r="C257" s="21" t="s">
-        <v>258</v>
+        <v>206</v>
       </c>
       <c r="D257" s="22" t="s">
-        <v>964</v>
+        <v>958</v>
       </c>
       <c r="E257" s="21" t="s">
-        <v>965</v>
+        <v>959</v>
       </c>
       <c r="F257" s="22" t="s">
         <v>942</v>
@@ -15043,13 +15318,13 @@
         <v>125</v>
       </c>
       <c r="C258" s="21" t="s">
-        <v>262</v>
+        <v>210</v>
       </c>
       <c r="D258" s="22" t="s">
-        <v>967</v>
+        <v>961</v>
       </c>
       <c r="E258" s="21" t="s">
-        <v>968</v>
+        <v>962</v>
       </c>
       <c r="F258" s="22" t="s">
         <v>942</v>
@@ -15068,13 +15343,13 @@
         <v>125</v>
       </c>
       <c r="C259" s="21" t="s">
-        <v>296</v>
+        <v>258</v>
       </c>
       <c r="D259" s="22" t="s">
-        <v>970</v>
+        <v>964</v>
       </c>
       <c r="E259" s="21" t="s">
-        <v>971</v>
+        <v>965</v>
       </c>
       <c r="F259" s="22" t="s">
         <v>942</v>
@@ -15093,13 +15368,13 @@
         <v>125</v>
       </c>
       <c r="C260" s="21" t="s">
-        <v>300</v>
+        <v>262</v>
       </c>
       <c r="D260" s="22" t="s">
-        <v>973</v>
+        <v>967</v>
       </c>
       <c r="E260" s="21" t="s">
-        <v>974</v>
+        <v>968</v>
       </c>
       <c r="F260" s="22" t="s">
         <v>942</v>
@@ -15118,13 +15393,13 @@
         <v>125</v>
       </c>
       <c r="C261" s="21" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="D261" s="22" t="s">
-        <v>976</v>
+        <v>970</v>
       </c>
       <c r="E261" s="21" t="s">
-        <v>977</v>
+        <v>971</v>
       </c>
       <c r="F261" s="22" t="s">
         <v>942</v>
@@ -15143,13 +15418,13 @@
         <v>125</v>
       </c>
       <c r="C262" s="21" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
       <c r="D262" s="22" t="s">
-        <v>979</v>
+        <v>973</v>
       </c>
       <c r="E262" s="21" t="s">
-        <v>980</v>
+        <v>974</v>
       </c>
       <c r="F262" s="22" t="s">
         <v>942</v>
@@ -15165,19 +15440,19 @@
         <v>981</v>
       </c>
       <c r="B263" s="21" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C263" s="21" t="s">
-        <v>174</v>
+        <v>304</v>
       </c>
       <c r="D263" s="22" t="s">
-        <v>982</v>
+        <v>976</v>
       </c>
       <c r="E263" s="21" t="s">
-        <v>983</v>
+        <v>977</v>
       </c>
       <c r="F263" s="22" t="s">
-        <v>984</v>
+        <v>942</v>
       </c>
       <c r="G263" s="20"/>
       <c r="H263" s="23"/>
@@ -15190,19 +15465,19 @@
         <v>985</v>
       </c>
       <c r="B264" s="21" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C264" s="21" t="s">
-        <v>179</v>
+        <v>308</v>
       </c>
       <c r="D264" s="22" t="s">
-        <v>986</v>
+        <v>979</v>
       </c>
       <c r="E264" s="21" t="s">
-        <v>987</v>
+        <v>980</v>
       </c>
       <c r="F264" s="22" t="s">
-        <v>984</v>
+        <v>942</v>
       </c>
       <c r="G264" s="20"/>
       <c r="H264" s="23"/>
@@ -15218,13 +15493,13 @@
         <v>128</v>
       </c>
       <c r="C265" s="21" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D265" s="22" t="s">
-        <v>989</v>
+        <v>982</v>
       </c>
       <c r="E265" s="21" t="s">
-        <v>990</v>
+        <v>983</v>
       </c>
       <c r="F265" s="22" t="s">
         <v>984</v>
@@ -15243,13 +15518,13 @@
         <v>128</v>
       </c>
       <c r="C266" s="21" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="D266" s="22" t="s">
-        <v>992</v>
+        <v>986</v>
       </c>
       <c r="E266" s="21" t="s">
-        <v>993</v>
+        <v>987</v>
       </c>
       <c r="F266" s="22" t="s">
         <v>984</v>
@@ -15268,13 +15543,13 @@
         <v>128</v>
       </c>
       <c r="C267" s="21" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="D267" s="22" t="s">
-        <v>995</v>
+        <v>989</v>
       </c>
       <c r="E267" s="21" t="s">
-        <v>996</v>
+        <v>990</v>
       </c>
       <c r="F267" s="22" t="s">
         <v>984</v>
@@ -15293,13 +15568,13 @@
         <v>128</v>
       </c>
       <c r="C268" s="21" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="D268" s="22" t="s">
-        <v>998</v>
+        <v>992</v>
       </c>
       <c r="E268" s="21" t="s">
-        <v>999</v>
+        <v>993</v>
       </c>
       <c r="F268" s="22" t="s">
         <v>984</v>
@@ -15318,13 +15593,13 @@
         <v>128</v>
       </c>
       <c r="C269" s="21" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="D269" s="22" t="s">
-        <v>1001</v>
+        <v>995</v>
       </c>
       <c r="E269" s="21" t="s">
-        <v>1002</v>
+        <v>996</v>
       </c>
       <c r="F269" s="22" t="s">
         <v>984</v>
@@ -15340,19 +15615,19 @@
         <v>1003</v>
       </c>
       <c r="B270" s="21" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C270" s="21" t="s">
-        <v>174</v>
+        <v>202</v>
       </c>
       <c r="D270" s="22" t="s">
-        <v>1004</v>
+        <v>998</v>
       </c>
       <c r="E270" s="21" t="s">
-        <v>1005</v>
+        <v>999</v>
       </c>
       <c r="F270" s="22" t="s">
-        <v>1006</v>
+        <v>984</v>
       </c>
       <c r="G270" s="20"/>
       <c r="H270" s="23"/>
@@ -15365,19 +15640,19 @@
         <v>1007</v>
       </c>
       <c r="B271" s="21" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C271" s="21" t="s">
-        <v>179</v>
+        <v>206</v>
       </c>
       <c r="D271" s="22" t="s">
-        <v>1008</v>
+        <v>1001</v>
       </c>
       <c r="E271" s="21" t="s">
-        <v>1009</v>
+        <v>1002</v>
       </c>
       <c r="F271" s="22" t="s">
-        <v>1006</v>
+        <v>984</v>
       </c>
       <c r="G271" s="20"/>
       <c r="H271" s="23"/>
@@ -15390,19 +15665,19 @@
         <v>1010</v>
       </c>
       <c r="B272" s="21" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C272" s="21" t="s">
         <v>174</v>
       </c>
       <c r="D272" s="22" t="s">
-        <v>1011</v>
+        <v>1004</v>
       </c>
       <c r="E272" s="21" t="s">
-        <v>1012</v>
+        <v>1005</v>
       </c>
       <c r="F272" s="22" t="s">
-        <v>1013</v>
+        <v>1006</v>
       </c>
       <c r="G272" s="20"/>
       <c r="H272" s="23"/>
@@ -15415,19 +15690,19 @@
         <v>1014</v>
       </c>
       <c r="B273" s="21" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C273" s="21" t="s">
         <v>179</v>
       </c>
       <c r="D273" s="22" t="s">
-        <v>1015</v>
+        <v>1008</v>
       </c>
       <c r="E273" s="21" t="s">
-        <v>1016</v>
+        <v>1009</v>
       </c>
       <c r="F273" s="22" t="s">
-        <v>1013</v>
+        <v>1006</v>
       </c>
       <c r="G273" s="20"/>
       <c r="H273" s="23"/>
@@ -15443,13 +15718,13 @@
         <v>132</v>
       </c>
       <c r="C274" s="21" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D274" s="22" t="s">
-        <v>1018</v>
+        <v>1011</v>
       </c>
       <c r="E274" s="21" t="s">
-        <v>1019</v>
+        <v>1012</v>
       </c>
       <c r="F274" s="22" t="s">
         <v>1013</v>
@@ -15468,13 +15743,13 @@
         <v>132</v>
       </c>
       <c r="C275" s="21" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="D275" s="22" t="s">
-        <v>1021</v>
+        <v>1015</v>
       </c>
       <c r="E275" s="21" t="s">
-        <v>1022</v>
+        <v>1016</v>
       </c>
       <c r="F275" s="22" t="s">
         <v>1013</v>
@@ -15490,19 +15765,19 @@
         <v>1023</v>
       </c>
       <c r="B276" s="21" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C276" s="21" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="D276" s="22" t="s">
-        <v>1024</v>
+        <v>1018</v>
       </c>
       <c r="E276" s="21" t="s">
-        <v>1025</v>
+        <v>1019</v>
       </c>
       <c r="F276" s="22" t="s">
-        <v>1026</v>
+        <v>1013</v>
       </c>
       <c r="G276" s="20"/>
       <c r="H276" s="23"/>
@@ -15515,19 +15790,19 @@
         <v>1027</v>
       </c>
       <c r="B277" s="21" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C277" s="21" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
       <c r="D277" s="22" t="s">
-        <v>1028</v>
+        <v>1021</v>
       </c>
       <c r="E277" s="21" t="s">
-        <v>1029</v>
+        <v>1022</v>
       </c>
       <c r="F277" s="22" t="s">
-        <v>1030</v>
+        <v>1013</v>
       </c>
       <c r="G277" s="20"/>
       <c r="H277" s="23"/>
@@ -15540,19 +15815,19 @@
         <v>1031</v>
       </c>
       <c r="B278" s="21" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C278" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D278" s="22" t="s">
-        <v>1032</v>
+        <v>1024</v>
       </c>
       <c r="E278" s="21" t="s">
-        <v>1033</v>
+        <v>1025</v>
       </c>
       <c r="F278" s="22" t="s">
-        <v>1030</v>
+        <v>1026</v>
       </c>
       <c r="G278" s="20"/>
       <c r="H278" s="23"/>
@@ -15568,13 +15843,13 @@
         <v>135</v>
       </c>
       <c r="C279" s="21" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D279" s="22" t="s">
-        <v>1035</v>
+        <v>1028</v>
       </c>
       <c r="E279" s="21" t="s">
-        <v>1036</v>
+        <v>1029</v>
       </c>
       <c r="F279" s="22" t="s">
         <v>1030</v>
@@ -15593,13 +15868,13 @@
         <v>135</v>
       </c>
       <c r="C280" s="21" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="D280" s="22" t="s">
-        <v>1038</v>
+        <v>1032</v>
       </c>
       <c r="E280" s="21" t="s">
-        <v>1039</v>
+        <v>1033</v>
       </c>
       <c r="F280" s="22" t="s">
         <v>1030</v>
@@ -15618,13 +15893,13 @@
         <v>135</v>
       </c>
       <c r="C281" s="21" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="D281" s="22" t="s">
-        <v>1041</v>
+        <v>1035</v>
       </c>
       <c r="E281" s="21" t="s">
-        <v>1042</v>
+        <v>1036</v>
       </c>
       <c r="F281" s="22" t="s">
         <v>1030</v>
@@ -15640,19 +15915,19 @@
         <v>1043</v>
       </c>
       <c r="B282" s="21" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C282" s="21" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
       <c r="D282" s="22" t="s">
-        <v>1044</v>
+        <v>1038</v>
       </c>
       <c r="E282" s="21" t="s">
-        <v>1045</v>
+        <v>1039</v>
       </c>
       <c r="F282" s="22" t="s">
-        <v>1046</v>
+        <v>1030</v>
       </c>
       <c r="G282" s="20"/>
       <c r="H282" s="23"/>
@@ -15665,19 +15940,19 @@
         <v>1047</v>
       </c>
       <c r="B283" s="21" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C283" s="21" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="D283" s="22" t="s">
-        <v>1048</v>
+        <v>1041</v>
       </c>
       <c r="E283" s="21" t="s">
-        <v>1049</v>
+        <v>1042</v>
       </c>
       <c r="F283" s="22" t="s">
-        <v>1046</v>
+        <v>1030</v>
       </c>
       <c r="G283" s="20"/>
       <c r="H283" s="23"/>
@@ -15693,13 +15968,13 @@
         <v>137</v>
       </c>
       <c r="C284" s="21" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D284" s="22" t="s">
-        <v>1051</v>
+        <v>1044</v>
       </c>
       <c r="E284" s="21" t="s">
-        <v>1052</v>
+        <v>1045</v>
       </c>
       <c r="F284" s="22" t="s">
         <v>1046</v>
@@ -15718,13 +15993,13 @@
         <v>137</v>
       </c>
       <c r="C285" s="21" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="D285" s="22" t="s">
-        <v>1054</v>
+        <v>1048</v>
       </c>
       <c r="E285" s="21" t="s">
-        <v>1055</v>
+        <v>1049</v>
       </c>
       <c r="F285" s="22" t="s">
         <v>1046</v>
@@ -15740,19 +16015,19 @@
         <v>1056</v>
       </c>
       <c r="B286" s="21" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C286" s="21" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="D286" s="22" t="s">
-        <v>1057</v>
+        <v>1051</v>
       </c>
       <c r="E286" s="21" t="s">
-        <v>1058</v>
+        <v>1052</v>
       </c>
       <c r="F286" s="22" t="s">
-        <v>1059</v>
+        <v>1046</v>
       </c>
       <c r="G286" s="20"/>
       <c r="H286" s="23"/>
@@ -15765,19 +16040,19 @@
         <v>1060</v>
       </c>
       <c r="B287" s="21" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C287" s="21" t="s">
-        <v>179</v>
+        <v>194</v>
       </c>
       <c r="D287" s="22" t="s">
-        <v>1061</v>
+        <v>1054</v>
       </c>
       <c r="E287" s="21" t="s">
-        <v>1062</v>
+        <v>1055</v>
       </c>
       <c r="F287" s="22" t="s">
-        <v>1059</v>
+        <v>1046</v>
       </c>
       <c r="G287" s="20"/>
       <c r="H287" s="23"/>
@@ -15793,13 +16068,13 @@
         <v>140</v>
       </c>
       <c r="C288" s="21" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D288" s="22" t="s">
-        <v>1064</v>
+        <v>1057</v>
       </c>
       <c r="E288" s="21" t="s">
-        <v>1065</v>
+        <v>1058</v>
       </c>
       <c r="F288" s="22" t="s">
         <v>1059</v>
@@ -15818,13 +16093,13 @@
         <v>140</v>
       </c>
       <c r="C289" s="21" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="D289" s="22" t="s">
-        <v>1067</v>
+        <v>1061</v>
       </c>
       <c r="E289" s="21" t="s">
-        <v>1068</v>
+        <v>1062</v>
       </c>
       <c r="F289" s="22" t="s">
         <v>1059</v>
@@ -15840,16 +16115,16 @@
         <v>1069</v>
       </c>
       <c r="B290" s="21" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C290" s="21" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="D290" s="22" t="s">
-        <v>1070</v>
+        <v>1064</v>
       </c>
       <c r="E290" s="21" t="s">
-        <v>1071</v>
+        <v>1065</v>
       </c>
       <c r="F290" s="22" t="s">
         <v>1059</v>
@@ -15865,16 +16140,16 @@
         <v>1072</v>
       </c>
       <c r="B291" s="21" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C291" s="21" t="s">
-        <v>179</v>
+        <v>194</v>
       </c>
       <c r="D291" s="22" t="s">
-        <v>1073</v>
+        <v>1067</v>
       </c>
       <c r="E291" s="21" t="s">
-        <v>1074</v>
+        <v>1068</v>
       </c>
       <c r="F291" s="22" t="s">
         <v>1059</v>
@@ -15893,13 +16168,13 @@
         <v>142</v>
       </c>
       <c r="C292" s="21" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D292" s="22" t="s">
-        <v>1076</v>
+        <v>1070</v>
       </c>
       <c r="E292" s="21" t="s">
-        <v>1077</v>
+        <v>1071</v>
       </c>
       <c r="F292" s="22" t="s">
         <v>1059</v>
@@ -15918,13 +16193,13 @@
         <v>142</v>
       </c>
       <c r="C293" s="21" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="D293" s="22" t="s">
-        <v>1079</v>
+        <v>1073</v>
       </c>
       <c r="E293" s="21" t="s">
-        <v>1080</v>
+        <v>1074</v>
       </c>
       <c r="F293" s="22" t="s">
         <v>1059</v>
@@ -15943,13 +16218,13 @@
         <v>142</v>
       </c>
       <c r="C294" s="21" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="D294" s="22" t="s">
-        <v>1082</v>
+        <v>1076</v>
       </c>
       <c r="E294" s="21" t="s">
-        <v>1083</v>
+        <v>1077</v>
       </c>
       <c r="F294" s="22" t="s">
         <v>1059</v>
@@ -15968,13 +16243,13 @@
         <v>142</v>
       </c>
       <c r="C295" s="21" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="D295" s="22" t="s">
-        <v>1085</v>
+        <v>1079</v>
       </c>
       <c r="E295" s="21" t="s">
-        <v>1086</v>
+        <v>1080</v>
       </c>
       <c r="F295" s="22" t="s">
         <v>1059</v>
@@ -15993,13 +16268,13 @@
         <v>142</v>
       </c>
       <c r="C296" s="21" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="D296" s="22" t="s">
-        <v>1088</v>
+        <v>1082</v>
       </c>
       <c r="E296" s="21" t="s">
-        <v>1089</v>
+        <v>1083</v>
       </c>
       <c r="F296" s="22" t="s">
         <v>1059</v>
@@ -16015,19 +16290,19 @@
         <v>1090</v>
       </c>
       <c r="B297" s="21" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C297" s="21" t="s">
-        <v>174</v>
+        <v>202</v>
       </c>
       <c r="D297" s="22" t="s">
-        <v>1091</v>
+        <v>1085</v>
       </c>
       <c r="E297" s="21" t="s">
-        <v>1092</v>
+        <v>1086</v>
       </c>
       <c r="F297" s="22" t="s">
-        <v>1093</v>
+        <v>1059</v>
       </c>
       <c r="G297" s="20"/>
       <c r="H297" s="23"/>
@@ -16040,19 +16315,19 @@
         <v>1094</v>
       </c>
       <c r="B298" s="21" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C298" s="21" t="s">
-        <v>174</v>
+        <v>206</v>
       </c>
       <c r="D298" s="22" t="s">
-        <v>1095</v>
+        <v>1088</v>
       </c>
       <c r="E298" s="21" t="s">
-        <v>1096</v>
+        <v>1089</v>
       </c>
       <c r="F298" s="22" t="s">
-        <v>1097</v>
+        <v>1059</v>
       </c>
       <c r="G298" s="20"/>
       <c r="H298" s="23"/>
@@ -16065,19 +16340,19 @@
         <v>1098</v>
       </c>
       <c r="B299" s="21" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C299" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D299" s="22" t="s">
-        <v>1099</v>
+        <v>1091</v>
       </c>
       <c r="E299" s="21" t="s">
-        <v>1100</v>
+        <v>1092</v>
       </c>
       <c r="F299" s="22" t="s">
-        <v>1097</v>
+        <v>1093</v>
       </c>
       <c r="G299" s="20"/>
       <c r="H299" s="23"/>
@@ -16093,13 +16368,13 @@
         <v>146</v>
       </c>
       <c r="C300" s="21" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D300" s="22" t="s">
-        <v>1102</v>
+        <v>1095</v>
       </c>
       <c r="E300" s="21" t="s">
-        <v>1103</v>
+        <v>1096</v>
       </c>
       <c r="F300" s="22" t="s">
         <v>1097</v>
@@ -16115,19 +16390,19 @@
         <v>1104</v>
       </c>
       <c r="B301" s="21" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C301" s="21" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="D301" s="22" t="s">
-        <v>1105</v>
+        <v>1099</v>
       </c>
       <c r="E301" s="21" t="s">
-        <v>1106</v>
+        <v>1100</v>
       </c>
       <c r="F301" s="22" t="s">
-        <v>1107</v>
+        <v>1097</v>
       </c>
       <c r="G301" s="20"/>
       <c r="H301" s="23"/>
@@ -16140,19 +16415,19 @@
         <v>1108</v>
       </c>
       <c r="B302" s="21" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C302" s="21" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="D302" s="22" t="s">
-        <v>1109</v>
+        <v>1102</v>
       </c>
       <c r="E302" s="21" t="s">
-        <v>1110</v>
+        <v>1103</v>
       </c>
       <c r="F302" s="22" t="s">
-        <v>1107</v>
+        <v>1097</v>
       </c>
       <c r="G302" s="20"/>
       <c r="H302" s="23"/>
@@ -16168,13 +16443,13 @@
         <v>147</v>
       </c>
       <c r="C303" s="21" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D303" s="22" t="s">
-        <v>1112</v>
+        <v>1105</v>
       </c>
       <c r="E303" s="21" t="s">
-        <v>1113</v>
+        <v>1106</v>
       </c>
       <c r="F303" s="22" t="s">
         <v>1107</v>
@@ -16190,19 +16465,19 @@
         <v>1114</v>
       </c>
       <c r="B304" s="21" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C304" s="21" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="D304" s="22" t="s">
-        <v>1115</v>
+        <v>1109</v>
       </c>
       <c r="E304" s="21" t="s">
-        <v>1116</v>
+        <v>1110</v>
       </c>
       <c r="F304" s="22" t="s">
-        <v>1117</v>
+        <v>1107</v>
       </c>
       <c r="G304" s="20"/>
       <c r="H304" s="23"/>
@@ -16215,19 +16490,19 @@
         <v>1118</v>
       </c>
       <c r="B305" s="21" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C305" s="21" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="D305" s="22" t="s">
-        <v>1119</v>
+        <v>1112</v>
       </c>
       <c r="E305" s="21" t="s">
-        <v>1120</v>
+        <v>1113</v>
       </c>
       <c r="F305" s="22" t="s">
-        <v>1117</v>
+        <v>1107</v>
       </c>
       <c r="G305" s="20"/>
       <c r="H305" s="23"/>
@@ -16243,13 +16518,13 @@
         <v>148</v>
       </c>
       <c r="C306" s="21" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D306" s="22" t="s">
-        <v>1122</v>
+        <v>1115</v>
       </c>
       <c r="E306" s="21" t="s">
-        <v>1123</v>
+        <v>1116</v>
       </c>
       <c r="F306" s="22" t="s">
         <v>1117</v>
@@ -16268,13 +16543,13 @@
         <v>148</v>
       </c>
       <c r="C307" s="21" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="D307" s="22" t="s">
-        <v>1115</v>
+        <v>1119</v>
       </c>
       <c r="E307" s="21" t="s">
-        <v>1116</v>
+        <v>1120</v>
       </c>
       <c r="F307" s="22" t="s">
         <v>1117</v>
@@ -16293,13 +16568,13 @@
         <v>148</v>
       </c>
       <c r="C308" s="21" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="D308" s="22" t="s">
-        <v>1126</v>
+        <v>1122</v>
       </c>
       <c r="E308" s="21" t="s">
-        <v>1127</v>
+        <v>1123</v>
       </c>
       <c r="F308" s="22" t="s">
         <v>1117</v>
@@ -16318,13 +16593,13 @@
         <v>148</v>
       </c>
       <c r="C309" s="21" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="D309" s="22" t="s">
-        <v>1129</v>
+        <v>1115</v>
       </c>
       <c r="E309" s="21" t="s">
-        <v>1130</v>
+        <v>1116</v>
       </c>
       <c r="F309" s="22" t="s">
         <v>1117</v>
@@ -16340,19 +16615,19 @@
         <v>1131</v>
       </c>
       <c r="B310" s="21" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C310" s="21" t="s">
-        <v>174</v>
+        <v>198</v>
       </c>
       <c r="D310" s="22" t="s">
-        <v>1132</v>
+        <v>1126</v>
       </c>
       <c r="E310" s="21" t="s">
-        <v>1133</v>
+        <v>1127</v>
       </c>
       <c r="F310" s="22" t="s">
-        <v>1134</v>
+        <v>1117</v>
       </c>
       <c r="G310" s="20"/>
       <c r="H310" s="23"/>
@@ -16365,19 +16640,19 @@
         <v>1135</v>
       </c>
       <c r="B311" s="21" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C311" s="21" t="s">
-        <v>179</v>
+        <v>202</v>
       </c>
       <c r="D311" s="22" t="s">
-        <v>1136</v>
+        <v>1129</v>
       </c>
       <c r="E311" s="21" t="s">
-        <v>1137</v>
+        <v>1130</v>
       </c>
       <c r="F311" s="22" t="s">
-        <v>1134</v>
+        <v>1117</v>
       </c>
       <c r="G311" s="20"/>
       <c r="H311" s="23"/>
@@ -16390,19 +16665,19 @@
         <v>1138</v>
       </c>
       <c r="B312" s="21" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C312" s="21" t="s">
         <v>174</v>
       </c>
       <c r="D312" s="22" t="s">
-        <v>1139</v>
+        <v>1132</v>
       </c>
       <c r="E312" s="21" t="s">
-        <v>1140</v>
+        <v>1133</v>
       </c>
       <c r="F312" s="22" t="s">
-        <v>1141</v>
+        <v>1134</v>
       </c>
       <c r="G312" s="20"/>
       <c r="H312" s="23"/>
@@ -16415,19 +16690,19 @@
         <v>1142</v>
       </c>
       <c r="B313" s="21" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C313" s="21" t="s">
         <v>179</v>
       </c>
       <c r="D313" s="22" t="s">
-        <v>1143</v>
+        <v>1136</v>
       </c>
       <c r="E313" s="21" t="s">
-        <v>1144</v>
+        <v>1137</v>
       </c>
       <c r="F313" s="22" t="s">
-        <v>1141</v>
+        <v>1134</v>
       </c>
       <c r="G313" s="20"/>
       <c r="H313" s="23"/>
@@ -16440,19 +16715,19 @@
         <v>1145</v>
       </c>
       <c r="B314" s="21" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C314" s="21" t="s">
         <v>174</v>
       </c>
       <c r="D314" s="22" t="s">
-        <v>1146</v>
+        <v>1139</v>
       </c>
       <c r="E314" s="21" t="s">
-        <v>1147</v>
+        <v>1140</v>
       </c>
       <c r="F314" s="22" t="s">
-        <v>1148</v>
+        <v>1141</v>
       </c>
       <c r="G314" s="20"/>
       <c r="H314" s="23"/>
@@ -16465,19 +16740,19 @@
         <v>1149</v>
       </c>
       <c r="B315" s="21" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C315" s="21" t="s">
         <v>179</v>
       </c>
       <c r="D315" s="22" t="s">
-        <v>1150</v>
+        <v>1143</v>
       </c>
       <c r="E315" s="21" t="s">
-        <v>1151</v>
+        <v>1144</v>
       </c>
       <c r="F315" s="22" t="s">
-        <v>1148</v>
+        <v>1141</v>
       </c>
       <c r="G315" s="20"/>
       <c r="H315" s="23"/>
@@ -16493,13 +16768,13 @@
         <v>155</v>
       </c>
       <c r="C316" s="21" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D316" s="22" t="s">
-        <v>1153</v>
+        <v>1146</v>
       </c>
       <c r="E316" s="21" t="s">
-        <v>1154</v>
+        <v>1147</v>
       </c>
       <c r="F316" s="22" t="s">
         <v>1148</v>
@@ -16518,13 +16793,13 @@
         <v>155</v>
       </c>
       <c r="C317" s="21" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="D317" s="22" t="s">
-        <v>1156</v>
+        <v>1150</v>
       </c>
       <c r="E317" s="21" t="s">
-        <v>1157</v>
+        <v>1151</v>
       </c>
       <c r="F317" s="22" t="s">
         <v>1148</v>
@@ -16543,13 +16818,13 @@
         <v>155</v>
       </c>
       <c r="C318" s="21" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="D318" s="22" t="s">
-        <v>1159</v>
+        <v>1153</v>
       </c>
       <c r="E318" s="21" t="s">
-        <v>1160</v>
+        <v>1154</v>
       </c>
       <c r="F318" s="22" t="s">
         <v>1148</v>
@@ -16568,13 +16843,13 @@
         <v>155</v>
       </c>
       <c r="C319" s="21" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="D319" s="22" t="s">
-        <v>1162</v>
+        <v>1156</v>
       </c>
       <c r="E319" s="21" t="s">
-        <v>1163</v>
+        <v>1157</v>
       </c>
       <c r="F319" s="22" t="s">
         <v>1148</v>
@@ -16593,13 +16868,13 @@
         <v>155</v>
       </c>
       <c r="C320" s="21" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="D320" s="22" t="s">
-        <v>1165</v>
+        <v>1159</v>
       </c>
       <c r="E320" s="21" t="s">
-        <v>1166</v>
+        <v>1160</v>
       </c>
       <c r="F320" s="22" t="s">
         <v>1148</v>
@@ -16618,13 +16893,13 @@
         <v>155</v>
       </c>
       <c r="C321" s="21" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="D321" s="22" t="s">
-        <v>1168</v>
+        <v>1162</v>
       </c>
       <c r="E321" s="21" t="s">
-        <v>1169</v>
+        <v>1163</v>
       </c>
       <c r="F321" s="22" t="s">
         <v>1148</v>
@@ -16643,13 +16918,13 @@
         <v>155</v>
       </c>
       <c r="C322" s="21" t="s">
-        <v>258</v>
+        <v>206</v>
       </c>
       <c r="D322" s="22" t="s">
-        <v>1171</v>
+        <v>1165</v>
       </c>
       <c r="E322" s="21" t="s">
-        <v>1172</v>
+        <v>1166</v>
       </c>
       <c r="F322" s="22" t="s">
         <v>1148</v>
@@ -16668,13 +16943,13 @@
         <v>155</v>
       </c>
       <c r="C323" s="21" t="s">
-        <v>262</v>
+        <v>210</v>
       </c>
       <c r="D323" s="22" t="s">
-        <v>1174</v>
+        <v>1168</v>
       </c>
       <c r="E323" s="21" t="s">
-        <v>1175</v>
+        <v>1169</v>
       </c>
       <c r="F323" s="22" t="s">
         <v>1148</v>
@@ -16693,13 +16968,13 @@
         <v>155</v>
       </c>
       <c r="C324" s="21" t="s">
-        <v>296</v>
+        <v>258</v>
       </c>
       <c r="D324" s="22" t="s">
-        <v>1177</v>
+        <v>1171</v>
       </c>
       <c r="E324" s="21" t="s">
-        <v>1178</v>
+        <v>1172</v>
       </c>
       <c r="F324" s="22" t="s">
         <v>1148</v>
@@ -16718,13 +16993,13 @@
         <v>155</v>
       </c>
       <c r="C325" s="21" t="s">
-        <v>300</v>
+        <v>262</v>
       </c>
       <c r="D325" s="22" t="s">
-        <v>1180</v>
+        <v>1174</v>
       </c>
       <c r="E325" s="21" t="s">
-        <v>1181</v>
+        <v>1175</v>
       </c>
       <c r="F325" s="22" t="s">
         <v>1148</v>
@@ -16743,13 +17018,13 @@
         <v>155</v>
       </c>
       <c r="C326" s="21" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="D326" s="22" t="s">
-        <v>1183</v>
+        <v>1177</v>
       </c>
       <c r="E326" s="21" t="s">
-        <v>1184</v>
+        <v>1178</v>
       </c>
       <c r="F326" s="22" t="s">
         <v>1148</v>
@@ -16768,13 +17043,13 @@
         <v>155</v>
       </c>
       <c r="C327" s="21" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
       <c r="D327" s="22" t="s">
-        <v>1186</v>
+        <v>1180</v>
       </c>
       <c r="E327" s="21" t="s">
-        <v>1187</v>
+        <v>1181</v>
       </c>
       <c r="F327" s="22" t="s">
         <v>1148</v>
@@ -16793,13 +17068,13 @@
         <v>155</v>
       </c>
       <c r="C328" s="21" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
       <c r="D328" s="22" t="s">
-        <v>1189</v>
+        <v>1183</v>
       </c>
       <c r="E328" s="21" t="s">
-        <v>1190</v>
+        <v>1184</v>
       </c>
       <c r="F328" s="22" t="s">
         <v>1148</v>
@@ -16818,13 +17093,13 @@
         <v>155</v>
       </c>
       <c r="C329" s="21" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="D329" s="22" t="s">
-        <v>1192</v>
+        <v>1186</v>
       </c>
       <c r="E329" s="21" t="s">
-        <v>1193</v>
+        <v>1187</v>
       </c>
       <c r="F329" s="22" t="s">
         <v>1148</v>
@@ -16843,13 +17118,13 @@
         <v>155</v>
       </c>
       <c r="C330" s="21" t="s">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="D330" s="22" t="s">
-        <v>1195</v>
+        <v>1189</v>
       </c>
       <c r="E330" s="21" t="s">
-        <v>1196</v>
+        <v>1190</v>
       </c>
       <c r="F330" s="22" t="s">
         <v>1148</v>
@@ -16868,13 +17143,13 @@
         <v>155</v>
       </c>
       <c r="C331" s="21" t="s">
-        <v>324</v>
+        <v>316</v>
       </c>
       <c r="D331" s="22" t="s">
-        <v>1198</v>
+        <v>1192</v>
       </c>
       <c r="E331" s="21" t="s">
-        <v>188</v>
+        <v>1193</v>
       </c>
       <c r="F331" s="22" t="s">
         <v>1148</v>
@@ -16893,13 +17168,13 @@
         <v>155</v>
       </c>
       <c r="C332" s="21" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="D332" s="22" t="s">
-        <v>1200</v>
+        <v>1195</v>
       </c>
       <c r="E332" s="21" t="s">
-        <v>1201</v>
+        <v>1196</v>
       </c>
       <c r="F332" s="22" t="s">
         <v>1148</v>
@@ -16918,13 +17193,13 @@
         <v>155</v>
       </c>
       <c r="C333" s="21" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="D333" s="22" t="s">
-        <v>1203</v>
+        <v>1198</v>
       </c>
       <c r="E333" s="21" t="s">
-        <v>1204</v>
+        <v>188</v>
       </c>
       <c r="F333" s="22" t="s">
         <v>1148</v>
@@ -16943,13 +17218,13 @@
         <v>155</v>
       </c>
       <c r="C334" s="21" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="D334" s="22" t="s">
-        <v>1206</v>
+        <v>1200</v>
       </c>
       <c r="E334" s="21" t="s">
-        <v>1207</v>
+        <v>1201</v>
       </c>
       <c r="F334" s="22" t="s">
         <v>1148</v>
@@ -16965,19 +17240,19 @@
         <v>1208</v>
       </c>
       <c r="B335" s="21" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C335" s="21" t="s">
-        <v>174</v>
+        <v>332</v>
       </c>
       <c r="D335" s="22" t="s">
-        <v>1209</v>
+        <v>1203</v>
       </c>
       <c r="E335" s="21" t="s">
-        <v>1163</v>
+        <v>1204</v>
       </c>
       <c r="F335" s="22" t="s">
-        <v>1210</v>
+        <v>1148</v>
       </c>
       <c r="G335" s="20"/>
       <c r="H335" s="23"/>
@@ -16990,19 +17265,19 @@
         <v>1211</v>
       </c>
       <c r="B336" s="21" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C336" s="21" t="s">
-        <v>179</v>
+        <v>336</v>
       </c>
       <c r="D336" s="22" t="s">
-        <v>1212</v>
+        <v>1206</v>
       </c>
       <c r="E336" s="21" t="s">
-        <v>1213</v>
+        <v>1207</v>
       </c>
       <c r="F336" s="22" t="s">
-        <v>1210</v>
+        <v>1148</v>
       </c>
       <c r="G336" s="20"/>
       <c r="H336" s="23"/>
@@ -17018,13 +17293,13 @@
         <v>156</v>
       </c>
       <c r="C337" s="21" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D337" s="22" t="s">
-        <v>1215</v>
+        <v>1209</v>
       </c>
       <c r="E337" s="21" t="s">
-        <v>1216</v>
+        <v>1163</v>
       </c>
       <c r="F337" s="22" t="s">
         <v>1210</v>
@@ -17043,13 +17318,13 @@
         <v>156</v>
       </c>
       <c r="C338" s="21" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="D338" s="22" t="s">
-        <v>1218</v>
+        <v>1212</v>
       </c>
       <c r="E338" s="21" t="s">
-        <v>1219</v>
+        <v>1213</v>
       </c>
       <c r="F338" s="22" t="s">
         <v>1210</v>
@@ -17068,13 +17343,13 @@
         <v>156</v>
       </c>
       <c r="C339" s="21" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="D339" s="22" t="s">
-        <v>1221</v>
+        <v>1215</v>
       </c>
       <c r="E339" s="21" t="s">
-        <v>1222</v>
+        <v>1216</v>
       </c>
       <c r="F339" s="22" t="s">
         <v>1210</v>
@@ -17093,13 +17368,13 @@
         <v>156</v>
       </c>
       <c r="C340" s="21" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="D340" s="22" t="s">
-        <v>1224</v>
+        <v>1218</v>
       </c>
       <c r="E340" s="21" t="s">
-        <v>1225</v>
+        <v>1219</v>
       </c>
       <c r="F340" s="22" t="s">
         <v>1210</v>
@@ -17118,13 +17393,13 @@
         <v>156</v>
       </c>
       <c r="C341" s="21" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="D341" s="22" t="s">
-        <v>1227</v>
+        <v>1221</v>
       </c>
       <c r="E341" s="21" t="s">
-        <v>1228</v>
+        <v>1222</v>
       </c>
       <c r="F341" s="22" t="s">
         <v>1210</v>
@@ -17143,13 +17418,13 @@
         <v>156</v>
       </c>
       <c r="C342" s="21" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="D342" s="22" t="s">
-        <v>1230</v>
+        <v>1224</v>
       </c>
       <c r="E342" s="21" t="s">
-        <v>1231</v>
+        <v>1225</v>
       </c>
       <c r="F342" s="22" t="s">
         <v>1210</v>
@@ -17168,13 +17443,13 @@
         <v>156</v>
       </c>
       <c r="C343" s="21" t="s">
-        <v>258</v>
+        <v>206</v>
       </c>
       <c r="D343" s="22" t="s">
-        <v>1233</v>
+        <v>1227</v>
       </c>
       <c r="E343" s="21" t="s">
-        <v>1234</v>
+        <v>1228</v>
       </c>
       <c r="F343" s="22" t="s">
         <v>1210</v>
@@ -17193,13 +17468,13 @@
         <v>156</v>
       </c>
       <c r="C344" s="21" t="s">
-        <v>262</v>
+        <v>210</v>
       </c>
       <c r="D344" s="22" t="s">
-        <v>1236</v>
+        <v>1230</v>
       </c>
       <c r="E344" s="21" t="s">
-        <v>1237</v>
+        <v>1231</v>
       </c>
       <c r="F344" s="22" t="s">
         <v>1210</v>
@@ -17218,13 +17493,13 @@
         <v>156</v>
       </c>
       <c r="C345" s="21" t="s">
-        <v>296</v>
+        <v>258</v>
       </c>
       <c r="D345" s="22" t="s">
-        <v>1239</v>
+        <v>1233</v>
       </c>
       <c r="E345" s="21" t="s">
-        <v>1240</v>
+        <v>1234</v>
       </c>
       <c r="F345" s="22" t="s">
         <v>1210</v>
@@ -17243,13 +17518,13 @@
         <v>156</v>
       </c>
       <c r="C346" s="21" t="s">
-        <v>300</v>
+        <v>262</v>
       </c>
       <c r="D346" s="22" t="s">
-        <v>1242</v>
+        <v>1236</v>
       </c>
       <c r="E346" s="21" t="s">
-        <v>1243</v>
+        <v>1237</v>
       </c>
       <c r="F346" s="22" t="s">
         <v>1210</v>
@@ -17265,19 +17540,19 @@
         <v>1244</v>
       </c>
       <c r="B347" s="21" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C347" s="21" t="s">
-        <v>174</v>
+        <v>296</v>
       </c>
       <c r="D347" s="22" t="s">
-        <v>1245</v>
+        <v>1239</v>
       </c>
       <c r="E347" s="21" t="s">
-        <v>1246</v>
+        <v>1240</v>
       </c>
       <c r="F347" s="22" t="s">
-        <v>877</v>
+        <v>1210</v>
       </c>
       <c r="G347" s="20"/>
       <c r="H347" s="23"/>
@@ -17290,19 +17565,19 @@
         <v>1247</v>
       </c>
       <c r="B348" s="21" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C348" s="21" t="s">
-        <v>179</v>
+        <v>300</v>
       </c>
       <c r="D348" s="22" t="s">
-        <v>1248</v>
+        <v>1242</v>
       </c>
       <c r="E348" s="21" t="s">
-        <v>1249</v>
+        <v>1243</v>
       </c>
       <c r="F348" s="22" t="s">
-        <v>877</v>
+        <v>1210</v>
       </c>
       <c r="G348" s="20"/>
       <c r="H348" s="23"/>
@@ -17318,13 +17593,13 @@
         <v>158</v>
       </c>
       <c r="C349" s="21" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D349" s="22" t="s">
-        <v>1251</v>
+        <v>1245</v>
       </c>
       <c r="E349" s="21" t="s">
-        <v>1252</v>
+        <v>1246</v>
       </c>
       <c r="F349" s="22" t="s">
         <v>877</v>
@@ -17343,13 +17618,13 @@
         <v>158</v>
       </c>
       <c r="C350" s="21" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="D350" s="22" t="s">
-        <v>1254</v>
+        <v>1248</v>
       </c>
       <c r="E350" s="21" t="s">
-        <v>1255</v>
+        <v>1249</v>
       </c>
       <c r="F350" s="22" t="s">
         <v>877</v>
@@ -17368,13 +17643,13 @@
         <v>158</v>
       </c>
       <c r="C351" s="21" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="D351" s="22" t="s">
-        <v>1257</v>
+        <v>1251</v>
       </c>
       <c r="E351" s="21" t="s">
-        <v>1258</v>
+        <v>1252</v>
       </c>
       <c r="F351" s="22" t="s">
         <v>877</v>
@@ -17386,12 +17661,24 @@
       <c r="K351" s="23"/>
     </row>
     <row r="352" spans="1:11">
-      <c r="A352" s="21"/>
-      <c r="B352" s="21"/>
-      <c r="C352" s="21"/>
-      <c r="D352" s="22"/>
-      <c r="E352" s="21"/>
-      <c r="F352" s="22"/>
+      <c r="A352" s="21" t="s">
+        <v>1287</v>
+      </c>
+      <c r="B352" s="21" t="s">
+        <v>158</v>
+      </c>
+      <c r="C352" s="21" t="s">
+        <v>194</v>
+      </c>
+      <c r="D352" s="22" t="s">
+        <v>1254</v>
+      </c>
+      <c r="E352" s="21" t="s">
+        <v>1255</v>
+      </c>
+      <c r="F352" s="22" t="s">
+        <v>877</v>
+      </c>
       <c r="G352" s="20"/>
       <c r="H352" s="23"/>
       <c r="I352" s="23"/>
@@ -17399,12 +17686,24 @@
       <c r="K352" s="23"/>
     </row>
     <row r="353" spans="1:11">
-      <c r="A353" s="21"/>
-      <c r="B353" s="21"/>
-      <c r="C353" s="21"/>
-      <c r="D353" s="22"/>
-      <c r="E353" s="21"/>
-      <c r="F353" s="22"/>
+      <c r="A353" s="21" t="s">
+        <v>1288</v>
+      </c>
+      <c r="B353" s="21" t="s">
+        <v>158</v>
+      </c>
+      <c r="C353" s="21" t="s">
+        <v>198</v>
+      </c>
+      <c r="D353" s="22" t="s">
+        <v>1257</v>
+      </c>
+      <c r="E353" s="21" t="s">
+        <v>1258</v>
+      </c>
+      <c r="F353" s="22" t="s">
+        <v>877</v>
+      </c>
       <c r="G353" s="20"/>
       <c r="H353" s="23"/>
       <c r="I353" s="23"/>
@@ -18107,7 +18406,7 @@
       <c r="D407" s="22"/>
       <c r="E407" s="21"/>
       <c r="F407" s="22"/>
-      <c r="G407" s="18"/>
+      <c r="G407" s="20"/>
       <c r="H407" s="23"/>
       <c r="I407" s="23"/>
       <c r="J407" s="23"/>
@@ -18120,7 +18419,7 @@
       <c r="D408" s="22"/>
       <c r="E408" s="21"/>
       <c r="F408" s="22"/>
-      <c r="G408" s="18"/>
+      <c r="G408" s="20"/>
       <c r="H408" s="23"/>
       <c r="I408" s="23"/>
       <c r="J408" s="23"/>
@@ -38822,26 +39121,52 @@
       <c r="J2000" s="23"/>
       <c r="K2000" s="23"/>
     </row>
+    <row r="2001" spans="1:11">
+      <c r="A2001" s="21"/>
+      <c r="B2001" s="21"/>
+      <c r="C2001" s="21"/>
+      <c r="D2001" s="22"/>
+      <c r="E2001" s="21"/>
+      <c r="F2001" s="22"/>
+      <c r="G2001" s="18"/>
+      <c r="H2001" s="23"/>
+      <c r="I2001" s="23"/>
+      <c r="J2001" s="23"/>
+      <c r="K2001" s="33"/>
+    </row>
+    <row r="2002" spans="1:11">
+      <c r="A2002" s="21"/>
+      <c r="B2002" s="21"/>
+      <c r="C2002" s="21"/>
+      <c r="D2002" s="22"/>
+      <c r="E2002" s="21"/>
+      <c r="F2002" s="22"/>
+      <c r="G2002" s="18"/>
+      <c r="H2002" s="23"/>
+      <c r="I2002" s="23"/>
+      <c r="J2002" s="23"/>
+      <c r="K2002" s="33"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A1:K1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A1996:A2000">
-    <cfRule type="duplicateValues" dxfId="1" priority="5"/>
+  <conditionalFormatting sqref="A1998:A2002">
+    <cfRule type="duplicateValues" dxfId="11" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A4:A1995">
-    <cfRule type="duplicateValues" dxfId="0" priority="40"/>
+  <conditionalFormatting sqref="A4:A1997">
+    <cfRule type="duplicateValues" dxfId="10" priority="2"/>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H214:H227" xr:uid="{904F9C07-3432-407C-9B6A-2B1BA8B10BD0}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4:H2002" xr:uid="{74B10176-32C1-4DCE-B9A9-308EB3B34100}">
       <formula1>"Daily 60 Days, Daily 120 Days, Weekly 12W, Weekly 24W, Monthly 3M, Monthly 6M, 60-Day Asset, 120-Day Asset, Weekly 12W Asset, Weekly 24W Asset, Monthly 3M Asset, Monthly 6M Asset"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -38860,27 +39185,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="33.9" customHeight="1">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>1259</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
       <c r="H1" s="29"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="38" t="s">
         <v>1260</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
       <c r="H2" s="26"/>
     </row>
     <row r="3" spans="1:8" ht="38.1" customHeight="1">

</xml_diff>

<commit_message>
feat(financial-integrity): implement 3-tier savings aggregation, excess payments isolation, misc savings dual-officer audit trace, and updated onboarding ingestion
</commit_message>
<xml_diff>
--- a/icare-group-member-onboarding-template.xlsx
+++ b/icare-group-member-onboarding-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\Master_ AY Projects\trustmicro-credit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0229BF08-1474-4D13-8242-FD8CCC815105}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D51AD34-718B-40DD-B5C8-D54B3B8CF329}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2503" uniqueCount="1289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2493" uniqueCount="1287">
   <si>
     <t>ICARE Group and Member Onboarding Template</t>
   </si>
@@ -3859,24 +3859,12 @@
     <t>Koleosho Sherifat</t>
   </si>
   <si>
-    <t>11750</t>
-  </si>
-  <si>
-    <t>7000</t>
-  </si>
-  <si>
-    <t>17000</t>
-  </si>
-  <si>
     <t>Weekly 12W</t>
   </si>
   <si>
     <t>Weekly 24W</t>
   </si>
   <si>
-    <t>Weekly 12W Asset</t>
-  </si>
-  <si>
     <t>Osho Bunmi</t>
   </si>
   <si>
@@ -3893,6 +3881,12 @@
   </si>
   <si>
     <t>MEM-350</t>
+  </si>
+  <si>
+    <t>36925</t>
+  </si>
+  <si>
+    <t>25125</t>
   </si>
 </sst>
 </file>
@@ -4188,6 +4182,9 @@
     <xf numFmtId="49" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="3" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -4218,14 +4215,44 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="17">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top"/>
+      <border outline="0">
+        <left style="thin">
+          <color rgb="FFD9E2F3"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FFD9E2F3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -4541,59 +4568,6 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos"/>
-      </font>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="top"/>
-      <border outline="0">
-        <left style="thin">
-          <color rgb="FFD9E2F3"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color rgb="FFD9E2F3"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9E2F3"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <alignment horizontal="left" vertical="top"/>
     </dxf>
     <dxf>
@@ -4702,31 +4676,31 @@
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Group Reference*"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Branch Name*"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Group Name*"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Group Leader Name*" dataDxfId="17"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Group Leader Name*" dataDxfId="15"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Meeting Day*"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Formation Date*"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Credit Officer Name*"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Credit Officer Phone"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Group Savings" dataDxfId="16"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Group Savings" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="MemberOnboardingTable" displayName="MemberOnboardingTable" ref="A3:K2002" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="MemberOnboardingTable" displayName="MemberOnboardingTable" ref="A3:K2002" dataDxfId="11">
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Member Reference*" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Group Reference*" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Member Number" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Full Name*" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Phone Number*" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Home Address*" dataDxfId="4"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Savings Balance*" dataDxfId="3"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0100-000015000000}" name="Loan Type (Product)*" dataDxfId="2"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0100-000016000000}" name="Principal Loan*" dataDxfId="1"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0100-000014000000}" name="Active Credit (Disbursed)*" dataDxfId="0"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0100-000013000000}" name="Current Credit Balance*" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Member Reference*" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Group Reference*" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Member Number" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Full Name*" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Phone Number*" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Home Address*" dataDxfId="5"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Savings Balance*" dataDxfId="4"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0100-000015000000}" name="Loan Type (Product)*" dataDxfId="3"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0100-000016000000}" name="Principal Loan*" dataDxfId="2"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0100-000014000000}" name="Active Credit (Disbursed)*" dataDxfId="1"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0100-000013000000}" name="Current Credit Balance*" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4891,28 +4865,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="33.9" customHeight="1">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="2"/>
@@ -4932,13 +4906,13 @@
         <v>3</v>
       </c>
       <c r="C4" s="2"/>
-      <c r="D4" s="40" t="s">
+      <c r="D4" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
-      <c r="H4" s="39"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="40"/>
     </row>
     <row r="5" spans="1:8" ht="27.9" customHeight="1">
       <c r="A5" s="3" t="s">
@@ -4946,13 +4920,13 @@
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="41" t="s">
+      <c r="D5" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="38"/>
     </row>
     <row r="6" spans="1:8" ht="27.9" customHeight="1">
       <c r="A6" s="3" t="s">
@@ -4960,13 +4934,13 @@
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="36"/>
-      <c r="F6" s="36"/>
-      <c r="G6" s="36"/>
-      <c r="H6" s="37"/>
+      <c r="E6" s="37"/>
+      <c r="F6" s="37"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="38"/>
     </row>
     <row r="7" spans="1:8" ht="27.9" customHeight="1">
       <c r="A7" s="3" t="s">
@@ -4974,13 +4948,13 @@
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="41" t="s">
+      <c r="D7" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="37"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:8" ht="27.9" customHeight="1">
       <c r="A8" s="3" t="s">
@@ -4988,13 +4962,13 @@
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="2"/>
-      <c r="D8" s="41" t="s">
+      <c r="D8" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="36"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="36"/>
-      <c r="H8" s="37"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="37"/>
+      <c r="H8" s="38"/>
     </row>
     <row r="9" spans="1:8" ht="27.9" customHeight="1">
       <c r="A9" s="3" t="s">
@@ -5002,25 +4976,25 @@
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="2"/>
-      <c r="D9" s="41" t="s">
+      <c r="D9" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="38"/>
     </row>
     <row r="10" spans="1:8" ht="27.9" customHeight="1">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
-      <c r="D10" s="41" t="s">
+      <c r="D10" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="36"/>
-      <c r="F10" s="36"/>
-      <c r="G10" s="36"/>
-      <c r="H10" s="37"/>
+      <c r="E10" s="37"/>
+      <c r="F10" s="37"/>
+      <c r="G10" s="37"/>
+      <c r="H10" s="38"/>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="2"/>
@@ -5033,142 +5007,142 @@
       <c r="H11" s="2"/>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="45" t="s">
+      <c r="A12" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="39"/>
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39"/>
-      <c r="G12" s="39"/>
-      <c r="H12" s="39"/>
+      <c r="B12" s="40"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="40"/>
+      <c r="F12" s="40"/>
+      <c r="G12" s="40"/>
+      <c r="H12" s="40"/>
     </row>
     <row r="13" spans="1:8" ht="38.1" customHeight="1">
       <c r="A13" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="43" t="s">
+      <c r="B13" s="44" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="36"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="36"/>
-      <c r="G13" s="36"/>
-      <c r="H13" s="37"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="37"/>
+      <c r="E13" s="37"/>
+      <c r="F13" s="37"/>
+      <c r="G13" s="37"/>
+      <c r="H13" s="38"/>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="42" t="s">
+      <c r="B14" s="43" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="36"/>
-      <c r="F14" s="36"/>
-      <c r="G14" s="36"/>
-      <c r="H14" s="37"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="37"/>
+      <c r="E14" s="37"/>
+      <c r="F14" s="37"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="38"/>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="42" t="s">
+      <c r="B15" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="36"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="36"/>
-      <c r="G15" s="36"/>
-      <c r="H15" s="37"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="37"/>
+      <c r="F15" s="37"/>
+      <c r="G15" s="37"/>
+      <c r="H15" s="38"/>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="42" t="s">
+      <c r="B16" s="43" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="36"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="36"/>
-      <c r="F16" s="36"/>
-      <c r="G16" s="36"/>
-      <c r="H16" s="37"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="37"/>
+      <c r="E16" s="37"/>
+      <c r="F16" s="37"/>
+      <c r="G16" s="37"/>
+      <c r="H16" s="38"/>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="42" t="s">
+      <c r="B17" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="36"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="36"/>
-      <c r="F17" s="36"/>
-      <c r="G17" s="36"/>
-      <c r="H17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="37"/>
+      <c r="G17" s="37"/>
+      <c r="H17" s="38"/>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="42" t="s">
+      <c r="B18" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="36"/>
-      <c r="F18" s="36"/>
-      <c r="G18" s="36"/>
-      <c r="H18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="38"/>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="42" t="s">
+      <c r="B19" s="43" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="36"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="36"/>
-      <c r="F19" s="36"/>
-      <c r="G19" s="36"/>
-      <c r="H19" s="37"/>
+      <c r="C19" s="37"/>
+      <c r="D19" s="37"/>
+      <c r="E19" s="37"/>
+      <c r="F19" s="37"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="38"/>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="42" t="s">
+      <c r="B20" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="36"/>
-      <c r="D20" s="36"/>
-      <c r="E20" s="36"/>
-      <c r="F20" s="36"/>
-      <c r="G20" s="36"/>
-      <c r="H20" s="37"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="37"/>
+      <c r="F20" s="37"/>
+      <c r="G20" s="37"/>
+      <c r="H20" s="38"/>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="35" t="s">
+      <c r="B21" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="C21" s="36"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="36"/>
-      <c r="F21" s="36"/>
-      <c r="G21" s="36"/>
-      <c r="H21" s="37"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="37"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="38"/>
     </row>
   </sheetData>
   <autoFilter ref="A12:H21" xr:uid="{00000000-0009-0000-0000-000000000000}">
@@ -5222,30 +5196,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="33.9" customHeight="1">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
+      <c r="I2" s="40"/>
     </row>
     <row r="3" spans="1:9" ht="38.1" customHeight="1">
       <c r="A3" s="28" t="s">
@@ -5901,9 +5875,7 @@
       <c r="H28" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="I28" s="14" t="s">
-        <v>1277</v>
-      </c>
+      <c r="I28" s="14"/>
     </row>
     <row r="29" spans="1:9">
       <c r="A29" s="6" t="s">
@@ -5930,9 +5902,7 @@
       <c r="H29" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="I29" s="14" t="s">
-        <v>1278</v>
-      </c>
+      <c r="I29" s="14"/>
     </row>
     <row r="30" spans="1:9">
       <c r="A30" s="6" t="s">
@@ -5959,9 +5929,7 @@
       <c r="H30" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="I30" s="14" t="s">
-        <v>1279</v>
-      </c>
+      <c r="I30" s="14"/>
     </row>
     <row r="31" spans="1:9">
       <c r="A31" s="6" t="s">
@@ -5988,7 +5956,9 @@
       <c r="H31" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="I31" s="34"/>
+      <c r="I31" s="34" t="s">
+        <v>1285</v>
+      </c>
     </row>
     <row r="32" spans="1:9">
       <c r="A32" s="6" t="s">
@@ -6015,7 +5985,9 @@
       <c r="H32" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="I32" s="34"/>
+      <c r="I32" s="34" t="s">
+        <v>1286</v>
+      </c>
     </row>
     <row r="33" spans="1:9">
       <c r="A33" s="6" t="s">
@@ -8734,7 +8706,7 @@
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <conditionalFormatting sqref="A4:A253">
-    <cfRule type="duplicateValues" dxfId="18" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="21"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -8758,34 +8730,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="33.9" customHeight="1">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>161</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="49"/>
+      <c r="H1" s="49"/>
+      <c r="I1" s="49"/>
+      <c r="J1" s="49"/>
+      <c r="K1" s="49"/>
     </row>
     <row r="2" spans="1:11" ht="30" customHeight="1">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="47" t="s">
         <v>162</v>
       </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
+      <c r="K2" s="48"/>
     </row>
     <row r="3" spans="1:11" ht="38.1" customHeight="1">
       <c r="A3" s="28" t="s">
@@ -13540,18 +13512,10 @@
       <c r="F193" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="G193" s="20">
-        <v>24550</v>
-      </c>
-      <c r="H193" s="23" t="s">
-        <v>1280</v>
-      </c>
-      <c r="I193" s="23">
-        <v>198000</v>
-      </c>
-      <c r="J193" s="23">
-        <v>82500</v>
-      </c>
+      <c r="G193" s="20"/>
+      <c r="H193" s="23"/>
+      <c r="I193" s="23"/>
+      <c r="J193" s="23"/>
       <c r="K193" s="23"/>
     </row>
     <row r="194" spans="1:11">
@@ -13573,18 +13537,10 @@
       <c r="F194" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="G194" s="20">
-        <v>22200</v>
-      </c>
-      <c r="H194" s="23" t="s">
-        <v>1280</v>
-      </c>
-      <c r="I194" s="23">
-        <v>48000</v>
-      </c>
-      <c r="J194" s="23">
-        <v>4000</v>
-      </c>
+      <c r="G194" s="20"/>
+      <c r="H194" s="23"/>
+      <c r="I194" s="23"/>
+      <c r="J194" s="23"/>
       <c r="K194" s="23"/>
     </row>
     <row r="195" spans="1:11">
@@ -13606,18 +13562,10 @@
       <c r="F195" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="G195" s="20">
-        <v>15000</v>
-      </c>
-      <c r="H195" s="23" t="s">
-        <v>1280</v>
-      </c>
-      <c r="I195" s="23">
-        <v>288000</v>
-      </c>
-      <c r="J195" s="23">
-        <v>288000</v>
-      </c>
+      <c r="G195" s="20"/>
+      <c r="H195" s="23"/>
+      <c r="I195" s="23"/>
+      <c r="J195" s="23"/>
       <c r="K195" s="23"/>
     </row>
     <row r="196" spans="1:11">
@@ -13639,18 +13587,10 @@
       <c r="F196" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="G196" s="20">
-        <v>13000</v>
-      </c>
-      <c r="H196" s="23" t="s">
-        <v>1280</v>
-      </c>
-      <c r="I196" s="23">
-        <v>60000</v>
-      </c>
-      <c r="J196" s="23">
-        <v>10000</v>
-      </c>
+      <c r="G196" s="20"/>
+      <c r="H196" s="23"/>
+      <c r="I196" s="23"/>
+      <c r="J196" s="23"/>
       <c r="K196" s="23"/>
     </row>
     <row r="197" spans="1:11">
@@ -13670,18 +13610,10 @@
       <c r="F197" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="G197" s="20">
-        <v>9500</v>
-      </c>
-      <c r="H197" s="23" t="s">
-        <v>1280</v>
-      </c>
-      <c r="I197" s="23">
-        <v>150000</v>
-      </c>
-      <c r="J197" s="23">
-        <v>100000</v>
-      </c>
+      <c r="G197" s="20"/>
+      <c r="H197" s="23"/>
+      <c r="I197" s="23"/>
+      <c r="J197" s="23"/>
       <c r="K197" s="23"/>
     </row>
     <row r="198" spans="1:11">
@@ -13704,9 +13636,7 @@
         <v>776</v>
       </c>
       <c r="G198" s="20"/>
-      <c r="H198" s="23" t="s">
-        <v>1281</v>
-      </c>
+      <c r="H198" s="23"/>
       <c r="I198" s="23"/>
       <c r="J198" s="23"/>
       <c r="K198" s="23"/>
@@ -13730,18 +13660,10 @@
       <c r="F199" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="G199" s="20">
-        <v>23600</v>
-      </c>
-      <c r="H199" s="23" t="s">
-        <v>1281</v>
-      </c>
-      <c r="I199" s="23">
-        <v>198000</v>
-      </c>
-      <c r="J199" s="23">
-        <v>41250</v>
-      </c>
+      <c r="G199" s="20"/>
+      <c r="H199" s="23"/>
+      <c r="I199" s="23"/>
+      <c r="J199" s="23"/>
       <c r="K199" s="23"/>
     </row>
     <row r="200" spans="1:11">
@@ -13763,12 +13685,8 @@
       <c r="F200" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="G200" s="20">
-        <v>63400</v>
-      </c>
-      <c r="H200" s="23" t="s">
-        <v>1281</v>
-      </c>
+      <c r="G200" s="20"/>
+      <c r="H200" s="23"/>
       <c r="I200" s="23"/>
       <c r="J200" s="23"/>
       <c r="K200" s="23"/>
@@ -13792,18 +13710,10 @@
       <c r="F201" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="G201" s="20">
-        <v>18725</v>
-      </c>
-      <c r="H201" s="23" t="s">
-        <v>1281</v>
-      </c>
-      <c r="I201" s="23">
-        <v>99000</v>
-      </c>
-      <c r="J201" s="23">
-        <v>28875</v>
-      </c>
+      <c r="G201" s="20"/>
+      <c r="H201" s="23"/>
+      <c r="I201" s="23"/>
+      <c r="J201" s="23"/>
       <c r="K201" s="23"/>
     </row>
     <row r="202" spans="1:11">
@@ -13825,12 +13735,8 @@
       <c r="F202" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="G202" s="20">
-        <v>89000</v>
-      </c>
-      <c r="H202" s="23" t="s">
-        <v>1281</v>
-      </c>
+      <c r="G202" s="20"/>
+      <c r="H202" s="23"/>
       <c r="I202" s="23"/>
       <c r="J202" s="23"/>
       <c r="K202" s="23"/>
@@ -13854,18 +13760,10 @@
       <c r="F203" s="22" t="s">
         <v>806</v>
       </c>
-      <c r="G203" s="20">
-        <v>5950</v>
-      </c>
-      <c r="H203" s="23" t="s">
-        <v>1280</v>
-      </c>
-      <c r="I203" s="23">
-        <v>99000</v>
-      </c>
-      <c r="J203" s="23">
-        <v>24750</v>
-      </c>
+      <c r="G203" s="20"/>
+      <c r="H203" s="23"/>
+      <c r="I203" s="23"/>
+      <c r="J203" s="23"/>
       <c r="K203" s="23"/>
     </row>
     <row r="204" spans="1:11">
@@ -13887,18 +13785,10 @@
       <c r="F204" s="22" t="s">
         <v>806</v>
       </c>
-      <c r="G204" s="20">
-        <v>4750</v>
-      </c>
-      <c r="H204" s="23" t="s">
-        <v>1280</v>
-      </c>
-      <c r="I204" s="23">
-        <v>99000</v>
-      </c>
-      <c r="J204" s="23">
-        <v>33000</v>
-      </c>
+      <c r="G204" s="20"/>
+      <c r="H204" s="23"/>
+      <c r="I204" s="23"/>
+      <c r="J204" s="23"/>
       <c r="K204" s="23"/>
     </row>
     <row r="205" spans="1:11">
@@ -13921,15 +13811,9 @@
         <v>806</v>
       </c>
       <c r="G205" s="20"/>
-      <c r="H205" s="23" t="s">
-        <v>1282</v>
-      </c>
-      <c r="I205" s="23">
-        <v>279000</v>
-      </c>
-      <c r="J205" s="23">
-        <v>46500</v>
-      </c>
+      <c r="H205" s="23"/>
+      <c r="I205" s="23"/>
+      <c r="J205" s="23"/>
       <c r="K205" s="23"/>
     </row>
     <row r="206" spans="1:11">
@@ -13951,18 +13835,10 @@
       <c r="F206" s="22" t="s">
         <v>806</v>
       </c>
-      <c r="G206" s="20">
-        <v>5000</v>
-      </c>
-      <c r="H206" s="23" t="s">
-        <v>1280</v>
-      </c>
-      <c r="I206" s="23">
-        <v>99000</v>
-      </c>
-      <c r="J206" s="23">
-        <v>24750</v>
-      </c>
+      <c r="G206" s="20"/>
+      <c r="H206" s="23"/>
+      <c r="I206" s="23"/>
+      <c r="J206" s="23"/>
       <c r="K206" s="23"/>
     </row>
     <row r="207" spans="1:11">
@@ -13984,18 +13860,10 @@
       <c r="F207" s="22" t="s">
         <v>806</v>
       </c>
-      <c r="G207" s="20">
-        <v>4750</v>
-      </c>
-      <c r="H207" s="23" t="s">
-        <v>1280</v>
-      </c>
-      <c r="I207" s="23">
-        <v>99000</v>
-      </c>
-      <c r="J207" s="23">
-        <v>33000</v>
-      </c>
+      <c r="G207" s="20"/>
+      <c r="H207" s="23"/>
+      <c r="I207" s="23"/>
+      <c r="J207" s="23"/>
       <c r="K207" s="23"/>
     </row>
     <row r="208" spans="1:11">
@@ -14017,18 +13885,10 @@
       <c r="F208" s="22" t="s">
         <v>806</v>
       </c>
-      <c r="G208" s="20">
-        <v>3000</v>
-      </c>
-      <c r="H208" s="23" t="s">
-        <v>1280</v>
-      </c>
-      <c r="I208" s="23">
-        <v>99000</v>
-      </c>
-      <c r="J208" s="23">
-        <v>57750</v>
-      </c>
+      <c r="G208" s="20"/>
+      <c r="H208" s="23"/>
+      <c r="I208" s="23"/>
+      <c r="J208" s="23"/>
       <c r="K208" s="23"/>
     </row>
     <row r="209" spans="1:11">
@@ -14042,27 +13902,19 @@
         <v>206</v>
       </c>
       <c r="D209" s="22" t="s">
-        <v>1283</v>
+        <v>1279</v>
       </c>
       <c r="E209" s="21" t="s">
-        <v>1284</v>
+        <v>1280</v>
       </c>
       <c r="F209" s="22" t="s">
         <v>806</v>
       </c>
-      <c r="G209" s="49">
-        <v>2750</v>
-      </c>
-      <c r="H209" s="23" t="s">
-        <v>1280</v>
-      </c>
-      <c r="I209" s="23">
-        <v>99000</v>
-      </c>
-      <c r="J209" s="33">
-        <v>66000</v>
-      </c>
-      <c r="K209" s="23"/>
+      <c r="G209" s="35"/>
+      <c r="H209" s="23"/>
+      <c r="I209" s="23"/>
+      <c r="J209" s="23"/>
+      <c r="K209" s="33"/>
     </row>
     <row r="210" spans="1:11">
       <c r="A210" s="21" t="s">
@@ -14075,27 +13927,19 @@
         <v>210</v>
       </c>
       <c r="D210" s="22" t="s">
-        <v>1285</v>
+        <v>1281</v>
       </c>
       <c r="E210" s="21" t="s">
-        <v>1286</v>
+        <v>1282</v>
       </c>
       <c r="F210" s="22" t="s">
         <v>806</v>
       </c>
-      <c r="G210" s="49">
-        <v>2750</v>
-      </c>
-      <c r="H210" s="23" t="s">
-        <v>1280</v>
-      </c>
-      <c r="I210" s="23">
-        <v>99000</v>
-      </c>
-      <c r="J210" s="33">
-        <v>66000</v>
-      </c>
-      <c r="K210" s="23"/>
+      <c r="G210" s="35"/>
+      <c r="H210" s="23"/>
+      <c r="I210" s="23"/>
+      <c r="J210" s="23"/>
+      <c r="K210" s="33"/>
     </row>
     <row r="211" spans="1:11">
       <c r="A211" s="21" t="s">
@@ -14116,18 +13960,10 @@
       <c r="F211" s="22" t="s">
         <v>711</v>
       </c>
-      <c r="G211" s="20">
-        <v>19200</v>
-      </c>
-      <c r="H211" s="23" t="s">
-        <v>1280</v>
-      </c>
-      <c r="I211" s="23">
-        <v>288000</v>
-      </c>
-      <c r="J211" s="23">
-        <v>288000</v>
-      </c>
+      <c r="G211" s="20"/>
+      <c r="H211" s="23"/>
+      <c r="I211" s="23"/>
+      <c r="J211" s="23"/>
       <c r="K211" s="23"/>
     </row>
     <row r="212" spans="1:11">
@@ -14149,18 +13985,10 @@
       <c r="F212" s="22" t="s">
         <v>698</v>
       </c>
-      <c r="G212" s="20">
-        <v>11700</v>
-      </c>
-      <c r="H212" s="23" t="s">
-        <v>1280</v>
-      </c>
-      <c r="I212" s="23">
-        <v>288000</v>
-      </c>
-      <c r="J212" s="23">
-        <v>288000</v>
-      </c>
+      <c r="G212" s="20"/>
+      <c r="H212" s="23"/>
+      <c r="I212" s="23"/>
+      <c r="J212" s="23"/>
       <c r="K212" s="23"/>
     </row>
     <row r="213" spans="1:11">
@@ -14182,18 +14010,10 @@
       <c r="F213" s="22" t="s">
         <v>698</v>
       </c>
-      <c r="G213" s="20">
-        <v>11700</v>
-      </c>
-      <c r="H213" s="23" t="s">
-        <v>1280</v>
-      </c>
-      <c r="I213" s="23">
-        <v>246000</v>
-      </c>
-      <c r="J213" s="23">
-        <v>246000</v>
-      </c>
+      <c r="G213" s="20"/>
+      <c r="H213" s="23"/>
+      <c r="I213" s="23"/>
+      <c r="J213" s="23"/>
       <c r="K213" s="23"/>
     </row>
     <row r="214" spans="1:11">
@@ -14215,18 +14035,10 @@
       <c r="F214" s="22" t="s">
         <v>711</v>
       </c>
-      <c r="G214" s="20">
-        <v>11000</v>
-      </c>
-      <c r="H214" s="23" t="s">
-        <v>1280</v>
-      </c>
-      <c r="I214" s="23">
-        <v>288000</v>
-      </c>
-      <c r="J214" s="23">
-        <v>288000</v>
-      </c>
+      <c r="G214" s="20"/>
+      <c r="H214" s="23"/>
+      <c r="I214" s="23"/>
+      <c r="J214" s="23"/>
       <c r="K214" s="23"/>
     </row>
     <row r="215" spans="1:11">
@@ -14248,18 +14060,10 @@
       <c r="F215" s="22" t="s">
         <v>711</v>
       </c>
-      <c r="G215" s="20">
-        <v>9250</v>
-      </c>
-      <c r="H215" s="23" t="s">
-        <v>1280</v>
-      </c>
-      <c r="I215" s="23">
-        <v>99000</v>
-      </c>
-      <c r="J215" s="23">
-        <v>24750</v>
-      </c>
+      <c r="G215" s="20"/>
+      <c r="H215" s="23"/>
+      <c r="I215" s="23"/>
+      <c r="J215" s="23"/>
       <c r="K215" s="23"/>
     </row>
     <row r="216" spans="1:11">
@@ -14281,8 +14085,12 @@
       <c r="F216" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G216" s="20"/>
-      <c r="H216" s="23"/>
+      <c r="G216" s="20">
+        <v>40100</v>
+      </c>
+      <c r="H216" s="23" t="s">
+        <v>1277</v>
+      </c>
       <c r="I216" s="23"/>
       <c r="J216" s="23"/>
       <c r="K216" s="23"/>
@@ -14306,11 +14114,21 @@
       <c r="F217" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G217" s="20"/>
-      <c r="H217" s="23"/>
-      <c r="I217" s="23"/>
-      <c r="J217" s="23"/>
-      <c r="K217" s="23"/>
+      <c r="G217" s="20">
+        <v>15600</v>
+      </c>
+      <c r="H217" s="23" t="s">
+        <v>1277</v>
+      </c>
+      <c r="I217" s="23">
+        <v>200000</v>
+      </c>
+      <c r="J217" s="23">
+        <v>198000</v>
+      </c>
+      <c r="K217" s="23">
+        <v>132000</v>
+      </c>
     </row>
     <row r="218" spans="1:11">
       <c r="A218" s="21" t="s">
@@ -14331,11 +14149,21 @@
       <c r="F218" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G218" s="20"/>
-      <c r="H218" s="23"/>
-      <c r="I218" s="23"/>
-      <c r="J218" s="23"/>
-      <c r="K218" s="23"/>
+      <c r="G218" s="20">
+        <v>17500</v>
+      </c>
+      <c r="H218" s="23" t="s">
+        <v>1277</v>
+      </c>
+      <c r="I218" s="23">
+        <v>200000</v>
+      </c>
+      <c r="J218" s="23">
+        <v>198000</v>
+      </c>
+      <c r="K218" s="23">
+        <v>132000</v>
+      </c>
     </row>
     <row r="219" spans="1:11">
       <c r="A219" s="21" t="s">
@@ -14356,8 +14184,12 @@
       <c r="F219" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G219" s="20"/>
-      <c r="H219" s="23"/>
+      <c r="G219" s="20">
+        <v>35500</v>
+      </c>
+      <c r="H219" s="23" t="s">
+        <v>1277</v>
+      </c>
       <c r="I219" s="23"/>
       <c r="J219" s="23"/>
       <c r="K219" s="23"/>
@@ -14382,7 +14214,9 @@
         <v>839</v>
       </c>
       <c r="G220" s="20"/>
-      <c r="H220" s="23"/>
+      <c r="H220" s="23" t="s">
+        <v>1277</v>
+      </c>
       <c r="I220" s="23"/>
       <c r="J220" s="23"/>
       <c r="K220" s="23"/>
@@ -14406,11 +14240,21 @@
       <c r="F221" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G221" s="20"/>
-      <c r="H221" s="23"/>
-      <c r="I221" s="23"/>
-      <c r="J221" s="23"/>
-      <c r="K221" s="23"/>
+      <c r="G221" s="20">
+        <v>3000</v>
+      </c>
+      <c r="H221" s="23" t="s">
+        <v>1277</v>
+      </c>
+      <c r="I221" s="23">
+        <v>100000</v>
+      </c>
+      <c r="J221" s="23">
+        <v>99000</v>
+      </c>
+      <c r="K221" s="23">
+        <v>99000</v>
+      </c>
     </row>
     <row r="222" spans="1:11">
       <c r="A222" s="21" t="s">
@@ -14431,11 +14275,21 @@
       <c r="F222" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G222" s="20"/>
-      <c r="H222" s="23"/>
-      <c r="I222" s="23"/>
-      <c r="J222" s="23"/>
-      <c r="K222" s="23"/>
+      <c r="G222" s="20">
+        <v>54250</v>
+      </c>
+      <c r="H222" s="23" t="s">
+        <v>1278</v>
+      </c>
+      <c r="I222" s="23">
+        <v>250000</v>
+      </c>
+      <c r="J222" s="23">
+        <v>246000</v>
+      </c>
+      <c r="K222" s="23">
+        <v>92250</v>
+      </c>
     </row>
     <row r="223" spans="1:11">
       <c r="A223" s="21" t="s">
@@ -14456,11 +14310,21 @@
       <c r="F223" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G223" s="20"/>
-      <c r="H223" s="23"/>
-      <c r="I223" s="23"/>
-      <c r="J223" s="23"/>
-      <c r="K223" s="23"/>
+      <c r="G223" s="20">
+        <v>31150</v>
+      </c>
+      <c r="H223" s="23" t="s">
+        <v>1278</v>
+      </c>
+      <c r="I223" s="23">
+        <v>250000</v>
+      </c>
+      <c r="J223" s="23">
+        <v>246000</v>
+      </c>
+      <c r="K223" s="23">
+        <v>102500</v>
+      </c>
     </row>
     <row r="224" spans="1:11">
       <c r="A224" s="21" t="s">
@@ -14481,11 +14345,21 @@
       <c r="F224" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G224" s="20"/>
-      <c r="H224" s="23"/>
-      <c r="I224" s="23"/>
-      <c r="J224" s="23"/>
-      <c r="K224" s="23"/>
+      <c r="G224" s="20">
+        <v>21250</v>
+      </c>
+      <c r="H224" s="23" t="s">
+        <v>1277</v>
+      </c>
+      <c r="I224" s="23">
+        <v>200000</v>
+      </c>
+      <c r="J224" s="23">
+        <v>198000</v>
+      </c>
+      <c r="K224" s="23">
+        <v>99000</v>
+      </c>
     </row>
     <row r="225" spans="1:11">
       <c r="A225" s="21" t="s">
@@ -14506,11 +14380,21 @@
       <c r="F225" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G225" s="20"/>
-      <c r="H225" s="23"/>
-      <c r="I225" s="23"/>
-      <c r="J225" s="23"/>
-      <c r="K225" s="23"/>
+      <c r="G225" s="20">
+        <v>12500</v>
+      </c>
+      <c r="H225" s="23" t="s">
+        <v>1277</v>
+      </c>
+      <c r="I225" s="23">
+        <v>100000</v>
+      </c>
+      <c r="J225" s="23">
+        <v>99000</v>
+      </c>
+      <c r="K225" s="23">
+        <v>49500</v>
+      </c>
     </row>
     <row r="226" spans="1:11">
       <c r="A226" s="21" t="s">
@@ -14531,11 +14415,21 @@
       <c r="F226" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G226" s="20"/>
-      <c r="H226" s="23"/>
-      <c r="I226" s="23"/>
-      <c r="J226" s="23"/>
-      <c r="K226" s="23"/>
+      <c r="G226" s="20">
+        <v>7700</v>
+      </c>
+      <c r="H226" s="23" t="s">
+        <v>1277</v>
+      </c>
+      <c r="I226" s="23">
+        <v>50000</v>
+      </c>
+      <c r="J226" s="23">
+        <v>48000</v>
+      </c>
+      <c r="K226" s="23">
+        <v>32000</v>
+      </c>
     </row>
     <row r="227" spans="1:11">
       <c r="A227" s="21" t="s">
@@ -14556,11 +14450,21 @@
       <c r="F227" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G227" s="20"/>
-      <c r="H227" s="23"/>
-      <c r="I227" s="23"/>
-      <c r="J227" s="23"/>
-      <c r="K227" s="23"/>
+      <c r="G227" s="20">
+        <v>11650</v>
+      </c>
+      <c r="H227" s="23" t="s">
+        <v>1278</v>
+      </c>
+      <c r="I227" s="23">
+        <v>80000</v>
+      </c>
+      <c r="J227" s="23">
+        <v>78000</v>
+      </c>
+      <c r="K227" s="23">
+        <v>42250</v>
+      </c>
     </row>
     <row r="228" spans="1:11">
       <c r="A228" s="21" t="s">
@@ -14581,11 +14485,21 @@
       <c r="F228" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G228" s="20"/>
-      <c r="H228" s="23"/>
-      <c r="I228" s="23"/>
-      <c r="J228" s="23"/>
-      <c r="K228" s="23"/>
+      <c r="G228" s="20">
+        <v>9300</v>
+      </c>
+      <c r="H228" s="23" t="s">
+        <v>1278</v>
+      </c>
+      <c r="I228" s="23">
+        <v>100000</v>
+      </c>
+      <c r="J228" s="23">
+        <v>99000</v>
+      </c>
+      <c r="K228" s="23">
+        <v>45375</v>
+      </c>
     </row>
     <row r="229" spans="1:11">
       <c r="A229" s="21" t="s">
@@ -14604,8 +14518,12 @@
       <c r="F229" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="G229" s="20"/>
-      <c r="H229" s="23"/>
+      <c r="G229" s="20">
+        <v>42925</v>
+      </c>
+      <c r="H229" s="23" t="s">
+        <v>1278</v>
+      </c>
       <c r="I229" s="23"/>
       <c r="J229" s="23"/>
       <c r="K229" s="23"/>
@@ -17662,7 +17580,7 @@
     </row>
     <row r="352" spans="1:11">
       <c r="A352" s="21" t="s">
-        <v>1287</v>
+        <v>1283</v>
       </c>
       <c r="B352" s="21" t="s">
         <v>158</v>
@@ -17687,7 +17605,7 @@
     </row>
     <row r="353" spans="1:11">
       <c r="A353" s="21" t="s">
-        <v>1288</v>
+        <v>1284</v>
       </c>
       <c r="B353" s="21" t="s">
         <v>158</v>
@@ -39153,10 +39071,10 @@
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1998:A2002">
-    <cfRule type="duplicateValues" dxfId="11" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A4:A1997">
-    <cfRule type="duplicateValues" dxfId="10" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="2"/>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4:H2002" xr:uid="{74B10176-32C1-4DCE-B9A9-308EB3B34100}">
@@ -39185,27 +39103,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="33.9" customHeight="1">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>1259</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
       <c r="H1" s="29"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="39" t="s">
         <v>1260</v>
       </c>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
       <c r="H2" s="26"/>
     </row>
     <row r="3" spans="1:8" ht="38.1" customHeight="1">

</xml_diff>

<commit_message>
fix(migration): onboard all 363 distinct member accounts preserving separate savings and asset loan accounts
</commit_message>
<xml_diff>
--- a/icare-group-member-onboarding-template.xlsx
+++ b/icare-group-member-onboarding-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\Master_ AY Projects\trustmicro-credit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46062980-C33F-44A2-AF4F-C191BFE649C3}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1D70E60-EC68-4E08-81C4-B8691B728FC5}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2575" uniqueCount="1321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2582" uniqueCount="1324">
   <si>
     <t>ICARE Group and Member Onboarding Template</t>
   </si>
@@ -3989,6 +3989,15 @@
   </si>
   <si>
     <t>Weekly 12W Asset</t>
+  </si>
+  <si>
+    <t>Awokoya Busayo</t>
+  </si>
+  <si>
+    <t>08070658141</t>
+  </si>
+  <si>
+    <t>MEM-363</t>
   </si>
 </sst>
 </file>
@@ -4188,7 +4197,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -4298,31 +4307,32 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4801,7 +4811,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="MemberOnboardingTable" displayName="MemberOnboardingTable" ref="A3:K2009" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="MemberOnboardingTable" displayName="MemberOnboardingTable" ref="A3:K2010" dataDxfId="14">
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Member Reference*" dataDxfId="13"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Group Reference*" dataDxfId="12"/>
@@ -4978,28 +4988,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="33.9" customHeight="1">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="2"/>
@@ -5019,13 +5029,13 @@
         <v>3</v>
       </c>
       <c r="C4" s="2"/>
-      <c r="D4" s="46" t="s">
+      <c r="D4" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="45"/>
-      <c r="H4" s="45"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="43"/>
     </row>
     <row r="5" spans="1:8" ht="27.9" customHeight="1">
       <c r="A5" s="3" t="s">
@@ -5036,10 +5046,10 @@
       <c r="D5" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="46"/>
     </row>
     <row r="6" spans="1:8" ht="27.9" customHeight="1">
       <c r="A6" s="3" t="s">
@@ -5050,10 +5060,10 @@
       <c r="D6" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="42"/>
-      <c r="H6" s="43"/>
+      <c r="E6" s="45"/>
+      <c r="F6" s="45"/>
+      <c r="G6" s="45"/>
+      <c r="H6" s="46"/>
     </row>
     <row r="7" spans="1:8" ht="27.9" customHeight="1">
       <c r="A7" s="3" t="s">
@@ -5064,10 +5074,10 @@
       <c r="D7" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="42"/>
-      <c r="F7" s="42"/>
-      <c r="G7" s="42"/>
-      <c r="H7" s="43"/>
+      <c r="E7" s="45"/>
+      <c r="F7" s="45"/>
+      <c r="G7" s="45"/>
+      <c r="H7" s="46"/>
     </row>
     <row r="8" spans="1:8" ht="27.9" customHeight="1">
       <c r="A8" s="3" t="s">
@@ -5078,10 +5088,10 @@
       <c r="D8" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="42"/>
-      <c r="F8" s="42"/>
-      <c r="G8" s="42"/>
-      <c r="H8" s="43"/>
+      <c r="E8" s="45"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="45"/>
+      <c r="H8" s="46"/>
     </row>
     <row r="9" spans="1:8" ht="27.9" customHeight="1">
       <c r="A9" s="3" t="s">
@@ -5092,10 +5102,10 @@
       <c r="D9" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="42"/>
-      <c r="F9" s="42"/>
-      <c r="G9" s="42"/>
-      <c r="H9" s="43"/>
+      <c r="E9" s="45"/>
+      <c r="F9" s="45"/>
+      <c r="G9" s="45"/>
+      <c r="H9" s="46"/>
     </row>
     <row r="10" spans="1:8" ht="27.9" customHeight="1">
       <c r="A10" s="2"/>
@@ -5104,10 +5114,10 @@
       <c r="D10" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="42"/>
-      <c r="F10" s="42"/>
-      <c r="G10" s="42"/>
-      <c r="H10" s="43"/>
+      <c r="E10" s="45"/>
+      <c r="F10" s="45"/>
+      <c r="G10" s="45"/>
+      <c r="H10" s="46"/>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="2"/>
@@ -5120,142 +5130,142 @@
       <c r="H11" s="2"/>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="51" t="s">
+      <c r="A12" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="45"/>
-      <c r="C12" s="45"/>
-      <c r="D12" s="45"/>
-      <c r="E12" s="45"/>
-      <c r="F12" s="45"/>
-      <c r="G12" s="45"/>
-      <c r="H12" s="45"/>
+      <c r="B12" s="43"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="43"/>
     </row>
     <row r="13" spans="1:8" ht="38.1" customHeight="1">
       <c r="A13" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="49" t="s">
+      <c r="B13" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="42"/>
-      <c r="D13" s="42"/>
-      <c r="E13" s="42"/>
-      <c r="F13" s="42"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="43"/>
+      <c r="C13" s="45"/>
+      <c r="D13" s="45"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="45"/>
+      <c r="G13" s="45"/>
+      <c r="H13" s="46"/>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="48" t="s">
+      <c r="B14" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="42"/>
-      <c r="D14" s="42"/>
-      <c r="E14" s="42"/>
-      <c r="F14" s="42"/>
-      <c r="G14" s="42"/>
-      <c r="H14" s="43"/>
+      <c r="C14" s="45"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="45"/>
+      <c r="F14" s="45"/>
+      <c r="G14" s="45"/>
+      <c r="H14" s="46"/>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="48" t="s">
+      <c r="B15" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="42"/>
-      <c r="D15" s="42"/>
-      <c r="E15" s="42"/>
-      <c r="F15" s="42"/>
-      <c r="G15" s="42"/>
-      <c r="H15" s="43"/>
+      <c r="C15" s="45"/>
+      <c r="D15" s="45"/>
+      <c r="E15" s="45"/>
+      <c r="F15" s="45"/>
+      <c r="G15" s="45"/>
+      <c r="H15" s="46"/>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="48" t="s">
+      <c r="B16" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="42"/>
-      <c r="D16" s="42"/>
-      <c r="E16" s="42"/>
-      <c r="F16" s="42"/>
-      <c r="G16" s="42"/>
-      <c r="H16" s="43"/>
+      <c r="C16" s="45"/>
+      <c r="D16" s="45"/>
+      <c r="E16" s="45"/>
+      <c r="F16" s="45"/>
+      <c r="G16" s="45"/>
+      <c r="H16" s="46"/>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="48" t="s">
+      <c r="B17" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="42"/>
-      <c r="D17" s="42"/>
-      <c r="E17" s="42"/>
-      <c r="F17" s="42"/>
-      <c r="G17" s="42"/>
-      <c r="H17" s="43"/>
+      <c r="C17" s="45"/>
+      <c r="D17" s="45"/>
+      <c r="E17" s="45"/>
+      <c r="F17" s="45"/>
+      <c r="G17" s="45"/>
+      <c r="H17" s="46"/>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="48" t="s">
+      <c r="B18" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="42"/>
-      <c r="D18" s="42"/>
-      <c r="E18" s="42"/>
-      <c r="F18" s="42"/>
-      <c r="G18" s="42"/>
-      <c r="H18" s="43"/>
+      <c r="C18" s="45"/>
+      <c r="D18" s="45"/>
+      <c r="E18" s="45"/>
+      <c r="F18" s="45"/>
+      <c r="G18" s="45"/>
+      <c r="H18" s="46"/>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="48" t="s">
+      <c r="B19" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="42"/>
-      <c r="D19" s="42"/>
-      <c r="E19" s="42"/>
-      <c r="F19" s="42"/>
-      <c r="G19" s="42"/>
-      <c r="H19" s="43"/>
+      <c r="C19" s="45"/>
+      <c r="D19" s="45"/>
+      <c r="E19" s="45"/>
+      <c r="F19" s="45"/>
+      <c r="G19" s="45"/>
+      <c r="H19" s="46"/>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="48" t="s">
+      <c r="B20" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="42"/>
-      <c r="D20" s="42"/>
-      <c r="E20" s="42"/>
-      <c r="F20" s="42"/>
-      <c r="G20" s="42"/>
-      <c r="H20" s="43"/>
+      <c r="C20" s="45"/>
+      <c r="D20" s="45"/>
+      <c r="E20" s="45"/>
+      <c r="F20" s="45"/>
+      <c r="G20" s="45"/>
+      <c r="H20" s="46"/>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="41" t="s">
+      <c r="B21" s="49" t="s">
         <v>34</v>
       </c>
-      <c r="C21" s="42"/>
-      <c r="D21" s="42"/>
-      <c r="E21" s="42"/>
-      <c r="F21" s="42"/>
-      <c r="G21" s="42"/>
-      <c r="H21" s="43"/>
+      <c r="C21" s="45"/>
+      <c r="D21" s="45"/>
+      <c r="E21" s="45"/>
+      <c r="F21" s="45"/>
+      <c r="G21" s="45"/>
+      <c r="H21" s="46"/>
     </row>
   </sheetData>
   <autoFilter ref="A12:H21" xr:uid="{00000000-0009-0000-0000-000000000000}">
@@ -5268,13 +5278,6 @@
     <filterColumn colId="6" showButton="0"/>
   </autoFilter>
   <mergeCells count="19">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="B20:H20"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="B16:H16"/>
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="B18:H18"/>
     <mergeCell ref="B21:H21"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="D4:H4"/>
@@ -5287,6 +5290,13 @@
     <mergeCell ref="B19:H19"/>
     <mergeCell ref="D10:H10"/>
     <mergeCell ref="B15:H15"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B20:H20"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="B18:H18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5309,30 +5319,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="33.9" customHeight="1">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
     </row>
     <row r="3" spans="1:9" ht="38.1" customHeight="1">
       <c r="A3" s="28" t="s">
@@ -8853,7 +8863,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K2009"/>
+  <dimension ref="A1:K2010"/>
   <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="2" width="22.09765625" style="27" customWidth="1"/>
@@ -8865,34 +8875,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="33.9" customHeight="1">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="42" t="s">
         <v>161</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+      <c r="I1" s="55"/>
+      <c r="J1" s="55"/>
+      <c r="K1" s="55"/>
     </row>
     <row r="2" spans="1:11" ht="30" customHeight="1">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="53" t="s">
         <v>162</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="53"/>
-      <c r="I2" s="53"/>
-      <c r="J2" s="53"/>
-      <c r="K2" s="53"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+      <c r="J2" s="54"/>
+      <c r="K2" s="54"/>
     </row>
     <row r="3" spans="1:11" ht="38.1" customHeight="1">
       <c r="A3" s="28" t="s">
@@ -13497,30 +13507,34 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="184" spans="1:11">
+    <row r="184" spans="1:11" s="41" customFormat="1">
       <c r="A184" s="21" t="s">
         <v>747</v>
       </c>
       <c r="B184" s="21" t="s">
-        <v>95</v>
-      </c>
-      <c r="C184" s="21" t="s">
-        <v>174</v>
-      </c>
-      <c r="D184" s="22" t="s">
-        <v>726</v>
-      </c>
-      <c r="E184" s="21" t="s">
-        <v>727</v>
+        <v>92</v>
+      </c>
+      <c r="C184" s="39" t="s">
+        <v>300</v>
+      </c>
+      <c r="D184" s="40" t="s">
+        <v>1321</v>
+      </c>
+      <c r="E184" s="39" t="s">
+        <v>1322</v>
       </c>
       <c r="F184" s="22" t="s">
-        <v>728</v>
-      </c>
-      <c r="G184" s="20"/>
-      <c r="H184" s="23"/>
-      <c r="I184" s="23"/>
-      <c r="J184" s="23"/>
-      <c r="K184" s="23"/>
+        <v>696</v>
+      </c>
+      <c r="G184" s="35">
+        <v>11000</v>
+      </c>
+      <c r="H184" s="33" t="s">
+        <v>1275</v>
+      </c>
+      <c r="I184" s="33"/>
+      <c r="J184" s="33"/>
+      <c r="K184" s="33"/>
     </row>
     <row r="185" spans="1:11">
       <c r="A185" s="21" t="s">
@@ -13530,13 +13544,13 @@
         <v>95</v>
       </c>
       <c r="C185" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D185" s="22" t="s">
-        <v>730</v>
+        <v>726</v>
       </c>
       <c r="E185" s="21" t="s">
-        <v>731</v>
+        <v>727</v>
       </c>
       <c r="F185" s="22" t="s">
         <v>728</v>
@@ -13555,16 +13569,16 @@
         <v>95</v>
       </c>
       <c r="C186" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D186" s="22" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
       <c r="E186" s="21" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
       <c r="F186" s="22" t="s">
-        <v>735</v>
+        <v>728</v>
       </c>
       <c r="G186" s="20"/>
       <c r="H186" s="23"/>
@@ -13580,13 +13594,13 @@
         <v>95</v>
       </c>
       <c r="C187" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D187" s="22" t="s">
-        <v>737</v>
+        <v>733</v>
       </c>
       <c r="E187" s="21" t="s">
-        <v>738</v>
+        <v>734</v>
       </c>
       <c r="F187" s="22" t="s">
         <v>735</v>
@@ -13605,13 +13619,13 @@
         <v>95</v>
       </c>
       <c r="C188" s="21" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D188" s="22" t="s">
-        <v>349</v>
+        <v>737</v>
       </c>
       <c r="E188" s="21" t="s">
-        <v>350</v>
+        <v>738</v>
       </c>
       <c r="F188" s="22" t="s">
         <v>735</v>
@@ -13627,19 +13641,19 @@
         <v>758</v>
       </c>
       <c r="B189" s="21" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C189" s="21" t="s">
-        <v>174</v>
+        <v>198</v>
       </c>
       <c r="D189" s="22" t="s">
-        <v>741</v>
+        <v>349</v>
       </c>
       <c r="E189" s="21" t="s">
-        <v>742</v>
+        <v>350</v>
       </c>
       <c r="F189" s="22" t="s">
-        <v>743</v>
+        <v>735</v>
       </c>
       <c r="G189" s="20"/>
       <c r="H189" s="23"/>
@@ -13655,13 +13669,13 @@
         <v>98</v>
       </c>
       <c r="C190" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D190" s="22" t="s">
-        <v>745</v>
+        <v>741</v>
       </c>
       <c r="E190" s="21" t="s">
-        <v>746</v>
+        <v>742</v>
       </c>
       <c r="F190" s="22" t="s">
         <v>743</v>
@@ -13680,13 +13694,13 @@
         <v>98</v>
       </c>
       <c r="C191" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D191" s="22" t="s">
-        <v>748</v>
+        <v>745</v>
       </c>
       <c r="E191" s="21" t="s">
-        <v>749</v>
+        <v>746</v>
       </c>
       <c r="F191" s="22" t="s">
         <v>743</v>
@@ -13705,12 +13719,14 @@
         <v>98</v>
       </c>
       <c r="C192" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D192" s="22" t="s">
-        <v>751</v>
-      </c>
-      <c r="E192" s="21"/>
+        <v>748</v>
+      </c>
+      <c r="E192" s="21" t="s">
+        <v>749</v>
+      </c>
       <c r="F192" s="22" t="s">
         <v>743</v>
       </c>
@@ -13725,17 +13741,17 @@
         <v>771</v>
       </c>
       <c r="B193" s="21" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C193" s="21" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
       <c r="D193" s="22" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="E193" s="21"/>
       <c r="F193" s="22" t="s">
-        <v>709</v>
+        <v>743</v>
       </c>
       <c r="G193" s="20"/>
       <c r="H193" s="23"/>
@@ -13751,14 +13767,14 @@
         <v>101</v>
       </c>
       <c r="C194" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D194" s="22" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="E194" s="21"/>
       <c r="F194" s="22" t="s">
-        <v>696</v>
+        <v>709</v>
       </c>
       <c r="G194" s="20"/>
       <c r="H194" s="23"/>
@@ -13774,10 +13790,10 @@
         <v>101</v>
       </c>
       <c r="C195" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D195" s="22" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="E195" s="21"/>
       <c r="F195" s="22" t="s">
@@ -13794,19 +13810,17 @@
         <v>781</v>
       </c>
       <c r="B196" s="21" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C196" s="21" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="D196" s="22" t="s">
-        <v>759</v>
-      </c>
-      <c r="E196" s="21" t="s">
-        <v>760</v>
-      </c>
+        <v>757</v>
+      </c>
+      <c r="E196" s="21"/>
       <c r="F196" s="22" t="s">
-        <v>761</v>
+        <v>696</v>
       </c>
       <c r="G196" s="20"/>
       <c r="H196" s="23"/>
@@ -13822,13 +13836,13 @@
         <v>103</v>
       </c>
       <c r="C197" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D197" s="22" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="E197" s="21" t="s">
-        <v>764</v>
+        <v>760</v>
       </c>
       <c r="F197" s="22" t="s">
         <v>761</v>
@@ -13847,13 +13861,13 @@
         <v>103</v>
       </c>
       <c r="C198" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D198" s="22" t="s">
-        <v>766</v>
+        <v>763</v>
       </c>
       <c r="E198" s="21" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
       <c r="F198" s="22" t="s">
         <v>761</v>
@@ -13872,13 +13886,13 @@
         <v>103</v>
       </c>
       <c r="C199" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D199" s="22" t="s">
-        <v>769</v>
+        <v>766</v>
       </c>
       <c r="E199" s="21" t="s">
-        <v>770</v>
+        <v>767</v>
       </c>
       <c r="F199" s="22" t="s">
         <v>761</v>
@@ -13894,19 +13908,19 @@
         <v>792</v>
       </c>
       <c r="B200" s="21" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C200" s="21" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
       <c r="D200" s="22" t="s">
-        <v>772</v>
+        <v>769</v>
       </c>
       <c r="E200" s="21" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="F200" s="22" t="s">
-        <v>774</v>
+        <v>761</v>
       </c>
       <c r="G200" s="20"/>
       <c r="H200" s="23"/>
@@ -13922,13 +13936,13 @@
         <v>105</v>
       </c>
       <c r="C201" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D201" s="22" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="E201" s="21" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="F201" s="22" t="s">
         <v>774</v>
@@ -13947,13 +13961,13 @@
         <v>105</v>
       </c>
       <c r="C202" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D202" s="22" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
       <c r="E202" s="21" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="F202" s="22" t="s">
         <v>774</v>
@@ -13972,13 +13986,13 @@
         <v>105</v>
       </c>
       <c r="C203" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D203" s="22" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
       <c r="E203" s="21" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
       <c r="F203" s="22" t="s">
         <v>774</v>
@@ -13997,12 +14011,14 @@
         <v>105</v>
       </c>
       <c r="C204" s="21" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D204" s="22" t="s">
-        <v>785</v>
-      </c>
-      <c r="E204" s="21"/>
+        <v>782</v>
+      </c>
+      <c r="E204" s="21" t="s">
+        <v>783</v>
+      </c>
       <c r="F204" s="22" t="s">
         <v>774</v>
       </c>
@@ -14020,14 +14036,12 @@
         <v>105</v>
       </c>
       <c r="C205" s="21" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D205" s="22" t="s">
-        <v>787</v>
-      </c>
-      <c r="E205" s="21" t="s">
-        <v>788</v>
-      </c>
+        <v>785</v>
+      </c>
+      <c r="E205" s="21"/>
       <c r="F205" s="22" t="s">
         <v>774</v>
       </c>
@@ -14045,13 +14059,13 @@
         <v>105</v>
       </c>
       <c r="C206" s="21" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D206" s="22" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
       <c r="E206" s="21" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
       <c r="F206" s="22" t="s">
         <v>774</v>
@@ -14070,13 +14084,13 @@
         <v>105</v>
       </c>
       <c r="C207" s="21" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="D207" s="22" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
       <c r="E207" s="21" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
       <c r="F207" s="22" t="s">
         <v>774</v>
@@ -14095,13 +14109,13 @@
         <v>105</v>
       </c>
       <c r="C208" s="21" t="s">
-        <v>258</v>
+        <v>210</v>
       </c>
       <c r="D208" s="22" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
       <c r="E208" s="21" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="F208" s="22" t="s">
         <v>774</v>
@@ -14120,13 +14134,13 @@
         <v>105</v>
       </c>
       <c r="C209" s="21" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D209" s="22" t="s">
-        <v>799</v>
+        <v>796</v>
       </c>
       <c r="E209" s="21" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="F209" s="22" t="s">
         <v>774</v>
@@ -14142,19 +14156,19 @@
         <v>823</v>
       </c>
       <c r="B210" s="21" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C210" s="21" t="s">
-        <v>174</v>
+        <v>262</v>
       </c>
       <c r="D210" s="22" t="s">
-        <v>802</v>
+        <v>799</v>
       </c>
       <c r="E210" s="21" t="s">
-        <v>803</v>
+        <v>800</v>
       </c>
       <c r="F210" s="22" t="s">
-        <v>804</v>
+        <v>774</v>
       </c>
       <c r="G210" s="20"/>
       <c r="H210" s="23"/>
@@ -14170,13 +14184,13 @@
         <v>108</v>
       </c>
       <c r="C211" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D211" s="22" t="s">
-        <v>806</v>
+        <v>802</v>
       </c>
       <c r="E211" s="21" t="s">
-        <v>807</v>
+        <v>803</v>
       </c>
       <c r="F211" s="22" t="s">
         <v>804</v>
@@ -14195,13 +14209,13 @@
         <v>108</v>
       </c>
       <c r="C212" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D212" s="22" t="s">
-        <v>809</v>
+        <v>806</v>
       </c>
       <c r="E212" s="21" t="s">
-        <v>810</v>
+        <v>807</v>
       </c>
       <c r="F212" s="22" t="s">
         <v>804</v>
@@ -14220,13 +14234,13 @@
         <v>108</v>
       </c>
       <c r="C213" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D213" s="22" t="s">
-        <v>812</v>
+        <v>809</v>
       </c>
       <c r="E213" s="21" t="s">
-        <v>813</v>
+        <v>810</v>
       </c>
       <c r="F213" s="22" t="s">
         <v>804</v>
@@ -14245,13 +14259,13 @@
         <v>108</v>
       </c>
       <c r="C214" s="21" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D214" s="22" t="s">
-        <v>815</v>
+        <v>812</v>
       </c>
       <c r="E214" s="21" t="s">
-        <v>816</v>
+        <v>813</v>
       </c>
       <c r="F214" s="22" t="s">
         <v>804</v>
@@ -14270,13 +14284,13 @@
         <v>108</v>
       </c>
       <c r="C215" s="21" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D215" s="22" t="s">
-        <v>818</v>
+        <v>815</v>
       </c>
       <c r="E215" s="21" t="s">
-        <v>819</v>
+        <v>816</v>
       </c>
       <c r="F215" s="22" t="s">
         <v>804</v>
@@ -14295,22 +14309,22 @@
         <v>108</v>
       </c>
       <c r="C216" s="21" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D216" s="22" t="s">
-        <v>1277</v>
+        <v>818</v>
       </c>
       <c r="E216" s="21" t="s">
-        <v>1278</v>
+        <v>819</v>
       </c>
       <c r="F216" s="22" t="s">
         <v>804</v>
       </c>
-      <c r="G216" s="35"/>
+      <c r="G216" s="20"/>
       <c r="H216" s="23"/>
       <c r="I216" s="23"/>
       <c r="J216" s="23"/>
-      <c r="K216" s="33"/>
+      <c r="K216" s="23"/>
     </row>
     <row r="217" spans="1:11">
       <c r="A217" s="21" t="s">
@@ -14320,13 +14334,13 @@
         <v>108</v>
       </c>
       <c r="C217" s="21" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="D217" s="22" t="s">
-        <v>1279</v>
+        <v>1277</v>
       </c>
       <c r="E217" s="21" t="s">
-        <v>1280</v>
+        <v>1278</v>
       </c>
       <c r="F217" s="22" t="s">
         <v>804</v>
@@ -14342,25 +14356,25 @@
         <v>847</v>
       </c>
       <c r="B218" s="21" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C218" s="21" t="s">
-        <v>174</v>
+        <v>210</v>
       </c>
       <c r="D218" s="22" t="s">
-        <v>821</v>
+        <v>1279</v>
       </c>
       <c r="E218" s="21" t="s">
-        <v>822</v>
+        <v>1280</v>
       </c>
       <c r="F218" s="22" t="s">
-        <v>709</v>
-      </c>
-      <c r="G218" s="20"/>
+        <v>804</v>
+      </c>
+      <c r="G218" s="35"/>
       <c r="H218" s="23"/>
       <c r="I218" s="23"/>
       <c r="J218" s="23"/>
-      <c r="K218" s="23"/>
+      <c r="K218" s="33"/>
     </row>
     <row r="219" spans="1:11">
       <c r="A219" s="21" t="s">
@@ -14370,16 +14384,16 @@
         <v>110</v>
       </c>
       <c r="C219" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D219" s="22" t="s">
-        <v>824</v>
+        <v>821</v>
       </c>
       <c r="E219" s="21" t="s">
-        <v>825</v>
+        <v>822</v>
       </c>
       <c r="F219" s="22" t="s">
-        <v>696</v>
+        <v>709</v>
       </c>
       <c r="G219" s="20"/>
       <c r="H219" s="23"/>
@@ -14395,13 +14409,13 @@
         <v>110</v>
       </c>
       <c r="C220" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D220" s="22" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="E220" s="21" t="s">
-        <v>828</v>
+        <v>825</v>
       </c>
       <c r="F220" s="22" t="s">
         <v>696</v>
@@ -14420,16 +14434,16 @@
         <v>110</v>
       </c>
       <c r="C221" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D221" s="22" t="s">
-        <v>830</v>
+        <v>827</v>
       </c>
       <c r="E221" s="21" t="s">
-        <v>831</v>
+        <v>828</v>
       </c>
       <c r="F221" s="22" t="s">
-        <v>709</v>
+        <v>696</v>
       </c>
       <c r="G221" s="20"/>
       <c r="H221" s="23"/>
@@ -14445,13 +14459,13 @@
         <v>110</v>
       </c>
       <c r="C222" s="21" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D222" s="22" t="s">
-        <v>833</v>
+        <v>830</v>
       </c>
       <c r="E222" s="21" t="s">
-        <v>834</v>
+        <v>831</v>
       </c>
       <c r="F222" s="22" t="s">
         <v>709</v>
@@ -14467,19 +14481,19 @@
         <v>858</v>
       </c>
       <c r="B223" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C223" s="21" t="s">
-        <v>174</v>
+        <v>198</v>
       </c>
       <c r="D223" s="22" t="s">
-        <v>1269</v>
+        <v>833</v>
       </c>
       <c r="E223" s="21" t="s">
-        <v>836</v>
+        <v>834</v>
       </c>
       <c r="F223" s="22" t="s">
-        <v>837</v>
+        <v>709</v>
       </c>
       <c r="G223" s="20"/>
       <c r="H223" s="23"/>
@@ -14495,13 +14509,13 @@
         <v>112</v>
       </c>
       <c r="C224" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D224" s="22" t="s">
-        <v>839</v>
+        <v>1269</v>
       </c>
       <c r="E224" s="21" t="s">
-        <v>840</v>
+        <v>836</v>
       </c>
       <c r="F224" s="22" t="s">
         <v>837</v>
@@ -14520,13 +14534,13 @@
         <v>112</v>
       </c>
       <c r="C225" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D225" s="22" t="s">
-        <v>842</v>
+        <v>839</v>
       </c>
       <c r="E225" s="21" t="s">
-        <v>843</v>
+        <v>840</v>
       </c>
       <c r="F225" s="22" t="s">
         <v>837</v>
@@ -14545,13 +14559,13 @@
         <v>112</v>
       </c>
       <c r="C226" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D226" s="22" t="s">
-        <v>845</v>
+        <v>842</v>
       </c>
       <c r="E226" s="21" t="s">
-        <v>846</v>
+        <v>843</v>
       </c>
       <c r="F226" s="22" t="s">
         <v>837</v>
@@ -14570,13 +14584,13 @@
         <v>112</v>
       </c>
       <c r="C227" s="21" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D227" s="22" t="s">
-        <v>1270</v>
+        <v>845</v>
       </c>
       <c r="E227" s="21" t="s">
-        <v>1272</v>
+        <v>846</v>
       </c>
       <c r="F227" s="22" t="s">
         <v>837</v>
@@ -14595,13 +14609,13 @@
         <v>112</v>
       </c>
       <c r="C228" s="21" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D228" s="22" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="E228" s="21" t="s">
-        <v>1273</v>
+        <v>1272</v>
       </c>
       <c r="F228" s="22" t="s">
         <v>837</v>
@@ -14620,13 +14634,13 @@
         <v>112</v>
       </c>
       <c r="C229" s="21" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D229" s="22" t="s">
-        <v>850</v>
+        <v>1271</v>
       </c>
       <c r="E229" s="21" t="s">
-        <v>851</v>
+        <v>1273</v>
       </c>
       <c r="F229" s="22" t="s">
         <v>837</v>
@@ -14645,13 +14659,13 @@
         <v>112</v>
       </c>
       <c r="C230" s="21" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="D230" s="22" t="s">
-        <v>853</v>
+        <v>850</v>
       </c>
       <c r="E230" s="21" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="F230" s="22" t="s">
         <v>837</v>
@@ -14670,13 +14684,13 @@
         <v>112</v>
       </c>
       <c r="C231" s="21" t="s">
-        <v>258</v>
+        <v>210</v>
       </c>
       <c r="D231" s="22" t="s">
-        <v>856</v>
+        <v>853</v>
       </c>
       <c r="E231" s="21" t="s">
-        <v>857</v>
+        <v>854</v>
       </c>
       <c r="F231" s="22" t="s">
         <v>837</v>
@@ -14692,16 +14706,16 @@
         <v>885</v>
       </c>
       <c r="B232" s="21" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C232" s="21" t="s">
-        <v>174</v>
+        <v>258</v>
       </c>
       <c r="D232" s="22" t="s">
-        <v>859</v>
+        <v>856</v>
       </c>
       <c r="E232" s="21" t="s">
-        <v>860</v>
+        <v>857</v>
       </c>
       <c r="F232" s="22" t="s">
         <v>837</v>
@@ -14720,13 +14734,13 @@
         <v>115</v>
       </c>
       <c r="C233" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D233" s="22" t="s">
-        <v>862</v>
+        <v>859</v>
       </c>
       <c r="E233" s="21" t="s">
-        <v>863</v>
+        <v>860</v>
       </c>
       <c r="F233" s="22" t="s">
         <v>837</v>
@@ -14745,13 +14759,13 @@
         <v>115</v>
       </c>
       <c r="C234" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D234" s="22" t="s">
-        <v>865</v>
+        <v>862</v>
       </c>
       <c r="E234" s="21" t="s">
-        <v>866</v>
+        <v>863</v>
       </c>
       <c r="F234" s="22" t="s">
         <v>837</v>
@@ -14770,13 +14784,13 @@
         <v>115</v>
       </c>
       <c r="C235" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D235" s="22" t="s">
-        <v>868</v>
+        <v>865</v>
       </c>
       <c r="E235" s="21" t="s">
-        <v>869</v>
+        <v>866</v>
       </c>
       <c r="F235" s="22" t="s">
         <v>837</v>
@@ -14795,12 +14809,14 @@
         <v>115</v>
       </c>
       <c r="C236" s="21" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D236" s="22" t="s">
-        <v>871</v>
-      </c>
-      <c r="E236" s="21"/>
+        <v>868</v>
+      </c>
+      <c r="E236" s="21" t="s">
+        <v>869</v>
+      </c>
       <c r="F236" s="22" t="s">
         <v>837</v>
       </c>
@@ -14815,19 +14831,17 @@
         <v>900</v>
       </c>
       <c r="B237" s="21" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C237" s="21" t="s">
-        <v>174</v>
+        <v>198</v>
       </c>
       <c r="D237" s="22" t="s">
-        <v>873</v>
-      </c>
-      <c r="E237" s="21" t="s">
-        <v>874</v>
-      </c>
+        <v>871</v>
+      </c>
+      <c r="E237" s="21"/>
       <c r="F237" s="22" t="s">
-        <v>875</v>
+        <v>837</v>
       </c>
       <c r="G237" s="20"/>
       <c r="H237" s="23"/>
@@ -14843,13 +14857,13 @@
         <v>117</v>
       </c>
       <c r="C238" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D238" s="22" t="s">
-        <v>877</v>
+        <v>873</v>
       </c>
       <c r="E238" s="21" t="s">
-        <v>878</v>
+        <v>874</v>
       </c>
       <c r="F238" s="22" t="s">
         <v>875</v>
@@ -14868,13 +14882,13 @@
         <v>117</v>
       </c>
       <c r="C239" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D239" s="22" t="s">
-        <v>880</v>
+        <v>877</v>
       </c>
       <c r="E239" s="21" t="s">
-        <v>881</v>
+        <v>878</v>
       </c>
       <c r="F239" s="22" t="s">
         <v>875</v>
@@ -14893,13 +14907,13 @@
         <v>117</v>
       </c>
       <c r="C240" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D240" s="22" t="s">
-        <v>883</v>
+        <v>880</v>
       </c>
       <c r="E240" s="21" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
       <c r="F240" s="22" t="s">
         <v>875</v>
@@ -14918,13 +14932,13 @@
         <v>117</v>
       </c>
       <c r="C241" s="21" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D241" s="22" t="s">
-        <v>886</v>
+        <v>883</v>
       </c>
       <c r="E241" s="21" t="s">
-        <v>887</v>
+        <v>884</v>
       </c>
       <c r="F241" s="22" t="s">
         <v>875</v>
@@ -14943,13 +14957,13 @@
         <v>117</v>
       </c>
       <c r="C242" s="21" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D242" s="22" t="s">
-        <v>889</v>
+        <v>886</v>
       </c>
       <c r="E242" s="21" t="s">
-        <v>890</v>
+        <v>887</v>
       </c>
       <c r="F242" s="22" t="s">
         <v>875</v>
@@ -14968,13 +14982,13 @@
         <v>117</v>
       </c>
       <c r="C243" s="21" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D243" s="22" t="s">
-        <v>892</v>
+        <v>889</v>
       </c>
       <c r="E243" s="21" t="s">
-        <v>893</v>
+        <v>890</v>
       </c>
       <c r="F243" s="22" t="s">
         <v>875</v>
@@ -14993,13 +15007,13 @@
         <v>117</v>
       </c>
       <c r="C244" s="21" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="D244" s="22" t="s">
-        <v>895</v>
+        <v>892</v>
       </c>
       <c r="E244" s="21" t="s">
-        <v>896</v>
+        <v>893</v>
       </c>
       <c r="F244" s="22" t="s">
         <v>875</v>
@@ -15018,13 +15032,13 @@
         <v>117</v>
       </c>
       <c r="C245" s="21" t="s">
-        <v>258</v>
+        <v>210</v>
       </c>
       <c r="D245" s="22" t="s">
-        <v>898</v>
+        <v>895</v>
       </c>
       <c r="E245" s="21" t="s">
-        <v>899</v>
+        <v>896</v>
       </c>
       <c r="F245" s="22" t="s">
         <v>875</v>
@@ -15043,13 +15057,13 @@
         <v>117</v>
       </c>
       <c r="C246" s="21" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D246" s="22" t="s">
-        <v>901</v>
+        <v>898</v>
       </c>
       <c r="E246" s="21" t="s">
-        <v>902</v>
+        <v>899</v>
       </c>
       <c r="F246" s="22" t="s">
         <v>875</v>
@@ -15068,13 +15082,13 @@
         <v>117</v>
       </c>
       <c r="C247" s="21" t="s">
-        <v>296</v>
+        <v>262</v>
       </c>
       <c r="D247" s="22" t="s">
-        <v>904</v>
+        <v>901</v>
       </c>
       <c r="E247" s="21" t="s">
-        <v>905</v>
+        <v>902</v>
       </c>
       <c r="F247" s="22" t="s">
         <v>875</v>
@@ -15093,13 +15107,13 @@
         <v>117</v>
       </c>
       <c r="C248" s="21" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D248" s="22" t="s">
-        <v>907</v>
+        <v>904</v>
       </c>
       <c r="E248" s="21" t="s">
-        <v>908</v>
+        <v>905</v>
       </c>
       <c r="F248" s="22" t="s">
         <v>875</v>
@@ -15118,13 +15132,13 @@
         <v>117</v>
       </c>
       <c r="C249" s="21" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="D249" s="22" t="s">
-        <v>910</v>
+        <v>907</v>
       </c>
       <c r="E249" s="21" t="s">
-        <v>911</v>
+        <v>908</v>
       </c>
       <c r="F249" s="22" t="s">
         <v>875</v>
@@ -15143,13 +15157,13 @@
         <v>117</v>
       </c>
       <c r="C250" s="21" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D250" s="22" t="s">
-        <v>913</v>
+        <v>910</v>
       </c>
       <c r="E250" s="21" t="s">
-        <v>914</v>
+        <v>911</v>
       </c>
       <c r="F250" s="22" t="s">
         <v>875</v>
@@ -15165,19 +15179,19 @@
         <v>944</v>
       </c>
       <c r="B251" s="21" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="C251" s="21" t="s">
-        <v>174</v>
+        <v>308</v>
       </c>
       <c r="D251" s="22" t="s">
-        <v>916</v>
+        <v>913</v>
       </c>
       <c r="E251" s="21" t="s">
-        <v>917</v>
+        <v>914</v>
       </c>
       <c r="F251" s="22" t="s">
-        <v>918</v>
+        <v>875</v>
       </c>
       <c r="G251" s="20"/>
       <c r="H251" s="23"/>
@@ -15193,13 +15207,13 @@
         <v>122</v>
       </c>
       <c r="C252" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D252" s="22" t="s">
-        <v>920</v>
+        <v>916</v>
       </c>
       <c r="E252" s="21" t="s">
-        <v>921</v>
+        <v>917</v>
       </c>
       <c r="F252" s="22" t="s">
         <v>918</v>
@@ -15218,13 +15232,13 @@
         <v>122</v>
       </c>
       <c r="C253" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D253" s="22" t="s">
-        <v>923</v>
+        <v>920</v>
       </c>
       <c r="E253" s="21" t="s">
-        <v>924</v>
+        <v>921</v>
       </c>
       <c r="F253" s="22" t="s">
         <v>918</v>
@@ -15243,13 +15257,13 @@
         <v>122</v>
       </c>
       <c r="C254" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D254" s="22" t="s">
-        <v>926</v>
+        <v>923</v>
       </c>
       <c r="E254" s="21" t="s">
-        <v>927</v>
+        <v>924</v>
       </c>
       <c r="F254" s="22" t="s">
         <v>918</v>
@@ -15268,13 +15282,13 @@
         <v>122</v>
       </c>
       <c r="C255" s="21" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D255" s="22" t="s">
-        <v>929</v>
+        <v>926</v>
       </c>
       <c r="E255" s="21" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="F255" s="22" t="s">
         <v>918</v>
@@ -15293,13 +15307,13 @@
         <v>122</v>
       </c>
       <c r="C256" s="21" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D256" s="22" t="s">
-        <v>932</v>
+        <v>929</v>
       </c>
       <c r="E256" s="21" t="s">
-        <v>933</v>
+        <v>930</v>
       </c>
       <c r="F256" s="22" t="s">
         <v>918</v>
@@ -15318,13 +15332,13 @@
         <v>122</v>
       </c>
       <c r="C257" s="21" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D257" s="22" t="s">
-        <v>935</v>
+        <v>932</v>
       </c>
       <c r="E257" s="21" t="s">
-        <v>936</v>
+        <v>933</v>
       </c>
       <c r="F257" s="22" t="s">
         <v>918</v>
@@ -15340,19 +15354,19 @@
         <v>964</v>
       </c>
       <c r="B258" s="21" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C258" s="21" t="s">
-        <v>174</v>
+        <v>206</v>
       </c>
       <c r="D258" s="22" t="s">
-        <v>938</v>
+        <v>935</v>
       </c>
       <c r="E258" s="21" t="s">
-        <v>939</v>
+        <v>936</v>
       </c>
       <c r="F258" s="22" t="s">
-        <v>940</v>
+        <v>918</v>
       </c>
       <c r="G258" s="20"/>
       <c r="H258" s="23"/>
@@ -15368,13 +15382,13 @@
         <v>125</v>
       </c>
       <c r="C259" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D259" s="22" t="s">
-        <v>942</v>
+        <v>938</v>
       </c>
       <c r="E259" s="21" t="s">
-        <v>943</v>
+        <v>939</v>
       </c>
       <c r="F259" s="22" t="s">
         <v>940</v>
@@ -15393,13 +15407,13 @@
         <v>125</v>
       </c>
       <c r="C260" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D260" s="22" t="s">
-        <v>945</v>
+        <v>942</v>
       </c>
       <c r="E260" s="21" t="s">
-        <v>946</v>
+        <v>943</v>
       </c>
       <c r="F260" s="22" t="s">
         <v>940</v>
@@ -15418,13 +15432,13 @@
         <v>125</v>
       </c>
       <c r="C261" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D261" s="22" t="s">
-        <v>948</v>
+        <v>945</v>
       </c>
       <c r="E261" s="21" t="s">
-        <v>949</v>
+        <v>946</v>
       </c>
       <c r="F261" s="22" t="s">
         <v>940</v>
@@ -15443,13 +15457,13 @@
         <v>125</v>
       </c>
       <c r="C262" s="21" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D262" s="22" t="s">
-        <v>929</v>
+        <v>948</v>
       </c>
       <c r="E262" s="21" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
       <c r="F262" s="22" t="s">
         <v>940</v>
@@ -15468,13 +15482,13 @@
         <v>125</v>
       </c>
       <c r="C263" s="21" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D263" s="22" t="s">
-        <v>953</v>
+        <v>929</v>
       </c>
       <c r="E263" s="21" t="s">
-        <v>954</v>
+        <v>951</v>
       </c>
       <c r="F263" s="22" t="s">
         <v>940</v>
@@ -15493,13 +15507,13 @@
         <v>125</v>
       </c>
       <c r="C264" s="21" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D264" s="22" t="s">
-        <v>956</v>
+        <v>953</v>
       </c>
       <c r="E264" s="21" t="s">
-        <v>957</v>
+        <v>954</v>
       </c>
       <c r="F264" s="22" t="s">
         <v>940</v>
@@ -15518,13 +15532,13 @@
         <v>125</v>
       </c>
       <c r="C265" s="21" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="D265" s="22" t="s">
-        <v>959</v>
+        <v>956</v>
       </c>
       <c r="E265" s="21" t="s">
-        <v>960</v>
+        <v>957</v>
       </c>
       <c r="F265" s="22" t="s">
         <v>940</v>
@@ -15543,13 +15557,13 @@
         <v>125</v>
       </c>
       <c r="C266" s="21" t="s">
-        <v>258</v>
+        <v>210</v>
       </c>
       <c r="D266" s="22" t="s">
-        <v>962</v>
+        <v>959</v>
       </c>
       <c r="E266" s="21" t="s">
-        <v>963</v>
+        <v>960</v>
       </c>
       <c r="F266" s="22" t="s">
         <v>940</v>
@@ -15568,13 +15582,13 @@
         <v>125</v>
       </c>
       <c r="C267" s="21" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D267" s="22" t="s">
-        <v>965</v>
+        <v>962</v>
       </c>
       <c r="E267" s="21" t="s">
-        <v>966</v>
+        <v>963</v>
       </c>
       <c r="F267" s="22" t="s">
         <v>940</v>
@@ -15593,13 +15607,13 @@
         <v>125</v>
       </c>
       <c r="C268" s="21" t="s">
-        <v>296</v>
+        <v>262</v>
       </c>
       <c r="D268" s="22" t="s">
-        <v>968</v>
+        <v>965</v>
       </c>
       <c r="E268" s="21" t="s">
-        <v>969</v>
+        <v>966</v>
       </c>
       <c r="F268" s="22" t="s">
         <v>940</v>
@@ -15618,13 +15632,13 @@
         <v>125</v>
       </c>
       <c r="C269" s="21" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D269" s="22" t="s">
-        <v>971</v>
+        <v>968</v>
       </c>
       <c r="E269" s="21" t="s">
-        <v>972</v>
+        <v>969</v>
       </c>
       <c r="F269" s="22" t="s">
         <v>940</v>
@@ -15643,13 +15657,13 @@
         <v>125</v>
       </c>
       <c r="C270" s="21" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="D270" s="22" t="s">
-        <v>974</v>
+        <v>971</v>
       </c>
       <c r="E270" s="21" t="s">
-        <v>975</v>
+        <v>972</v>
       </c>
       <c r="F270" s="22" t="s">
         <v>940</v>
@@ -15668,13 +15682,13 @@
         <v>125</v>
       </c>
       <c r="C271" s="21" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D271" s="22" t="s">
-        <v>977</v>
+        <v>974</v>
       </c>
       <c r="E271" s="21" t="s">
-        <v>978</v>
+        <v>975</v>
       </c>
       <c r="F271" s="22" t="s">
         <v>940</v>
@@ -15690,19 +15704,19 @@
         <v>1008</v>
       </c>
       <c r="B272" s="21" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C272" s="21" t="s">
-        <v>174</v>
+        <v>308</v>
       </c>
       <c r="D272" s="22" t="s">
-        <v>980</v>
+        <v>977</v>
       </c>
       <c r="E272" s="21" t="s">
-        <v>981</v>
+        <v>978</v>
       </c>
       <c r="F272" s="22" t="s">
-        <v>982</v>
+        <v>940</v>
       </c>
       <c r="G272" s="20"/>
       <c r="H272" s="23"/>
@@ -15718,13 +15732,13 @@
         <v>128</v>
       </c>
       <c r="C273" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D273" s="22" t="s">
-        <v>984</v>
+        <v>980</v>
       </c>
       <c r="E273" s="21" t="s">
-        <v>985</v>
+        <v>981</v>
       </c>
       <c r="F273" s="22" t="s">
         <v>982</v>
@@ -15743,13 +15757,13 @@
         <v>128</v>
       </c>
       <c r="C274" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D274" s="22" t="s">
-        <v>987</v>
+        <v>984</v>
       </c>
       <c r="E274" s="21" t="s">
-        <v>988</v>
+        <v>985</v>
       </c>
       <c r="F274" s="22" t="s">
         <v>982</v>
@@ -15768,13 +15782,13 @@
         <v>128</v>
       </c>
       <c r="C275" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D275" s="22" t="s">
-        <v>990</v>
+        <v>987</v>
       </c>
       <c r="E275" s="21" t="s">
-        <v>991</v>
+        <v>988</v>
       </c>
       <c r="F275" s="22" t="s">
         <v>982</v>
@@ -15793,13 +15807,13 @@
         <v>128</v>
       </c>
       <c r="C276" s="21" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D276" s="22" t="s">
-        <v>993</v>
+        <v>990</v>
       </c>
       <c r="E276" s="21" t="s">
-        <v>994</v>
+        <v>991</v>
       </c>
       <c r="F276" s="22" t="s">
         <v>982</v>
@@ -15818,13 +15832,13 @@
         <v>128</v>
       </c>
       <c r="C277" s="21" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D277" s="22" t="s">
-        <v>996</v>
+        <v>993</v>
       </c>
       <c r="E277" s="21" t="s">
-        <v>997</v>
+        <v>994</v>
       </c>
       <c r="F277" s="22" t="s">
         <v>982</v>
@@ -15843,13 +15857,13 @@
         <v>128</v>
       </c>
       <c r="C278" s="21" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D278" s="22" t="s">
-        <v>999</v>
+        <v>996</v>
       </c>
       <c r="E278" s="21" t="s">
-        <v>1000</v>
+        <v>997</v>
       </c>
       <c r="F278" s="22" t="s">
         <v>982</v>
@@ -15865,19 +15879,19 @@
         <v>1032</v>
       </c>
       <c r="B279" s="21" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C279" s="21" t="s">
-        <v>174</v>
+        <v>206</v>
       </c>
       <c r="D279" s="22" t="s">
-        <v>1002</v>
+        <v>999</v>
       </c>
       <c r="E279" s="21" t="s">
-        <v>1003</v>
+        <v>1000</v>
       </c>
       <c r="F279" s="22" t="s">
-        <v>1004</v>
+        <v>982</v>
       </c>
       <c r="G279" s="20"/>
       <c r="H279" s="23"/>
@@ -15893,13 +15907,13 @@
         <v>130</v>
       </c>
       <c r="C280" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D280" s="22" t="s">
-        <v>1006</v>
+        <v>1002</v>
       </c>
       <c r="E280" s="21" t="s">
-        <v>1007</v>
+        <v>1003</v>
       </c>
       <c r="F280" s="22" t="s">
         <v>1004</v>
@@ -15915,19 +15929,19 @@
         <v>1038</v>
       </c>
       <c r="B281" s="21" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C281" s="21" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="D281" s="22" t="s">
-        <v>1009</v>
+        <v>1006</v>
       </c>
       <c r="E281" s="21" t="s">
-        <v>1010</v>
+        <v>1007</v>
       </c>
       <c r="F281" s="22" t="s">
-        <v>1011</v>
+        <v>1004</v>
       </c>
       <c r="G281" s="20"/>
       <c r="H281" s="23"/>
@@ -15943,13 +15957,13 @@
         <v>132</v>
       </c>
       <c r="C282" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D282" s="22" t="s">
-        <v>1013</v>
+        <v>1009</v>
       </c>
       <c r="E282" s="21" t="s">
-        <v>1014</v>
+        <v>1010</v>
       </c>
       <c r="F282" s="22" t="s">
         <v>1011</v>
@@ -15968,13 +15982,13 @@
         <v>132</v>
       </c>
       <c r="C283" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D283" s="22" t="s">
-        <v>1016</v>
+        <v>1013</v>
       </c>
       <c r="E283" s="21" t="s">
-        <v>1017</v>
+        <v>1014</v>
       </c>
       <c r="F283" s="22" t="s">
         <v>1011</v>
@@ -15993,13 +16007,13 @@
         <v>132</v>
       </c>
       <c r="C284" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D284" s="22" t="s">
-        <v>1019</v>
+        <v>1016</v>
       </c>
       <c r="E284" s="21" t="s">
-        <v>1020</v>
+        <v>1017</v>
       </c>
       <c r="F284" s="22" t="s">
         <v>1011</v>
@@ -16015,19 +16029,19 @@
         <v>1051</v>
       </c>
       <c r="B285" s="21" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C285" s="21" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
       <c r="D285" s="22" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="E285" s="21" t="s">
-        <v>1023</v>
+        <v>1020</v>
       </c>
       <c r="F285" s="22" t="s">
-        <v>1024</v>
+        <v>1011</v>
       </c>
       <c r="G285" s="20"/>
       <c r="H285" s="23"/>
@@ -16040,19 +16054,19 @@
         <v>1054</v>
       </c>
       <c r="B286" s="21" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C286" s="21" t="s">
         <v>174</v>
       </c>
       <c r="D286" s="22" t="s">
-        <v>1026</v>
+        <v>1022</v>
       </c>
       <c r="E286" s="21" t="s">
-        <v>1027</v>
+        <v>1023</v>
       </c>
       <c r="F286" s="22" t="s">
-        <v>1028</v>
+        <v>1024</v>
       </c>
       <c r="G286" s="20"/>
       <c r="H286" s="23"/>
@@ -16068,13 +16082,13 @@
         <v>135</v>
       </c>
       <c r="C287" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D287" s="22" t="s">
-        <v>1030</v>
+        <v>1026</v>
       </c>
       <c r="E287" s="21" t="s">
-        <v>1031</v>
+        <v>1027</v>
       </c>
       <c r="F287" s="22" t="s">
         <v>1028</v>
@@ -16093,13 +16107,13 @@
         <v>135</v>
       </c>
       <c r="C288" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D288" s="22" t="s">
-        <v>1033</v>
+        <v>1030</v>
       </c>
       <c r="E288" s="21" t="s">
-        <v>1034</v>
+        <v>1031</v>
       </c>
       <c r="F288" s="22" t="s">
         <v>1028</v>
@@ -16118,13 +16132,13 @@
         <v>135</v>
       </c>
       <c r="C289" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D289" s="22" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="E289" s="21" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="F289" s="22" t="s">
         <v>1028</v>
@@ -16143,13 +16157,13 @@
         <v>135</v>
       </c>
       <c r="C290" s="21" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D290" s="22" t="s">
-        <v>1039</v>
+        <v>1036</v>
       </c>
       <c r="E290" s="21" t="s">
-        <v>1040</v>
+        <v>1037</v>
       </c>
       <c r="F290" s="22" t="s">
         <v>1028</v>
@@ -16165,19 +16179,19 @@
         <v>1070</v>
       </c>
       <c r="B291" s="21" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C291" s="21" t="s">
-        <v>174</v>
+        <v>198</v>
       </c>
       <c r="D291" s="22" t="s">
-        <v>1042</v>
+        <v>1039</v>
       </c>
       <c r="E291" s="21" t="s">
-        <v>1043</v>
+        <v>1040</v>
       </c>
       <c r="F291" s="22" t="s">
-        <v>1044</v>
+        <v>1028</v>
       </c>
       <c r="G291" s="20"/>
       <c r="H291" s="23"/>
@@ -16193,13 +16207,13 @@
         <v>137</v>
       </c>
       <c r="C292" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D292" s="22" t="s">
-        <v>1046</v>
+        <v>1042</v>
       </c>
       <c r="E292" s="21" t="s">
-        <v>1047</v>
+        <v>1043</v>
       </c>
       <c r="F292" s="22" t="s">
         <v>1044</v>
@@ -16218,13 +16232,13 @@
         <v>137</v>
       </c>
       <c r="C293" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D293" s="22" t="s">
-        <v>1049</v>
+        <v>1046</v>
       </c>
       <c r="E293" s="21" t="s">
-        <v>1050</v>
+        <v>1047</v>
       </c>
       <c r="F293" s="22" t="s">
         <v>1044</v>
@@ -16243,13 +16257,13 @@
         <v>137</v>
       </c>
       <c r="C294" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D294" s="22" t="s">
-        <v>1052</v>
+        <v>1049</v>
       </c>
       <c r="E294" s="21" t="s">
-        <v>1053</v>
+        <v>1050</v>
       </c>
       <c r="F294" s="22" t="s">
         <v>1044</v>
@@ -16265,19 +16279,19 @@
         <v>1082</v>
       </c>
       <c r="B295" s="21" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C295" s="21" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
       <c r="D295" s="22" t="s">
-        <v>1055</v>
+        <v>1052</v>
       </c>
       <c r="E295" s="21" t="s">
-        <v>1056</v>
+        <v>1053</v>
       </c>
       <c r="F295" s="22" t="s">
-        <v>1057</v>
+        <v>1044</v>
       </c>
       <c r="G295" s="20"/>
       <c r="H295" s="23"/>
@@ -16293,13 +16307,13 @@
         <v>140</v>
       </c>
       <c r="C296" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D296" s="22" t="s">
-        <v>1059</v>
+        <v>1055</v>
       </c>
       <c r="E296" s="21" t="s">
-        <v>1060</v>
+        <v>1056</v>
       </c>
       <c r="F296" s="22" t="s">
         <v>1057</v>
@@ -16318,13 +16332,13 @@
         <v>140</v>
       </c>
       <c r="C297" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D297" s="22" t="s">
-        <v>1062</v>
+        <v>1059</v>
       </c>
       <c r="E297" s="21" t="s">
-        <v>1063</v>
+        <v>1060</v>
       </c>
       <c r="F297" s="22" t="s">
         <v>1057</v>
@@ -16343,13 +16357,13 @@
         <v>140</v>
       </c>
       <c r="C298" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D298" s="22" t="s">
-        <v>1065</v>
+        <v>1062</v>
       </c>
       <c r="E298" s="21" t="s">
-        <v>1066</v>
+        <v>1063</v>
       </c>
       <c r="F298" s="22" t="s">
         <v>1057</v>
@@ -16365,16 +16379,16 @@
         <v>1096</v>
       </c>
       <c r="B299" s="21" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C299" s="21" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
       <c r="D299" s="22" t="s">
-        <v>1068</v>
+        <v>1065</v>
       </c>
       <c r="E299" s="21" t="s">
-        <v>1069</v>
+        <v>1066</v>
       </c>
       <c r="F299" s="22" t="s">
         <v>1057</v>
@@ -16393,13 +16407,13 @@
         <v>142</v>
       </c>
       <c r="C300" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D300" s="22" t="s">
-        <v>1071</v>
+        <v>1068</v>
       </c>
       <c r="E300" s="21" t="s">
-        <v>1072</v>
+        <v>1069</v>
       </c>
       <c r="F300" s="22" t="s">
         <v>1057</v>
@@ -16418,13 +16432,13 @@
         <v>142</v>
       </c>
       <c r="C301" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D301" s="22" t="s">
-        <v>1074</v>
+        <v>1071</v>
       </c>
       <c r="E301" s="21" t="s">
-        <v>1075</v>
+        <v>1072</v>
       </c>
       <c r="F301" s="22" t="s">
         <v>1057</v>
@@ -16443,13 +16457,13 @@
         <v>142</v>
       </c>
       <c r="C302" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D302" s="22" t="s">
-        <v>1077</v>
+        <v>1074</v>
       </c>
       <c r="E302" s="21" t="s">
-        <v>1078</v>
+        <v>1075</v>
       </c>
       <c r="F302" s="22" t="s">
         <v>1057</v>
@@ -16468,13 +16482,13 @@
         <v>142</v>
       </c>
       <c r="C303" s="21" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D303" s="22" t="s">
-        <v>1080</v>
+        <v>1077</v>
       </c>
       <c r="E303" s="21" t="s">
-        <v>1081</v>
+        <v>1078</v>
       </c>
       <c r="F303" s="22" t="s">
         <v>1057</v>
@@ -16493,13 +16507,13 @@
         <v>142</v>
       </c>
       <c r="C304" s="21" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D304" s="22" t="s">
-        <v>1083</v>
+        <v>1080</v>
       </c>
       <c r="E304" s="21" t="s">
-        <v>1084</v>
+        <v>1081</v>
       </c>
       <c r="F304" s="22" t="s">
         <v>1057</v>
@@ -16518,13 +16532,13 @@
         <v>142</v>
       </c>
       <c r="C305" s="21" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D305" s="22" t="s">
-        <v>1086</v>
+        <v>1083</v>
       </c>
       <c r="E305" s="21" t="s">
-        <v>1087</v>
+        <v>1084</v>
       </c>
       <c r="F305" s="22" t="s">
         <v>1057</v>
@@ -16540,19 +16554,19 @@
         <v>1119</v>
       </c>
       <c r="B306" s="21" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C306" s="21" t="s">
-        <v>174</v>
+        <v>206</v>
       </c>
       <c r="D306" s="22" t="s">
-        <v>1089</v>
+        <v>1086</v>
       </c>
       <c r="E306" s="21" t="s">
-        <v>1090</v>
+        <v>1087</v>
       </c>
       <c r="F306" s="22" t="s">
-        <v>1091</v>
+        <v>1057</v>
       </c>
       <c r="G306" s="20"/>
       <c r="H306" s="23"/>
@@ -16565,19 +16579,19 @@
         <v>1122</v>
       </c>
       <c r="B307" s="21" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C307" s="21" t="s">
         <v>174</v>
       </c>
       <c r="D307" s="22" t="s">
-        <v>1093</v>
+        <v>1089</v>
       </c>
       <c r="E307" s="21" t="s">
-        <v>1094</v>
+        <v>1090</v>
       </c>
       <c r="F307" s="22" t="s">
-        <v>1095</v>
+        <v>1091</v>
       </c>
       <c r="G307" s="20"/>
       <c r="H307" s="23"/>
@@ -16593,13 +16607,13 @@
         <v>146</v>
       </c>
       <c r="C308" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D308" s="22" t="s">
-        <v>1097</v>
+        <v>1093</v>
       </c>
       <c r="E308" s="21" t="s">
-        <v>1098</v>
+        <v>1094</v>
       </c>
       <c r="F308" s="22" t="s">
         <v>1095</v>
@@ -16618,13 +16632,13 @@
         <v>146</v>
       </c>
       <c r="C309" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D309" s="22" t="s">
-        <v>1100</v>
+        <v>1097</v>
       </c>
       <c r="E309" s="21" t="s">
-        <v>1101</v>
+        <v>1098</v>
       </c>
       <c r="F309" s="22" t="s">
         <v>1095</v>
@@ -16640,19 +16654,19 @@
         <v>1129</v>
       </c>
       <c r="B310" s="21" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C310" s="21" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="D310" s="22" t="s">
-        <v>1103</v>
+        <v>1100</v>
       </c>
       <c r="E310" s="21" t="s">
-        <v>1104</v>
+        <v>1101</v>
       </c>
       <c r="F310" s="22" t="s">
-        <v>1105</v>
+        <v>1095</v>
       </c>
       <c r="G310" s="20"/>
       <c r="H310" s="23"/>
@@ -16668,13 +16682,13 @@
         <v>147</v>
       </c>
       <c r="C311" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D311" s="22" t="s">
-        <v>1107</v>
+        <v>1103</v>
       </c>
       <c r="E311" s="21" t="s">
-        <v>1108</v>
+        <v>1104</v>
       </c>
       <c r="F311" s="22" t="s">
         <v>1105</v>
@@ -16693,13 +16707,13 @@
         <v>147</v>
       </c>
       <c r="C312" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D312" s="22" t="s">
-        <v>1110</v>
+        <v>1107</v>
       </c>
       <c r="E312" s="21" t="s">
-        <v>1111</v>
+        <v>1108</v>
       </c>
       <c r="F312" s="22" t="s">
         <v>1105</v>
@@ -16715,19 +16729,19 @@
         <v>1140</v>
       </c>
       <c r="B313" s="21" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C313" s="21" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="D313" s="22" t="s">
-        <v>1113</v>
+        <v>1110</v>
       </c>
       <c r="E313" s="21" t="s">
-        <v>1114</v>
+        <v>1111</v>
       </c>
       <c r="F313" s="22" t="s">
-        <v>1115</v>
+        <v>1105</v>
       </c>
       <c r="G313" s="20"/>
       <c r="H313" s="23"/>
@@ -16743,13 +16757,13 @@
         <v>148</v>
       </c>
       <c r="C314" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D314" s="22" t="s">
-        <v>1117</v>
+        <v>1113</v>
       </c>
       <c r="E314" s="21" t="s">
-        <v>1118</v>
+        <v>1114</v>
       </c>
       <c r="F314" s="22" t="s">
         <v>1115</v>
@@ -16768,13 +16782,13 @@
         <v>148</v>
       </c>
       <c r="C315" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D315" s="22" t="s">
-        <v>1120</v>
+        <v>1117</v>
       </c>
       <c r="E315" s="21" t="s">
-        <v>1121</v>
+        <v>1118</v>
       </c>
       <c r="F315" s="22" t="s">
         <v>1115</v>
@@ -16793,13 +16807,13 @@
         <v>148</v>
       </c>
       <c r="C316" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D316" s="22" t="s">
-        <v>1113</v>
+        <v>1120</v>
       </c>
       <c r="E316" s="21" t="s">
-        <v>1114</v>
+        <v>1121</v>
       </c>
       <c r="F316" s="22" t="s">
         <v>1115</v>
@@ -16818,13 +16832,13 @@
         <v>148</v>
       </c>
       <c r="C317" s="21" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D317" s="22" t="s">
-        <v>1124</v>
+        <v>1113</v>
       </c>
       <c r="E317" s="21" t="s">
-        <v>1125</v>
+        <v>1114</v>
       </c>
       <c r="F317" s="22" t="s">
         <v>1115</v>
@@ -16843,13 +16857,13 @@
         <v>148</v>
       </c>
       <c r="C318" s="21" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D318" s="22" t="s">
-        <v>1127</v>
+        <v>1124</v>
       </c>
       <c r="E318" s="21" t="s">
-        <v>1128</v>
+        <v>1125</v>
       </c>
       <c r="F318" s="22" t="s">
         <v>1115</v>
@@ -16865,19 +16879,19 @@
         <v>1159</v>
       </c>
       <c r="B319" s="21" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C319" s="21" t="s">
-        <v>174</v>
+        <v>202</v>
       </c>
       <c r="D319" s="22" t="s">
-        <v>1130</v>
+        <v>1127</v>
       </c>
       <c r="E319" s="21" t="s">
-        <v>1131</v>
+        <v>1128</v>
       </c>
       <c r="F319" s="22" t="s">
-        <v>1132</v>
+        <v>1115</v>
       </c>
       <c r="G319" s="20"/>
       <c r="H319" s="23"/>
@@ -16893,13 +16907,13 @@
         <v>150</v>
       </c>
       <c r="C320" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D320" s="22" t="s">
-        <v>1134</v>
+        <v>1130</v>
       </c>
       <c r="E320" s="21" t="s">
-        <v>1135</v>
+        <v>1131</v>
       </c>
       <c r="F320" s="22" t="s">
         <v>1132</v>
@@ -16915,19 +16929,19 @@
         <v>1165</v>
       </c>
       <c r="B321" s="21" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C321" s="21" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="D321" s="22" t="s">
-        <v>1137</v>
+        <v>1134</v>
       </c>
       <c r="E321" s="21" t="s">
-        <v>1138</v>
+        <v>1135</v>
       </c>
       <c r="F321" s="22" t="s">
-        <v>1139</v>
+        <v>1132</v>
       </c>
       <c r="G321" s="20"/>
       <c r="H321" s="23"/>
@@ -16943,13 +16957,13 @@
         <v>153</v>
       </c>
       <c r="C322" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D322" s="22" t="s">
-        <v>1141</v>
+        <v>1137</v>
       </c>
       <c r="E322" s="21" t="s">
-        <v>1142</v>
+        <v>1138</v>
       </c>
       <c r="F322" s="22" t="s">
         <v>1139</v>
@@ -16965,19 +16979,19 @@
         <v>1171</v>
       </c>
       <c r="B323" s="21" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C323" s="21" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="D323" s="22" t="s">
-        <v>1144</v>
+        <v>1141</v>
       </c>
       <c r="E323" s="21" t="s">
-        <v>1145</v>
+        <v>1142</v>
       </c>
       <c r="F323" s="22" t="s">
-        <v>1146</v>
+        <v>1139</v>
       </c>
       <c r="G323" s="20"/>
       <c r="H323" s="23"/>
@@ -16993,13 +17007,13 @@
         <v>155</v>
       </c>
       <c r="C324" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D324" s="22" t="s">
-        <v>1148</v>
+        <v>1144</v>
       </c>
       <c r="E324" s="21" t="s">
-        <v>1149</v>
+        <v>1145</v>
       </c>
       <c r="F324" s="22" t="s">
         <v>1146</v>
@@ -17018,13 +17032,13 @@
         <v>155</v>
       </c>
       <c r="C325" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D325" s="22" t="s">
-        <v>1151</v>
+        <v>1148</v>
       </c>
       <c r="E325" s="21" t="s">
-        <v>1152</v>
+        <v>1149</v>
       </c>
       <c r="F325" s="22" t="s">
         <v>1146</v>
@@ -17043,13 +17057,13 @@
         <v>155</v>
       </c>
       <c r="C326" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D326" s="22" t="s">
-        <v>1154</v>
+        <v>1151</v>
       </c>
       <c r="E326" s="21" t="s">
-        <v>1155</v>
+        <v>1152</v>
       </c>
       <c r="F326" s="22" t="s">
         <v>1146</v>
@@ -17068,13 +17082,13 @@
         <v>155</v>
       </c>
       <c r="C327" s="21" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D327" s="22" t="s">
-        <v>1157</v>
+        <v>1154</v>
       </c>
       <c r="E327" s="21" t="s">
-        <v>1158</v>
+        <v>1155</v>
       </c>
       <c r="F327" s="22" t="s">
         <v>1146</v>
@@ -17093,13 +17107,13 @@
         <v>155</v>
       </c>
       <c r="C328" s="21" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D328" s="22" t="s">
-        <v>1160</v>
+        <v>1157</v>
       </c>
       <c r="E328" s="21" t="s">
-        <v>1161</v>
+        <v>1158</v>
       </c>
       <c r="F328" s="22" t="s">
         <v>1146</v>
@@ -17118,13 +17132,13 @@
         <v>155</v>
       </c>
       <c r="C329" s="21" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D329" s="22" t="s">
-        <v>1163</v>
+        <v>1160</v>
       </c>
       <c r="E329" s="21" t="s">
-        <v>1164</v>
+        <v>1161</v>
       </c>
       <c r="F329" s="22" t="s">
         <v>1146</v>
@@ -17143,13 +17157,13 @@
         <v>155</v>
       </c>
       <c r="C330" s="21" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="D330" s="22" t="s">
-        <v>1166</v>
+        <v>1163</v>
       </c>
       <c r="E330" s="21" t="s">
-        <v>1167</v>
+        <v>1164</v>
       </c>
       <c r="F330" s="22" t="s">
         <v>1146</v>
@@ -17168,13 +17182,13 @@
         <v>155</v>
       </c>
       <c r="C331" s="21" t="s">
-        <v>258</v>
+        <v>210</v>
       </c>
       <c r="D331" s="22" t="s">
-        <v>1169</v>
+        <v>1166</v>
       </c>
       <c r="E331" s="21" t="s">
-        <v>1170</v>
+        <v>1167</v>
       </c>
       <c r="F331" s="22" t="s">
         <v>1146</v>
@@ -17193,13 +17207,13 @@
         <v>155</v>
       </c>
       <c r="C332" s="21" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D332" s="22" t="s">
-        <v>1172</v>
+        <v>1169</v>
       </c>
       <c r="E332" s="21" t="s">
-        <v>1173</v>
+        <v>1170</v>
       </c>
       <c r="F332" s="22" t="s">
         <v>1146</v>
@@ -17218,13 +17232,13 @@
         <v>155</v>
       </c>
       <c r="C333" s="21" t="s">
-        <v>296</v>
+        <v>262</v>
       </c>
       <c r="D333" s="22" t="s">
-        <v>1175</v>
+        <v>1172</v>
       </c>
       <c r="E333" s="21" t="s">
-        <v>1176</v>
+        <v>1173</v>
       </c>
       <c r="F333" s="22" t="s">
         <v>1146</v>
@@ -17243,13 +17257,13 @@
         <v>155</v>
       </c>
       <c r="C334" s="21" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D334" s="22" t="s">
-        <v>1178</v>
+        <v>1175</v>
       </c>
       <c r="E334" s="21" t="s">
-        <v>1179</v>
+        <v>1176</v>
       </c>
       <c r="F334" s="22" t="s">
         <v>1146</v>
@@ -17268,13 +17282,13 @@
         <v>155</v>
       </c>
       <c r="C335" s="21" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="D335" s="22" t="s">
-        <v>1181</v>
+        <v>1178</v>
       </c>
       <c r="E335" s="21" t="s">
-        <v>1182</v>
+        <v>1179</v>
       </c>
       <c r="F335" s="22" t="s">
         <v>1146</v>
@@ -17293,13 +17307,13 @@
         <v>155</v>
       </c>
       <c r="C336" s="21" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D336" s="22" t="s">
-        <v>1184</v>
+        <v>1181</v>
       </c>
       <c r="E336" s="21" t="s">
-        <v>1185</v>
+        <v>1182</v>
       </c>
       <c r="F336" s="22" t="s">
         <v>1146</v>
@@ -17318,13 +17332,13 @@
         <v>155</v>
       </c>
       <c r="C337" s="21" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D337" s="22" t="s">
-        <v>1187</v>
+        <v>1184</v>
       </c>
       <c r="E337" s="21" t="s">
-        <v>1188</v>
+        <v>1185</v>
       </c>
       <c r="F337" s="22" t="s">
         <v>1146</v>
@@ -17343,13 +17357,13 @@
         <v>155</v>
       </c>
       <c r="C338" s="21" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D338" s="22" t="s">
-        <v>1190</v>
+        <v>1187</v>
       </c>
       <c r="E338" s="21" t="s">
-        <v>1191</v>
+        <v>1188</v>
       </c>
       <c r="F338" s="22" t="s">
         <v>1146</v>
@@ -17368,13 +17382,13 @@
         <v>155</v>
       </c>
       <c r="C339" s="21" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="D339" s="22" t="s">
-        <v>1193</v>
+        <v>1190</v>
       </c>
       <c r="E339" s="21" t="s">
-        <v>1194</v>
+        <v>1191</v>
       </c>
       <c r="F339" s="22" t="s">
         <v>1146</v>
@@ -17393,13 +17407,13 @@
         <v>155</v>
       </c>
       <c r="C340" s="21" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D340" s="22" t="s">
-        <v>1196</v>
+        <v>1193</v>
       </c>
       <c r="E340" s="21" t="s">
-        <v>188</v>
+        <v>1194</v>
       </c>
       <c r="F340" s="22" t="s">
         <v>1146</v>
@@ -17418,13 +17432,13 @@
         <v>155</v>
       </c>
       <c r="C341" s="21" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D341" s="22" t="s">
-        <v>1198</v>
+        <v>1196</v>
       </c>
       <c r="E341" s="21" t="s">
-        <v>1199</v>
+        <v>188</v>
       </c>
       <c r="F341" s="22" t="s">
         <v>1146</v>
@@ -17443,13 +17457,13 @@
         <v>155</v>
       </c>
       <c r="C342" s="21" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="D342" s="22" t="s">
-        <v>1201</v>
+        <v>1198</v>
       </c>
       <c r="E342" s="21" t="s">
-        <v>1202</v>
+        <v>1199</v>
       </c>
       <c r="F342" s="22" t="s">
         <v>1146</v>
@@ -17468,13 +17482,13 @@
         <v>155</v>
       </c>
       <c r="C343" s="21" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="D343" s="22" t="s">
-        <v>1204</v>
+        <v>1201</v>
       </c>
       <c r="E343" s="21" t="s">
-        <v>1205</v>
+        <v>1202</v>
       </c>
       <c r="F343" s="22" t="s">
         <v>1146</v>
@@ -17490,19 +17504,19 @@
         <v>1233</v>
       </c>
       <c r="B344" s="21" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C344" s="21" t="s">
-        <v>174</v>
+        <v>336</v>
       </c>
       <c r="D344" s="22" t="s">
-        <v>1207</v>
+        <v>1204</v>
       </c>
       <c r="E344" s="21" t="s">
-        <v>1161</v>
+        <v>1205</v>
       </c>
       <c r="F344" s="22" t="s">
-        <v>1208</v>
+        <v>1146</v>
       </c>
       <c r="G344" s="20"/>
       <c r="H344" s="23"/>
@@ -17518,13 +17532,13 @@
         <v>156</v>
       </c>
       <c r="C345" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D345" s="22" t="s">
-        <v>1210</v>
+        <v>1207</v>
       </c>
       <c r="E345" s="21" t="s">
-        <v>1211</v>
+        <v>1161</v>
       </c>
       <c r="F345" s="22" t="s">
         <v>1208</v>
@@ -17543,13 +17557,13 @@
         <v>156</v>
       </c>
       <c r="C346" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D346" s="22" t="s">
-        <v>1213</v>
+        <v>1210</v>
       </c>
       <c r="E346" s="21" t="s">
-        <v>1214</v>
+        <v>1211</v>
       </c>
       <c r="F346" s="22" t="s">
         <v>1208</v>
@@ -17568,13 +17582,13 @@
         <v>156</v>
       </c>
       <c r="C347" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D347" s="22" t="s">
-        <v>1216</v>
+        <v>1213</v>
       </c>
       <c r="E347" s="21" t="s">
-        <v>1217</v>
+        <v>1214</v>
       </c>
       <c r="F347" s="22" t="s">
         <v>1208</v>
@@ -17593,13 +17607,13 @@
         <v>156</v>
       </c>
       <c r="C348" s="21" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D348" s="22" t="s">
-        <v>1219</v>
+        <v>1216</v>
       </c>
       <c r="E348" s="21" t="s">
-        <v>1220</v>
+        <v>1217</v>
       </c>
       <c r="F348" s="22" t="s">
         <v>1208</v>
@@ -17618,13 +17632,13 @@
         <v>156</v>
       </c>
       <c r="C349" s="21" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D349" s="22" t="s">
-        <v>1222</v>
+        <v>1219</v>
       </c>
       <c r="E349" s="21" t="s">
-        <v>1223</v>
+        <v>1220</v>
       </c>
       <c r="F349" s="22" t="s">
         <v>1208</v>
@@ -17643,13 +17657,13 @@
         <v>156</v>
       </c>
       <c r="C350" s="21" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D350" s="22" t="s">
-        <v>1225</v>
+        <v>1222</v>
       </c>
       <c r="E350" s="21" t="s">
-        <v>1226</v>
+        <v>1223</v>
       </c>
       <c r="F350" s="22" t="s">
         <v>1208</v>
@@ -17668,13 +17682,13 @@
         <v>156</v>
       </c>
       <c r="C351" s="21" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="D351" s="22" t="s">
-        <v>1228</v>
+        <v>1225</v>
       </c>
       <c r="E351" s="21" t="s">
-        <v>1229</v>
+        <v>1226</v>
       </c>
       <c r="F351" s="22" t="s">
         <v>1208</v>
@@ -17693,13 +17707,13 @@
         <v>156</v>
       </c>
       <c r="C352" s="21" t="s">
-        <v>258</v>
+        <v>210</v>
       </c>
       <c r="D352" s="22" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="E352" s="21" t="s">
-        <v>1232</v>
+        <v>1229</v>
       </c>
       <c r="F352" s="22" t="s">
         <v>1208</v>
@@ -17718,13 +17732,13 @@
         <v>156</v>
       </c>
       <c r="C353" s="21" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D353" s="22" t="s">
-        <v>1234</v>
+        <v>1231</v>
       </c>
       <c r="E353" s="21" t="s">
-        <v>1235</v>
+        <v>1232</v>
       </c>
       <c r="F353" s="22" t="s">
         <v>1208</v>
@@ -17743,13 +17757,13 @@
         <v>156</v>
       </c>
       <c r="C354" s="21" t="s">
-        <v>296</v>
+        <v>262</v>
       </c>
       <c r="D354" s="22" t="s">
-        <v>1237</v>
+        <v>1234</v>
       </c>
       <c r="E354" s="21" t="s">
-        <v>1238</v>
+        <v>1235</v>
       </c>
       <c r="F354" s="22" t="s">
         <v>1208</v>
@@ -17768,13 +17782,13 @@
         <v>156</v>
       </c>
       <c r="C355" s="21" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D355" s="22" t="s">
-        <v>1240</v>
+        <v>1237</v>
       </c>
       <c r="E355" s="21" t="s">
-        <v>1241</v>
+        <v>1238</v>
       </c>
       <c r="F355" s="22" t="s">
         <v>1208</v>
@@ -17790,19 +17804,19 @@
         <v>1300</v>
       </c>
       <c r="B356" s="21" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C356" s="21" t="s">
-        <v>174</v>
+        <v>300</v>
       </c>
       <c r="D356" s="22" t="s">
-        <v>1243</v>
+        <v>1240</v>
       </c>
       <c r="E356" s="21" t="s">
-        <v>1244</v>
+        <v>1241</v>
       </c>
       <c r="F356" s="22" t="s">
-        <v>875</v>
+        <v>1208</v>
       </c>
       <c r="G356" s="20"/>
       <c r="H356" s="23"/>
@@ -17818,13 +17832,13 @@
         <v>158</v>
       </c>
       <c r="C357" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D357" s="22" t="s">
-        <v>1246</v>
+        <v>1243</v>
       </c>
       <c r="E357" s="21" t="s">
-        <v>1247</v>
+        <v>1244</v>
       </c>
       <c r="F357" s="22" t="s">
         <v>875</v>
@@ -17843,13 +17857,13 @@
         <v>158</v>
       </c>
       <c r="C358" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D358" s="22" t="s">
-        <v>1249</v>
+        <v>1246</v>
       </c>
       <c r="E358" s="21" t="s">
-        <v>1250</v>
+        <v>1247</v>
       </c>
       <c r="F358" s="22" t="s">
         <v>875</v>
@@ -17868,13 +17882,13 @@
         <v>158</v>
       </c>
       <c r="C359" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D359" s="22" t="s">
-        <v>1252</v>
+        <v>1249</v>
       </c>
       <c r="E359" s="21" t="s">
-        <v>1253</v>
+        <v>1250</v>
       </c>
       <c r="F359" s="22" t="s">
         <v>875</v>
@@ -17893,13 +17907,13 @@
         <v>158</v>
       </c>
       <c r="C360" s="21" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D360" s="22" t="s">
-        <v>1255</v>
+        <v>1252</v>
       </c>
       <c r="E360" s="21" t="s">
-        <v>1256</v>
+        <v>1253</v>
       </c>
       <c r="F360" s="22" t="s">
         <v>875</v>
@@ -17915,35 +17929,25 @@
         <v>1305</v>
       </c>
       <c r="B361" s="21" t="s">
-        <v>1295</v>
+        <v>158</v>
       </c>
       <c r="C361" s="21" t="s">
-        <v>174</v>
+        <v>198</v>
       </c>
       <c r="D361" s="22" t="s">
-        <v>1298</v>
+        <v>1255</v>
       </c>
       <c r="E361" s="21" t="s">
-        <v>1310</v>
+        <v>1256</v>
       </c>
       <c r="F361" s="22" t="s">
-        <v>1311</v>
-      </c>
-      <c r="G361" s="20">
-        <v>4500</v>
-      </c>
-      <c r="H361" s="23" t="s">
-        <v>1275</v>
-      </c>
-      <c r="I361" s="23">
-        <v>100000</v>
-      </c>
-      <c r="J361" s="23">
-        <v>99000</v>
-      </c>
-      <c r="K361" s="23">
-        <v>82500</v>
-      </c>
+        <v>875</v>
+      </c>
+      <c r="G361" s="20"/>
+      <c r="H361" s="23"/>
+      <c r="I361" s="23"/>
+      <c r="J361" s="23"/>
+      <c r="K361" s="23"/>
     </row>
     <row r="362" spans="1:11">
       <c r="A362" s="21" t="s">
@@ -17953,19 +17957,19 @@
         <v>1295</v>
       </c>
       <c r="C362" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D362" s="22" t="s">
-        <v>1312</v>
+        <v>1298</v>
       </c>
       <c r="E362" s="21" t="s">
-        <v>1316</v>
+        <v>1310</v>
       </c>
       <c r="F362" s="22" t="s">
         <v>1311</v>
       </c>
       <c r="G362" s="20">
-        <v>5000</v>
+        <v>4500</v>
       </c>
       <c r="H362" s="23" t="s">
         <v>1275</v>
@@ -17988,13 +17992,13 @@
         <v>1295</v>
       </c>
       <c r="C363" s="21" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D363" s="22" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="E363" s="21" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="F363" s="22" t="s">
         <v>1311</v>
@@ -18023,13 +18027,13 @@
         <v>1295</v>
       </c>
       <c r="C364" s="21" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D364" s="22" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="E364" s="21" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
       <c r="F364" s="22" t="s">
         <v>1311</v>
@@ -18058,13 +18062,13 @@
         <v>1295</v>
       </c>
       <c r="C365" s="21" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D365" s="22" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="E365" s="21" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
       <c r="F365" s="22" t="s">
         <v>1311</v>
@@ -18086,17 +18090,39 @@
       </c>
     </row>
     <row r="366" spans="1:11">
-      <c r="A366" s="21"/>
-      <c r="B366" s="21"/>
-      <c r="C366" s="21"/>
-      <c r="D366" s="22"/>
-      <c r="E366" s="21"/>
-      <c r="F366" s="22"/>
-      <c r="G366" s="20"/>
-      <c r="H366" s="23"/>
-      <c r="I366" s="23"/>
-      <c r="J366" s="23"/>
-      <c r="K366" s="23"/>
+      <c r="A366" s="21" t="s">
+        <v>1323</v>
+      </c>
+      <c r="B366" s="21" t="s">
+        <v>1295</v>
+      </c>
+      <c r="C366" s="21" t="s">
+        <v>198</v>
+      </c>
+      <c r="D366" s="22" t="s">
+        <v>1315</v>
+      </c>
+      <c r="E366" s="21" t="s">
+        <v>1319</v>
+      </c>
+      <c r="F366" s="22" t="s">
+        <v>1311</v>
+      </c>
+      <c r="G366" s="20">
+        <v>5000</v>
+      </c>
+      <c r="H366" s="23" t="s">
+        <v>1275</v>
+      </c>
+      <c r="I366" s="23">
+        <v>100000</v>
+      </c>
+      <c r="J366" s="23">
+        <v>99000</v>
+      </c>
+      <c r="K366" s="23">
+        <v>82500</v>
+      </c>
     </row>
     <row r="367" spans="1:11">
       <c r="A367" s="21"/>
@@ -18742,7 +18768,7 @@
       <c r="D416" s="22"/>
       <c r="E416" s="21"/>
       <c r="F416" s="22"/>
-      <c r="G416" s="18"/>
+      <c r="G416" s="20"/>
       <c r="H416" s="23"/>
       <c r="I416" s="23"/>
       <c r="J416" s="23"/>
@@ -39442,7 +39468,7 @@
       <c r="H2008" s="23"/>
       <c r="I2008" s="23"/>
       <c r="J2008" s="23"/>
-      <c r="K2008" s="33"/>
+      <c r="K2008" s="23"/>
     </row>
     <row r="2009" spans="1:11">
       <c r="A2009" s="21"/>
@@ -39457,15 +39483,28 @@
       <c r="J2009" s="23"/>
       <c r="K2009" s="33"/>
     </row>
+    <row r="2010" spans="1:11">
+      <c r="A2010" s="21"/>
+      <c r="B2010" s="21"/>
+      <c r="C2010" s="21"/>
+      <c r="D2010" s="22"/>
+      <c r="E2010" s="21"/>
+      <c r="F2010" s="22"/>
+      <c r="G2010" s="18"/>
+      <c r="H2010" s="23"/>
+      <c r="I2010" s="23"/>
+      <c r="J2010" s="23"/>
+      <c r="K2010" s="33"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A1:K1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A2005:A2009">
+  <conditionalFormatting sqref="A2006:A2010">
     <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A4:A2004">
+  <conditionalFormatting sqref="A4:A2005">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -39495,27 +39534,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="33.9" customHeight="1">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="42" t="s">
         <v>1257</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
       <c r="H1" s="29"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="50" t="s">
         <v>1258</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
+      <c r="B2" s="50"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
       <c r="H2" s="26"/>
     </row>
     <row r="3" spans="1:8" ht="38.1" customHeight="1">

</xml_diff>